<commit_message>
2x mobs and 200x unique mobs
</commit_message>
<xml_diff>
--- a/Diablo II.xlsx
+++ b/Diablo II.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yatyr\workspace\d2r-loot-filter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C07B0CB4-5F2F-47CB-8A34-008D968FA796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0684022-83CC-4D77-8283-24D7E01BD039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{4FA0E628-D5C1-45F8-838A-535ABF901563}"/>
+    <workbookView xWindow="0" yWindow="435" windowWidth="33990" windowHeight="19155" activeTab="1" xr2:uid="{4FA0E628-D5C1-45F8-838A-535ABF901563}"/>
   </bookViews>
   <sheets>
     <sheet name="Mod-ItemName" sheetId="2" r:id="rId1"/>
@@ -11614,34 +11614,34 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -11649,7 +11649,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -12192,8 +12192,8 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{53F17FA5-8A83-41A1-8800-C9AE149B41E5}"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="10">
     <dxf>
@@ -12620,20 +12620,20 @@
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:L171"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" style="32" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.58203125" style="32" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" style="33" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.58203125" style="32" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.4140625" style="32" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" style="33" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" style="32" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.4140625" style="32" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" style="33" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.33203125" style="32" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="4.4140625" style="32" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.9140625" style="33" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.375" style="32" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.625" style="32" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.625" style="33" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.625" style="32" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.375" style="32" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.625" style="33" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.625" style="32" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.375" style="32" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.625" style="33" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.375" style="32" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.375" style="32" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.875" style="33" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="9" style="32"/>
   </cols>
   <sheetData>
@@ -17996,7 +17996,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>A1:I171 J1:L169</xm:sqref>
+          <xm:sqref>J1:L169 A1:I171</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -18010,14 +18010,14 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:F247"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="57.08203125" style="71" customWidth="1"/>
-    <col min="2" max="2" width="14.58203125" style="52" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="57.125" style="71" customWidth="1"/>
+    <col min="2" max="2" width="14.625" style="52" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.5" style="52" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" style="52" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.08203125" style="52" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.83203125" style="52" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.875" style="52" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.125" style="52" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.875" style="52" bestFit="1" customWidth="1"/>
     <col min="7" max="16384" width="9" style="52"/>
   </cols>
   <sheetData>
@@ -19685,7 +19685,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="95" spans="1:6" ht="46.5">
+    <row r="95" spans="1:6" ht="47.25">
       <c r="A95" s="76" t="s">
         <v>3124</v>
       </c>
@@ -22538,14 +22538,14 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:F34"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="3.5" style="72" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.58203125" style="72" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="58.33203125" style="72" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.625" style="72" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58.375" style="72" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="38.25" style="72" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="38.25" style="75" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.83203125" style="72" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.875" style="72" bestFit="1" customWidth="1"/>
     <col min="7" max="16384" width="9" style="72"/>
   </cols>
   <sheetData>
@@ -23241,14 +23241,14 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:G105"/>
-  <sheetFormatPr defaultColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.08203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.58203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.08203125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="37.1640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.125" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.625" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="37.125" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="26.5" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="70.83203125" style="10" customWidth="1"/>
+    <col min="6" max="6" width="70.875" style="10" customWidth="1"/>
     <col min="7" max="7" width="34.75" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="8" style="5"/>
   </cols>
@@ -23276,7 +23276,7 @@
         <v>2678</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="58">
+    <row r="2" spans="1:7" ht="60">
       <c r="A2" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23299,7 +23299,7 @@
         <v>1853</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="87">
+    <row r="3" spans="1:7" ht="90">
       <c r="A3" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23322,7 +23322,7 @@
         <v>1857</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="101.5">
+    <row r="4" spans="1:7" ht="105">
       <c r="A4" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23345,7 +23345,7 @@
         <v>1862</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="101.5">
+    <row r="5" spans="1:7" ht="105">
       <c r="A5" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23368,7 +23368,7 @@
         <v>1866</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="87">
+    <row r="6" spans="1:7" ht="90">
       <c r="A6" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23391,7 +23391,7 @@
         <v>1870</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="87">
+    <row r="7" spans="1:7" ht="90">
       <c r="A7" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23414,7 +23414,7 @@
         <v>1874</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="87">
+    <row r="8" spans="1:7" ht="90">
       <c r="A8" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23437,7 +23437,7 @@
         <v>1879</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="87">
+    <row r="9" spans="1:7" ht="90">
       <c r="A9" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23460,7 +23460,7 @@
         <v>1884</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="58">
+    <row r="10" spans="1:7" ht="60">
       <c r="A10" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23483,7 +23483,7 @@
         <v>1888</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="87">
+    <row r="11" spans="1:7" ht="90">
       <c r="A11" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23506,7 +23506,7 @@
         <v>1892</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="87">
+    <row r="12" spans="1:7" ht="90">
       <c r="A12" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23529,7 +23529,7 @@
         <v>1897</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="101.5">
+    <row r="13" spans="1:7" ht="105">
       <c r="A13" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23552,7 +23552,7 @@
         <v>1902</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="87">
+    <row r="14" spans="1:7" ht="90">
       <c r="A14" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23575,7 +23575,7 @@
         <v>1906</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="87">
+    <row r="15" spans="1:7" ht="90">
       <c r="A15" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23598,7 +23598,7 @@
         <v>1910</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="87">
+    <row r="16" spans="1:7" ht="90">
       <c r="A16" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23621,7 +23621,7 @@
         <v>1914</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="101.5">
+    <row r="17" spans="1:7" ht="105">
       <c r="A17" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23644,7 +23644,7 @@
         <v>1919</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="87">
+    <row r="18" spans="1:7" ht="90">
       <c r="A18" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23667,7 +23667,7 @@
         <v>1923</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="87">
+    <row r="19" spans="1:7" ht="90">
       <c r="A19" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23690,7 +23690,7 @@
         <v>2546</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="72.5">
+    <row r="20" spans="1:7" ht="75">
       <c r="A20" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23713,7 +23713,7 @@
         <v>2548</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="58">
+    <row r="21" spans="1:7" ht="60">
       <c r="A21" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23736,7 +23736,7 @@
         <v>2550</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="72.5">
+    <row r="22" spans="1:7" ht="75">
       <c r="A22" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23759,7 +23759,7 @@
         <v>2552</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="43.5">
+    <row r="23" spans="1:7" ht="45">
       <c r="A23" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23782,7 +23782,7 @@
         <v>2554</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="101.5">
+    <row r="24" spans="1:7" ht="105">
       <c r="A24" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23805,7 +23805,7 @@
         <v>2556</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="87">
+    <row r="25" spans="1:7" ht="90">
       <c r="A25" s="6" t="s">
         <v>1652</v>
       </c>
@@ -23828,7 +23828,7 @@
         <v>2558</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="101.5">
+    <row r="26" spans="1:7" ht="105">
       <c r="A26" s="6" t="s">
         <v>1937</v>
       </c>
@@ -23851,7 +23851,7 @@
         <v>2560</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="101.5">
+    <row r="27" spans="1:7" ht="105">
       <c r="A27" s="6" t="s">
         <v>1937</v>
       </c>
@@ -23874,7 +23874,7 @@
         <v>2562</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="101.5">
+    <row r="28" spans="1:7" ht="105">
       <c r="A28" s="6" t="s">
         <v>1937</v>
       </c>
@@ -23897,7 +23897,7 @@
         <v>2564</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="101.5">
+    <row r="29" spans="1:7" ht="105">
       <c r="A29" s="6" t="s">
         <v>1937</v>
       </c>
@@ -23920,7 +23920,7 @@
         <v>2565</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="101.5">
+    <row r="30" spans="1:7" ht="105">
       <c r="A30" s="6" t="s">
         <v>1937</v>
       </c>
@@ -23943,7 +23943,7 @@
         <v>2567</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="101.5">
+    <row r="31" spans="1:7" ht="105">
       <c r="A31" s="6" t="s">
         <v>1937</v>
       </c>
@@ -23966,7 +23966,7 @@
         <v>2569</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="101.5">
+    <row r="32" spans="1:7" ht="105">
       <c r="A32" s="6" t="s">
         <v>1937</v>
       </c>
@@ -23989,7 +23989,7 @@
         <v>2571</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="101.5">
+    <row r="33" spans="1:7" ht="105">
       <c r="A33" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24012,7 +24012,7 @@
         <v>2573</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="101.5">
+    <row r="34" spans="1:7" ht="105">
       <c r="A34" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24035,7 +24035,7 @@
         <v>2574</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="101.5">
+    <row r="35" spans="1:7" ht="105">
       <c r="A35" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24058,7 +24058,7 @@
         <v>2576</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="116">
+    <row r="36" spans="1:7" ht="120">
       <c r="A36" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24081,7 +24081,7 @@
         <v>2577</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="101.5">
+    <row r="37" spans="1:7" ht="105">
       <c r="A37" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24104,7 +24104,7 @@
         <v>2578</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="101.5">
+    <row r="38" spans="1:7" ht="105">
       <c r="A38" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24127,7 +24127,7 @@
         <v>2579</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="116">
+    <row r="39" spans="1:7" ht="120">
       <c r="A39" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24150,7 +24150,7 @@
         <v>2580</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="101.5">
+    <row r="40" spans="1:7" ht="105">
       <c r="A40" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24173,7 +24173,7 @@
         <v>2582</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="101.5">
+    <row r="41" spans="1:7" ht="105">
       <c r="A41" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24196,7 +24196,7 @@
         <v>2584</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="101.5">
+    <row r="42" spans="1:7" ht="105">
       <c r="A42" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24219,7 +24219,7 @@
         <v>2586</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="101.5">
+    <row r="43" spans="1:7" ht="105">
       <c r="A43" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24242,7 +24242,7 @@
         <v>2587</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="101.5">
+    <row r="44" spans="1:7" ht="105">
       <c r="A44" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24265,7 +24265,7 @@
         <v>2589</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="101.5">
+    <row r="45" spans="1:7" ht="105">
       <c r="A45" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24288,7 +24288,7 @@
         <v>2591</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="101.5">
+    <row r="46" spans="1:7" ht="105">
       <c r="A46" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24311,7 +24311,7 @@
         <v>2593</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="101.5">
+    <row r="47" spans="1:7" ht="105">
       <c r="A47" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24334,7 +24334,7 @@
         <v>2595</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="101.5">
+    <row r="48" spans="1:7" ht="105">
       <c r="A48" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24357,7 +24357,7 @@
         <v>2597</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="101.5">
+    <row r="49" spans="1:7" ht="105">
       <c r="A49" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24380,7 +24380,7 @@
         <v>2599</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="87">
+    <row r="50" spans="1:7" ht="90">
       <c r="A50" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24403,7 +24403,7 @@
         <v>2601</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="101.5">
+    <row r="51" spans="1:7" ht="105">
       <c r="A51" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24426,7 +24426,7 @@
         <v>2603</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="101.5">
+    <row r="52" spans="1:7" ht="105">
       <c r="A52" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24449,7 +24449,7 @@
         <v>2604</v>
       </c>
     </row>
-    <row r="53" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="53" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A53" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24472,7 +24472,7 @@
         <v>2605</v>
       </c>
     </row>
-    <row r="54" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="54" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A54" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24495,7 +24495,7 @@
         <v>2607</v>
       </c>
     </row>
-    <row r="55" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="55" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A55" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24518,7 +24518,7 @@
         <v>2608</v>
       </c>
     </row>
-    <row r="56" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="56" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A56" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24541,7 +24541,7 @@
         <v>2610</v>
       </c>
     </row>
-    <row r="57" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="57" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A57" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24564,7 +24564,7 @@
         <v>2611</v>
       </c>
     </row>
-    <row r="58" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="58" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A58" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24587,7 +24587,7 @@
         <v>2613</v>
       </c>
     </row>
-    <row r="59" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="59" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A59" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24610,7 +24610,7 @@
         <v>2615</v>
       </c>
     </row>
-    <row r="60" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="60" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A60" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24633,7 +24633,7 @@
         <v>2617</v>
       </c>
     </row>
-    <row r="61" spans="1:7" s="4" customFormat="1" ht="116">
+    <row r="61" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A61" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24656,7 +24656,7 @@
         <v>2618</v>
       </c>
     </row>
-    <row r="62" spans="1:7" s="4" customFormat="1" ht="130.5">
+    <row r="62" spans="1:7" s="4" customFormat="1" ht="135">
       <c r="A62" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24679,7 +24679,7 @@
         <v>2619</v>
       </c>
     </row>
-    <row r="63" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="63" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A63" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24702,7 +24702,7 @@
         <v>2621</v>
       </c>
     </row>
-    <row r="64" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="64" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A64" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24725,7 +24725,7 @@
         <v>2623</v>
       </c>
     </row>
-    <row r="65" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="65" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A65" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24748,7 +24748,7 @@
         <v>2625</v>
       </c>
     </row>
-    <row r="66" spans="1:7" s="4" customFormat="1" ht="116">
+    <row r="66" spans="1:7" s="4" customFormat="1" ht="120">
       <c r="A66" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24771,7 +24771,7 @@
         <v>2627</v>
       </c>
     </row>
-    <row r="67" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="67" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A67" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24794,7 +24794,7 @@
         <v>2628</v>
       </c>
     </row>
-    <row r="68" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="68" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A68" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24817,7 +24817,7 @@
         <v>2630</v>
       </c>
     </row>
-    <row r="69" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="69" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A69" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24840,7 +24840,7 @@
         <v>2632</v>
       </c>
     </row>
-    <row r="70" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="70" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A70" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24863,7 +24863,7 @@
         <v>2634</v>
       </c>
     </row>
-    <row r="71" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="71" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A71" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24886,7 +24886,7 @@
         <v>2635</v>
       </c>
     </row>
-    <row r="72" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="72" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A72" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24909,7 +24909,7 @@
         <v>2638</v>
       </c>
     </row>
-    <row r="73" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="73" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A73" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24932,7 +24932,7 @@
         <v>2640</v>
       </c>
     </row>
-    <row r="74" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="74" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A74" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24955,7 +24955,7 @@
         <v>2642</v>
       </c>
     </row>
-    <row r="75" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="75" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A75" s="6" t="s">
         <v>1937</v>
       </c>
@@ -24978,7 +24978,7 @@
         <v>2644</v>
       </c>
     </row>
-    <row r="76" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="76" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A76" s="6" t="s">
         <v>1937</v>
       </c>
@@ -25001,7 +25001,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="77" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="77" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A77" s="6" t="s">
         <v>1937</v>
       </c>
@@ -25024,7 +25024,7 @@
         <v>2647</v>
       </c>
     </row>
-    <row r="78" spans="1:7" s="4" customFormat="1" ht="58">
+    <row r="78" spans="1:7" s="4" customFormat="1" ht="60">
       <c r="A78" s="6" t="s">
         <v>2027</v>
       </c>
@@ -25047,7 +25047,7 @@
         <v>2649</v>
       </c>
     </row>
-    <row r="79" spans="1:7" s="4" customFormat="1" ht="58">
+    <row r="79" spans="1:7" s="4" customFormat="1" ht="60">
       <c r="A79" s="6" t="s">
         <v>2027</v>
       </c>
@@ -25070,7 +25070,7 @@
         <v>2651</v>
       </c>
     </row>
-    <row r="80" spans="1:7" s="4" customFormat="1" ht="58">
+    <row r="80" spans="1:7" s="4" customFormat="1" ht="60">
       <c r="A80" s="6" t="s">
         <v>2027</v>
       </c>
@@ -25093,7 +25093,7 @@
         <v>2653</v>
       </c>
     </row>
-    <row r="81" spans="1:7" s="4" customFormat="1" ht="58">
+    <row r="81" spans="1:7" s="4" customFormat="1" ht="60">
       <c r="A81" s="6" t="s">
         <v>2027</v>
       </c>
@@ -25116,7 +25116,7 @@
         <v>2655</v>
       </c>
     </row>
-    <row r="82" spans="1:7" s="4" customFormat="1" ht="58">
+    <row r="82" spans="1:7" s="4" customFormat="1" ht="60">
       <c r="A82" s="6" t="s">
         <v>2027</v>
       </c>
@@ -25139,7 +25139,7 @@
         <v>2657</v>
       </c>
     </row>
-    <row r="83" spans="1:7" s="4" customFormat="1" ht="58">
+    <row r="83" spans="1:7" s="4" customFormat="1" ht="60">
       <c r="A83" s="6" t="s">
         <v>2027</v>
       </c>
@@ -25162,7 +25162,7 @@
         <v>2659</v>
       </c>
     </row>
-    <row r="84" spans="1:7" s="4" customFormat="1" ht="58">
+    <row r="84" spans="1:7" s="4" customFormat="1" ht="60">
       <c r="A84" s="6" t="s">
         <v>2027</v>
       </c>
@@ -25185,7 +25185,7 @@
         <v>2661</v>
       </c>
     </row>
-    <row r="85" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="85" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A85" s="6" t="s">
         <v>2042</v>
       </c>
@@ -25208,7 +25208,7 @@
         <v>2663</v>
       </c>
     </row>
-    <row r="86" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="86" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A86" s="6" t="s">
         <v>2042</v>
       </c>
@@ -25231,7 +25231,7 @@
         <v>2665</v>
       </c>
     </row>
-    <row r="87" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="87" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A87" s="6" t="s">
         <v>2042</v>
       </c>
@@ -25254,7 +25254,7 @@
         <v>2667</v>
       </c>
     </row>
-    <row r="88" spans="1:7" s="4" customFormat="1" ht="87">
+    <row r="88" spans="1:7" s="4" customFormat="1" ht="90">
       <c r="A88" s="6" t="s">
         <v>2042</v>
       </c>
@@ -25277,7 +25277,7 @@
         <v>2669</v>
       </c>
     </row>
-    <row r="89" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="89" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A89" s="6" t="s">
         <v>2042</v>
       </c>
@@ -25300,7 +25300,7 @@
         <v>2671</v>
       </c>
     </row>
-    <row r="90" spans="1:7" s="4" customFormat="1" ht="87">
+    <row r="90" spans="1:7" s="4" customFormat="1" ht="90">
       <c r="A90" s="6" t="s">
         <v>2042</v>
       </c>
@@ -25323,7 +25323,7 @@
         <v>2674</v>
       </c>
     </row>
-    <row r="91" spans="1:7" s="4" customFormat="1" ht="87">
+    <row r="91" spans="1:7" s="4" customFormat="1" ht="90">
       <c r="A91" s="6" t="s">
         <v>2042</v>
       </c>
@@ -25346,7 +25346,7 @@
         <v>2676</v>
       </c>
     </row>
-    <row r="92" spans="1:7" ht="72.5">
+    <row r="92" spans="1:7" ht="75">
       <c r="A92" s="6" t="s">
         <v>2681</v>
       </c>
@@ -25369,7 +25369,7 @@
         <v>2684</v>
       </c>
     </row>
-    <row r="93" spans="1:7" ht="72.5">
+    <row r="93" spans="1:7" ht="75">
       <c r="A93" s="6" t="s">
         <v>2681</v>
       </c>
@@ -25392,7 +25392,7 @@
         <v>2688</v>
       </c>
     </row>
-    <row r="94" spans="1:7" ht="72.5">
+    <row r="94" spans="1:7" ht="75">
       <c r="A94" s="6" t="s">
         <v>2681</v>
       </c>
@@ -25415,7 +25415,7 @@
         <v>2692</v>
       </c>
     </row>
-    <row r="95" spans="1:7" ht="58">
+    <row r="95" spans="1:7" ht="60">
       <c r="A95" s="6" t="s">
         <v>2681</v>
       </c>
@@ -25438,7 +25438,7 @@
         <v>2694</v>
       </c>
     </row>
-    <row r="96" spans="1:7" ht="116">
+    <row r="96" spans="1:7" ht="120">
       <c r="A96" s="6" t="s">
         <v>2681</v>
       </c>
@@ -25461,7 +25461,7 @@
         <v>2698</v>
       </c>
     </row>
-    <row r="97" spans="1:7" ht="145">
+    <row r="97" spans="1:7" ht="150">
       <c r="A97" s="6" t="s">
         <v>2681</v>
       </c>
@@ -25484,7 +25484,7 @@
         <v>2702</v>
       </c>
     </row>
-    <row r="98" spans="1:7" ht="72.5">
+    <row r="98" spans="1:7" ht="75">
       <c r="A98" s="6" t="s">
         <v>2681</v>
       </c>
@@ -25507,7 +25507,7 @@
         <v>2706</v>
       </c>
     </row>
-    <row r="99" spans="1:7" ht="58">
+    <row r="99" spans="1:7" ht="60">
       <c r="A99" s="6" t="s">
         <v>2681</v>
       </c>
@@ -25530,7 +25530,7 @@
         <v>2710</v>
       </c>
     </row>
-    <row r="100" spans="1:7" ht="58">
+    <row r="100" spans="1:7" ht="60">
       <c r="A100" s="6" t="s">
         <v>2681</v>
       </c>
@@ -25553,7 +25553,7 @@
         <v>2714</v>
       </c>
     </row>
-    <row r="101" spans="1:7" ht="58">
+    <row r="101" spans="1:7" ht="60">
       <c r="A101" s="6" t="s">
         <v>3284</v>
       </c>
@@ -25576,7 +25576,7 @@
         <v>3286</v>
       </c>
     </row>
-    <row r="102" spans="1:7" ht="87">
+    <row r="102" spans="1:7" ht="90">
       <c r="A102" s="6" t="s">
         <v>3284</v>
       </c>
@@ -25599,7 +25599,7 @@
         <v>3291</v>
       </c>
     </row>
-    <row r="103" spans="1:7" ht="87">
+    <row r="103" spans="1:7" ht="90">
       <c r="A103" s="6" t="s">
         <v>3284</v>
       </c>
@@ -25622,7 +25622,7 @@
         <v>3295</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="101.5">
+    <row r="104" spans="1:7" ht="105">
       <c r="A104" s="6" t="s">
         <v>3284</v>
       </c>
@@ -25645,7 +25645,7 @@
         <v>3300</v>
       </c>
     </row>
-    <row r="105" spans="1:7" ht="101.5">
+    <row r="105" spans="1:7" ht="105">
       <c r="A105" s="6" t="s">
         <v>3284</v>
       </c>
@@ -25682,16 +25682,16 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:M140"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.75" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="3.33203125" style="5" customWidth="1"/>
+    <col min="3" max="5" width="3.375" style="5" customWidth="1"/>
     <col min="6" max="6" width="16" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="3.58203125" style="5" customWidth="1"/>
-    <col min="10" max="10" width="16.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="3.33203125" style="5" customWidth="1"/>
-    <col min="14" max="16384" width="7.83203125" style="5"/>
+    <col min="7" max="9" width="3.625" style="5" customWidth="1"/>
+    <col min="10" max="10" width="16.375" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="3.375" style="5" customWidth="1"/>
+    <col min="14" max="16384" width="7.875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -31465,12 +31465,12 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:F120"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.25" style="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="12.58203125" style="6" customWidth="1"/>
+    <col min="2" max="4" width="12.625" style="6" customWidth="1"/>
     <col min="5" max="5" width="35.75" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="7.83203125" style="5"/>
+    <col min="6" max="16384" width="7.875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -33887,14 +33887,14 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:F119"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="7.83203125" style="21"/>
+    <col min="1" max="2" width="7.875" style="21"/>
     <col min="3" max="3" width="16.5" style="21" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="40.33203125" style="40" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="40.375" style="40" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="60.75" style="40" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" style="21" customWidth="1"/>
-    <col min="7" max="16384" width="7.83203125" style="21"/>
+    <col min="6" max="6" width="45.875" style="21" customWidth="1"/>
+    <col min="7" max="16384" width="7.875" style="21"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="16" customFormat="1">
@@ -34463,7 +34463,7 @@
         <v>2356</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="29" hidden="1">
+    <row r="31" spans="1:6" ht="30" hidden="1">
       <c r="A31" s="20" t="s">
         <v>2282</v>
       </c>
@@ -34501,7 +34501,7 @@
       </c>
       <c r="F32" s="22"/>
     </row>
-    <row r="33" spans="1:6" ht="58" hidden="1">
+    <row r="33" spans="1:6" ht="60" hidden="1">
       <c r="A33" s="23" t="s">
         <v>2282</v>
       </c>
@@ -34519,7 +34519,7 @@
       </c>
       <c r="F33" s="23"/>
     </row>
-    <row r="34" spans="1:6" s="25" customFormat="1" ht="58" hidden="1">
+    <row r="34" spans="1:6" s="25" customFormat="1" ht="60" hidden="1">
       <c r="A34" s="24" t="s">
         <v>2282</v>
       </c>
@@ -34537,7 +34537,7 @@
       </c>
       <c r="F34" s="24"/>
     </row>
-    <row r="35" spans="1:6" s="26" customFormat="1" ht="58" hidden="1">
+    <row r="35" spans="1:6" s="26" customFormat="1" ht="60" hidden="1">
       <c r="A35" s="23" t="s">
         <v>2282</v>
       </c>
@@ -34555,7 +34555,7 @@
       </c>
       <c r="F35" s="23"/>
     </row>
-    <row r="36" spans="1:6" s="25" customFormat="1" ht="58" hidden="1">
+    <row r="36" spans="1:6" s="25" customFormat="1" ht="60" hidden="1">
       <c r="A36" s="24" t="s">
         <v>2282</v>
       </c>
@@ -34573,7 +34573,7 @@
       </c>
       <c r="F36" s="24"/>
     </row>
-    <row r="37" spans="1:6" s="26" customFormat="1" ht="58" hidden="1">
+    <row r="37" spans="1:6" s="26" customFormat="1" ht="60" hidden="1">
       <c r="A37" s="23" t="s">
         <v>2282</v>
       </c>
@@ -34591,7 +34591,7 @@
       </c>
       <c r="F37" s="23"/>
     </row>
-    <row r="38" spans="1:6" s="27" customFormat="1" ht="58" hidden="1">
+    <row r="38" spans="1:6" s="27" customFormat="1" ht="60" hidden="1">
       <c r="A38" s="24" t="s">
         <v>2282</v>
       </c>
@@ -34609,7 +34609,7 @@
       </c>
       <c r="F38" s="24"/>
     </row>
-    <row r="39" spans="1:6" s="19" customFormat="1" ht="58" hidden="1">
+    <row r="39" spans="1:6" s="19" customFormat="1" ht="60" hidden="1">
       <c r="A39" s="23" t="s">
         <v>2282</v>
       </c>
@@ -34627,7 +34627,7 @@
       </c>
       <c r="F39" s="23"/>
     </row>
-    <row r="40" spans="1:6" s="27" customFormat="1" ht="58" hidden="1">
+    <row r="40" spans="1:6" s="27" customFormat="1" ht="60" hidden="1">
       <c r="A40" s="24" t="s">
         <v>2282</v>
       </c>
@@ -34645,7 +34645,7 @@
       </c>
       <c r="F40" s="24"/>
     </row>
-    <row r="41" spans="1:6" s="19" customFormat="1" ht="58" hidden="1">
+    <row r="41" spans="1:6" s="19" customFormat="1" ht="60" hidden="1">
       <c r="A41" s="23" t="s">
         <v>2282</v>
       </c>
@@ -34663,7 +34663,7 @@
       </c>
       <c r="F41" s="23"/>
     </row>
-    <row r="42" spans="1:6" s="22" customFormat="1" ht="58" hidden="1">
+    <row r="42" spans="1:6" s="22" customFormat="1" ht="60" hidden="1">
       <c r="A42" s="24" t="s">
         <v>2282</v>
       </c>
@@ -34681,7 +34681,7 @@
       </c>
       <c r="F42" s="24"/>
     </row>
-    <row r="43" spans="1:6" s="22" customFormat="1" ht="58" hidden="1">
+    <row r="43" spans="1:6" s="22" customFormat="1" ht="60" hidden="1">
       <c r="A43" s="23" t="s">
         <v>2282</v>
       </c>
@@ -34699,7 +34699,7 @@
       </c>
       <c r="F43" s="23"/>
     </row>
-    <row r="44" spans="1:6" s="22" customFormat="1" ht="58" hidden="1">
+    <row r="44" spans="1:6" s="22" customFormat="1" ht="60" hidden="1">
       <c r="A44" s="24" t="s">
         <v>2282</v>
       </c>
@@ -34717,7 +34717,7 @@
       </c>
       <c r="F44" s="24"/>
     </row>
-    <row r="45" spans="1:6" s="22" customFormat="1" ht="58" hidden="1">
+    <row r="45" spans="1:6" s="22" customFormat="1" ht="60" hidden="1">
       <c r="A45" s="23" t="s">
         <v>2282</v>
       </c>
@@ -34735,7 +34735,7 @@
       </c>
       <c r="F45" s="23"/>
     </row>
-    <row r="46" spans="1:6" s="22" customFormat="1" ht="58" hidden="1">
+    <row r="46" spans="1:6" s="22" customFormat="1" ht="60" hidden="1">
       <c r="A46" s="24" t="s">
         <v>2282</v>
       </c>
@@ -34753,7 +34753,7 @@
       </c>
       <c r="F46" s="24"/>
     </row>
-    <row r="47" spans="1:6" s="22" customFormat="1" ht="58" hidden="1">
+    <row r="47" spans="1:6" s="22" customFormat="1" ht="60" hidden="1">
       <c r="A47" s="23" t="s">
         <v>2282</v>
       </c>
@@ -34771,7 +34771,7 @@
       </c>
       <c r="F47" s="23"/>
     </row>
-    <row r="48" spans="1:6" s="18" customFormat="1" ht="58" hidden="1">
+    <row r="48" spans="1:6" s="18" customFormat="1" ht="60" hidden="1">
       <c r="A48" s="24" t="s">
         <v>2282</v>
       </c>
@@ -34789,7 +34789,7 @@
       </c>
       <c r="F48" s="24"/>
     </row>
-    <row r="49" spans="1:6" s="17" customFormat="1" ht="58" hidden="1">
+    <row r="49" spans="1:6" s="17" customFormat="1" ht="60" hidden="1">
       <c r="A49" s="23" t="s">
         <v>2282</v>
       </c>
@@ -34807,7 +34807,7 @@
       </c>
       <c r="F49" s="23"/>
     </row>
-    <row r="50" spans="1:6" s="18" customFormat="1" ht="58" hidden="1">
+    <row r="50" spans="1:6" s="18" customFormat="1" ht="60" hidden="1">
       <c r="A50" s="24" t="s">
         <v>2282</v>
       </c>
@@ -34825,7 +34825,7 @@
       </c>
       <c r="F50" s="24"/>
     </row>
-    <row r="51" spans="1:6" s="17" customFormat="1" ht="58" hidden="1">
+    <row r="51" spans="1:6" s="17" customFormat="1" ht="60" hidden="1">
       <c r="A51" s="23" t="s">
         <v>2282</v>
       </c>
@@ -34843,7 +34843,7 @@
       </c>
       <c r="F51" s="23"/>
     </row>
-    <row r="52" spans="1:6" s="18" customFormat="1" ht="58" hidden="1">
+    <row r="52" spans="1:6" s="18" customFormat="1" ht="60" hidden="1">
       <c r="A52" s="24" t="s">
         <v>2282</v>
       </c>
@@ -34861,7 +34861,7 @@
       </c>
       <c r="F52" s="24"/>
     </row>
-    <row r="53" spans="1:6" s="17" customFormat="1" ht="58" hidden="1">
+    <row r="53" spans="1:6" s="17" customFormat="1" ht="60" hidden="1">
       <c r="A53" s="23" t="s">
         <v>2282</v>
       </c>
@@ -34879,7 +34879,7 @@
       </c>
       <c r="F53" s="23"/>
     </row>
-    <row r="54" spans="1:6" s="18" customFormat="1" ht="58" hidden="1">
+    <row r="54" spans="1:6" s="18" customFormat="1" ht="60" hidden="1">
       <c r="A54" s="24" t="s">
         <v>2282</v>
       </c>
@@ -34897,7 +34897,7 @@
       </c>
       <c r="F54" s="24"/>
     </row>
-    <row r="55" spans="1:6" s="17" customFormat="1" ht="58" hidden="1">
+    <row r="55" spans="1:6" s="17" customFormat="1" ht="60" hidden="1">
       <c r="A55" s="23" t="s">
         <v>2282</v>
       </c>
@@ -34915,7 +34915,7 @@
       </c>
       <c r="F55" s="23"/>
     </row>
-    <row r="56" spans="1:6" s="18" customFormat="1" ht="58" hidden="1">
+    <row r="56" spans="1:6" s="18" customFormat="1" ht="60" hidden="1">
       <c r="A56" s="24" t="s">
         <v>2282</v>
       </c>
@@ -34933,7 +34933,7 @@
       </c>
       <c r="F56" s="24"/>
     </row>
-    <row r="57" spans="1:6" s="17" customFormat="1" ht="58" hidden="1">
+    <row r="57" spans="1:6" s="17" customFormat="1" ht="60" hidden="1">
       <c r="A57" s="23" t="s">
         <v>2282</v>
       </c>
@@ -34951,7 +34951,7 @@
       </c>
       <c r="F57" s="23"/>
     </row>
-    <row r="58" spans="1:6" s="18" customFormat="1" ht="58" hidden="1">
+    <row r="58" spans="1:6" s="18" customFormat="1" ht="60" hidden="1">
       <c r="A58" s="24" t="s">
         <v>2282</v>
       </c>
@@ -34969,7 +34969,7 @@
       </c>
       <c r="F58" s="24"/>
     </row>
-    <row r="59" spans="1:6" s="17" customFormat="1" ht="58" hidden="1">
+    <row r="59" spans="1:6" s="17" customFormat="1" ht="60" hidden="1">
       <c r="A59" s="23" t="s">
         <v>2282</v>
       </c>
@@ -34987,7 +34987,7 @@
       </c>
       <c r="F59" s="23"/>
     </row>
-    <row r="60" spans="1:6" s="18" customFormat="1" ht="58" hidden="1">
+    <row r="60" spans="1:6" s="18" customFormat="1" ht="60" hidden="1">
       <c r="A60" s="24" t="s">
         <v>2282</v>
       </c>
@@ -35005,7 +35005,7 @@
       </c>
       <c r="F60" s="24"/>
     </row>
-    <row r="61" spans="1:6" s="17" customFormat="1" ht="58" hidden="1">
+    <row r="61" spans="1:6" s="17" customFormat="1" ht="60" hidden="1">
       <c r="A61" s="23" t="s">
         <v>2282</v>
       </c>
@@ -35023,7 +35023,7 @@
       </c>
       <c r="F61" s="23"/>
     </row>
-    <row r="62" spans="1:6" s="18" customFormat="1" ht="58" hidden="1">
+    <row r="62" spans="1:6" s="18" customFormat="1" ht="60" hidden="1">
       <c r="A62" s="24" t="s">
         <v>2282</v>
       </c>
@@ -35041,7 +35041,7 @@
       </c>
       <c r="F62" s="24"/>
     </row>
-    <row r="63" spans="1:6" s="17" customFormat="1" ht="58" hidden="1">
+    <row r="63" spans="1:6" s="17" customFormat="1" ht="60" hidden="1">
       <c r="A63" s="23" t="s">
         <v>2282</v>
       </c>
@@ -35059,7 +35059,7 @@
       </c>
       <c r="F63" s="23"/>
     </row>
-    <row r="64" spans="1:6" s="18" customFormat="1" ht="58" hidden="1">
+    <row r="64" spans="1:6" s="18" customFormat="1" ht="60" hidden="1">
       <c r="A64" s="24" t="s">
         <v>2282</v>
       </c>
@@ -35077,7 +35077,7 @@
       </c>
       <c r="F64" s="24"/>
     </row>
-    <row r="65" spans="1:6" s="17" customFormat="1" ht="58" hidden="1">
+    <row r="65" spans="1:6" s="17" customFormat="1" ht="60" hidden="1">
       <c r="A65" s="23" t="s">
         <v>2282</v>
       </c>
@@ -35095,7 +35095,7 @@
       </c>
       <c r="F65" s="23"/>
     </row>
-    <row r="66" spans="1:6" s="18" customFormat="1" ht="58" hidden="1">
+    <row r="66" spans="1:6" s="18" customFormat="1" ht="60" hidden="1">
       <c r="A66" s="24" t="s">
         <v>2282</v>
       </c>
@@ -35113,7 +35113,7 @@
       </c>
       <c r="F66" s="24"/>
     </row>
-    <row r="67" spans="1:6" s="17" customFormat="1" ht="58" hidden="1">
+    <row r="67" spans="1:6" s="17" customFormat="1" ht="60" hidden="1">
       <c r="A67" s="23" t="s">
         <v>2282</v>
       </c>
@@ -35131,7 +35131,7 @@
       </c>
       <c r="F67" s="23"/>
     </row>
-    <row r="68" spans="1:6" s="18" customFormat="1" ht="58" hidden="1">
+    <row r="68" spans="1:6" s="18" customFormat="1" ht="60" hidden="1">
       <c r="A68" s="24" t="s">
         <v>2282</v>
       </c>
@@ -36116,11 +36116,11 @@
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="21.83203125" style="53" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.875" style="53" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" style="53"/>
-    <col min="3" max="3" width="63.4140625" style="53" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="63.375" style="53" bestFit="1" customWidth="1"/>
     <col min="4" max="16384" width="9" style="53"/>
   </cols>
   <sheetData>
@@ -36211,7 +36211,7 @@
         <v>3307</v>
       </c>
       <c r="B9" s="53">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -36219,7 +36219,7 @@
         <v>3308</v>
       </c>
       <c r="B10" s="53">
-        <v>100</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -36234,7 +36234,7 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="9" style="53"/>
     <col min="2" max="2" width="45.75" style="53" customWidth="1"/>
@@ -36358,20 +36358,20 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:Q21"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.83203125" style="1"/>
+    <col min="1" max="1" width="7.875" style="1"/>
     <col min="2" max="2" width="6.5" style="1" customWidth="1"/>
-    <col min="3" max="4" width="7.83203125" style="1"/>
+    <col min="3" max="4" width="7.875" style="1"/>
     <col min="5" max="5" width="12.5" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" style="1" customWidth="1"/>
-    <col min="7" max="8" width="7.83203125" style="1"/>
+    <col min="6" max="6" width="8.875" style="1" customWidth="1"/>
+    <col min="7" max="8" width="7.875" style="1"/>
     <col min="9" max="9" width="10.25" style="1" customWidth="1"/>
     <col min="10" max="10" width="7.25" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.33203125" style="1" customWidth="1"/>
-    <col min="12" max="14" width="7.83203125" style="1"/>
-    <col min="15" max="15" width="9.33203125" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="7.83203125" style="1"/>
+    <col min="11" max="11" width="9.375" style="1" customWidth="1"/>
+    <col min="12" max="14" width="7.875" style="1"/>
+    <col min="15" max="15" width="9.375" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="7.875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -36947,22 +36947,22 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:M20"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.83203125" style="1"/>
-    <col min="2" max="2" width="6.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" style="1"/>
+    <col min="2" max="2" width="6.625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.75" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.08203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.75" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.83203125" style="1"/>
-    <col min="12" max="12" width="10.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.875" style="1"/>
+    <col min="12" max="12" width="10.625" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="7.83203125" style="1"/>
+    <col min="14" max="16384" width="7.875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -37403,20 +37403,20 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:L21"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.83203125" style="1"/>
-    <col min="2" max="2" width="15.08203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" style="1"/>
+    <col min="2" max="2" width="15.125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.5" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.75" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5.25" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.08203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.08203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="7.83203125" style="1"/>
+    <col min="10" max="10" width="16.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="7.875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -37772,7 +37772,7 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="9" style="52"/>
     <col min="2" max="2" width="15" style="52" bestFit="1" customWidth="1"/>
@@ -37886,7 +37886,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83C84FF1-A0EA-48F0-9BC3-5F8DC52E9A0A}">
   <dimension ref="A1:O210"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15" style="12" customWidth="1"/>
     <col min="2" max="5" width="15" style="5" customWidth="1"/>
@@ -37894,7 +37894,7 @@
     <col min="7" max="10" width="15" style="5" customWidth="1"/>
     <col min="11" max="11" width="15" style="12" customWidth="1"/>
     <col min="12" max="15" width="15" style="5" customWidth="1"/>
-    <col min="16" max="16384" width="7.83203125" style="5"/>
+    <col min="16" max="16384" width="7.875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="12" customFormat="1">
@@ -43505,15 +43505,15 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F6A446E-DC4A-45B3-A3E3-4049BF48BC30}">
   <dimension ref="A1:G503"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.58203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.375" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.5" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="7.83203125" style="5"/>
+    <col min="5" max="5" width="6.875" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.875" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="7.875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="12" customFormat="1">
@@ -54504,7 +54504,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="459" spans="1:7" ht="15.5">
+    <row r="459" spans="1:7">
       <c r="A459" t="s">
         <v>694</v>
       </c>

</xml_diff>

<commit_message>
added reforge recipes, but don't use, it may reforge you uniques into rare
</commit_message>
<xml_diff>
--- a/Diablo II.xlsx
+++ b/Diablo II.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yatyr\workspace\d2r-loot-filter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8296B1F8-4853-4409-96E9-D48D267DBCF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C91EBA1-4EC3-4CB0-AF7B-5034F85FDFFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="12" xr2:uid="{4FA0E628-D5C1-45F8-838A-535ABF901563}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{4FA0E628-D5C1-45F8-838A-535ABF901563}"/>
   </bookViews>
   <sheets>
     <sheet name="Mod-Config" sheetId="6" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8368" uniqueCount="3362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8371" uniqueCount="3364">
   <si>
     <t>Key</t>
   </si>
@@ -11836,6 +11836,14 @@
     <t>Normal items + Rune01~06 -&gt; Add 1~6 sockets; Any item + Ort + Jewel -&gt; Larzuk Socket</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>Enable Reforge Recipes</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Unique/Set item + Scroll of Identify -&gt; Salvage to Andariel Essence, 3x Andariel Essence -&gt; Mephisto Essence, 3x Mephisto Essence -&gt; Diablo Essence, 3x Diablo Essence -&gt; Baal Essence, Unique/Set item + Token of Absolution -&gt; Reforged unique/set item</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -11845,13 +11853,13 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -11859,7 +11867,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -12409,8 +12417,8 @@
     <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{53F17FA5-8A83-41A1-8800-C9AE149B41E5}"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="10">
     <dxf>
@@ -12836,10 +12844,10 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.83203125" style="88" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.875" style="88" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" style="88"/>
     <col min="3" max="3" width="72.25" style="88" bestFit="1" customWidth="1"/>
     <col min="4" max="16384" width="9" style="88"/>
@@ -12952,6 +12960,17 @@
       </c>
       <c r="C11" s="88" t="s">
         <v>3361</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="88" t="s">
+        <v>3362</v>
+      </c>
+      <c r="B12" s="88" t="s">
+        <v>3360</v>
+      </c>
+      <c r="C12" s="88" t="s">
+        <v>3363</v>
       </c>
     </row>
   </sheetData>
@@ -12966,14 +12985,14 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:F247"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="57.08203125" style="64" customWidth="1"/>
-    <col min="2" max="2" width="14.58203125" style="46" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="57.125" style="64" customWidth="1"/>
+    <col min="2" max="2" width="14.625" style="46" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.5" style="46" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" style="46" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.08203125" style="46" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.83203125" style="46" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.875" style="46" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.125" style="46" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.875" style="46" bestFit="1" customWidth="1"/>
     <col min="7" max="16384" width="9" style="46"/>
   </cols>
   <sheetData>
@@ -14641,7 +14660,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="95" spans="1:6" ht="46.5">
+    <row r="95" spans="1:6" ht="47.25">
       <c r="A95" s="69" t="s">
         <v>3090</v>
       </c>
@@ -17494,14 +17513,14 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:F34"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="3.5" style="65" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.58203125" style="65" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="58.33203125" style="65" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.625" style="65" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58.375" style="65" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="38.25" style="65" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="38.25" style="68" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.83203125" style="65" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.875" style="65" bestFit="1" customWidth="1"/>
     <col min="7" max="16384" width="9" style="65"/>
   </cols>
   <sheetData>
@@ -18197,14 +18216,14 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:G105"/>
-  <sheetFormatPr defaultColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.08203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.58203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.08203125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="37.08203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.125" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.625" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="37.125" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="26.5" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="70.83203125" style="10" customWidth="1"/>
+    <col min="6" max="6" width="70.875" style="10" customWidth="1"/>
     <col min="7" max="7" width="34.75" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="8" style="5"/>
   </cols>
@@ -18232,7 +18251,7 @@
         <v>2675</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="58">
+    <row r="2" spans="1:7" ht="60">
       <c r="A2" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18255,7 +18274,7 @@
         <v>1850</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="87">
+    <row r="3" spans="1:7" ht="90">
       <c r="A3" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18278,7 +18297,7 @@
         <v>1854</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="101.5">
+    <row r="4" spans="1:7" ht="105">
       <c r="A4" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18301,7 +18320,7 @@
         <v>1859</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="101.5">
+    <row r="5" spans="1:7" ht="105">
       <c r="A5" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18324,7 +18343,7 @@
         <v>1863</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="87">
+    <row r="6" spans="1:7" ht="90">
       <c r="A6" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18347,7 +18366,7 @@
         <v>1867</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="87">
+    <row r="7" spans="1:7" ht="90">
       <c r="A7" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18370,7 +18389,7 @@
         <v>1871</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="87">
+    <row r="8" spans="1:7" ht="90">
       <c r="A8" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18393,7 +18412,7 @@
         <v>1876</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="87">
+    <row r="9" spans="1:7" ht="90">
       <c r="A9" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18416,7 +18435,7 @@
         <v>1881</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="58">
+    <row r="10" spans="1:7" ht="60">
       <c r="A10" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18439,7 +18458,7 @@
         <v>1885</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="87">
+    <row r="11" spans="1:7" ht="90">
       <c r="A11" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18462,7 +18481,7 @@
         <v>1889</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="87">
+    <row r="12" spans="1:7" ht="90">
       <c r="A12" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18485,7 +18504,7 @@
         <v>1894</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="101.5">
+    <row r="13" spans="1:7" ht="105">
       <c r="A13" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18508,7 +18527,7 @@
         <v>1899</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="87">
+    <row r="14" spans="1:7" ht="90">
       <c r="A14" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18531,7 +18550,7 @@
         <v>1903</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="87">
+    <row r="15" spans="1:7" ht="90">
       <c r="A15" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18554,7 +18573,7 @@
         <v>1907</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="87">
+    <row r="16" spans="1:7" ht="90">
       <c r="A16" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18577,7 +18596,7 @@
         <v>1911</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="101.5">
+    <row r="17" spans="1:7" ht="105">
       <c r="A17" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18600,7 +18619,7 @@
         <v>1916</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="87">
+    <row r="18" spans="1:7" ht="90">
       <c r="A18" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18623,7 +18642,7 @@
         <v>1920</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="87">
+    <row r="19" spans="1:7" ht="90">
       <c r="A19" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18646,7 +18665,7 @@
         <v>2543</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="72.5">
+    <row r="20" spans="1:7" ht="75">
       <c r="A20" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18669,7 +18688,7 @@
         <v>2545</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="58">
+    <row r="21" spans="1:7" ht="60">
       <c r="A21" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18692,7 +18711,7 @@
         <v>2547</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="72.5">
+    <row r="22" spans="1:7" ht="75">
       <c r="A22" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18715,7 +18734,7 @@
         <v>2549</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="43.5">
+    <row r="23" spans="1:7" ht="45">
       <c r="A23" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18738,7 +18757,7 @@
         <v>2551</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="101.5">
+    <row r="24" spans="1:7" ht="105">
       <c r="A24" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18761,7 +18780,7 @@
         <v>2553</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="87">
+    <row r="25" spans="1:7" ht="90">
       <c r="A25" s="6" t="s">
         <v>1652</v>
       </c>
@@ -18784,7 +18803,7 @@
         <v>2555</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="101.5">
+    <row r="26" spans="1:7" ht="105">
       <c r="A26" s="6" t="s">
         <v>1934</v>
       </c>
@@ -18807,7 +18826,7 @@
         <v>2557</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="101.5">
+    <row r="27" spans="1:7" ht="105">
       <c r="A27" s="6" t="s">
         <v>1934</v>
       </c>
@@ -18830,7 +18849,7 @@
         <v>2559</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="101.5">
+    <row r="28" spans="1:7" ht="105">
       <c r="A28" s="6" t="s">
         <v>1934</v>
       </c>
@@ -18853,7 +18872,7 @@
         <v>2561</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="101.5">
+    <row r="29" spans="1:7" ht="105">
       <c r="A29" s="6" t="s">
         <v>1934</v>
       </c>
@@ -18876,7 +18895,7 @@
         <v>2562</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="101.5">
+    <row r="30" spans="1:7" ht="105">
       <c r="A30" s="6" t="s">
         <v>1934</v>
       </c>
@@ -18899,7 +18918,7 @@
         <v>2564</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="101.5">
+    <row r="31" spans="1:7" ht="105">
       <c r="A31" s="6" t="s">
         <v>1934</v>
       </c>
@@ -18922,7 +18941,7 @@
         <v>2566</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="101.5">
+    <row r="32" spans="1:7" ht="105">
       <c r="A32" s="6" t="s">
         <v>1934</v>
       </c>
@@ -18945,7 +18964,7 @@
         <v>2568</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="101.5">
+    <row r="33" spans="1:7" ht="105">
       <c r="A33" s="6" t="s">
         <v>1934</v>
       </c>
@@ -18968,7 +18987,7 @@
         <v>2570</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="101.5">
+    <row r="34" spans="1:7" ht="105">
       <c r="A34" s="6" t="s">
         <v>1934</v>
       </c>
@@ -18991,7 +19010,7 @@
         <v>2571</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="101.5">
+    <row r="35" spans="1:7" ht="105">
       <c r="A35" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19014,7 +19033,7 @@
         <v>2573</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="116">
+    <row r="36" spans="1:7" ht="120">
       <c r="A36" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19037,7 +19056,7 @@
         <v>2574</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="101.5">
+    <row r="37" spans="1:7" ht="105">
       <c r="A37" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19060,7 +19079,7 @@
         <v>2575</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="101.5">
+    <row r="38" spans="1:7" ht="105">
       <c r="A38" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19083,7 +19102,7 @@
         <v>2576</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="116">
+    <row r="39" spans="1:7" ht="120">
       <c r="A39" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19106,7 +19125,7 @@
         <v>2577</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="101.5">
+    <row r="40" spans="1:7" ht="105">
       <c r="A40" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19129,7 +19148,7 @@
         <v>2579</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="101.5">
+    <row r="41" spans="1:7" ht="105">
       <c r="A41" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19152,7 +19171,7 @@
         <v>2581</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="101.5">
+    <row r="42" spans="1:7" ht="105">
       <c r="A42" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19175,7 +19194,7 @@
         <v>2583</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="101.5">
+    <row r="43" spans="1:7" ht="105">
       <c r="A43" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19198,7 +19217,7 @@
         <v>2584</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="101.5">
+    <row r="44" spans="1:7" ht="105">
       <c r="A44" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19221,7 +19240,7 @@
         <v>2586</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="101.5">
+    <row r="45" spans="1:7" ht="105">
       <c r="A45" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19244,7 +19263,7 @@
         <v>2588</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="101.5">
+    <row r="46" spans="1:7" ht="105">
       <c r="A46" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19267,7 +19286,7 @@
         <v>2590</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="101.5">
+    <row r="47" spans="1:7" ht="105">
       <c r="A47" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19290,7 +19309,7 @@
         <v>2592</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="101.5">
+    <row r="48" spans="1:7" ht="105">
       <c r="A48" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19313,7 +19332,7 @@
         <v>2594</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="101.5">
+    <row r="49" spans="1:7" ht="105">
       <c r="A49" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19336,7 +19355,7 @@
         <v>2596</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="87">
+    <row r="50" spans="1:7" ht="90">
       <c r="A50" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19359,7 +19378,7 @@
         <v>2598</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="101.5">
+    <row r="51" spans="1:7" ht="105">
       <c r="A51" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19382,7 +19401,7 @@
         <v>2600</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="101.5">
+    <row r="52" spans="1:7" ht="105">
       <c r="A52" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19405,7 +19424,7 @@
         <v>2601</v>
       </c>
     </row>
-    <row r="53" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="53" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A53" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19428,7 +19447,7 @@
         <v>2602</v>
       </c>
     </row>
-    <row r="54" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="54" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A54" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19451,7 +19470,7 @@
         <v>2604</v>
       </c>
     </row>
-    <row r="55" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="55" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A55" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19474,7 +19493,7 @@
         <v>2605</v>
       </c>
     </row>
-    <row r="56" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="56" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A56" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19497,7 +19516,7 @@
         <v>2607</v>
       </c>
     </row>
-    <row r="57" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="57" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A57" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19520,7 +19539,7 @@
         <v>2608</v>
       </c>
     </row>
-    <row r="58" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="58" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A58" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19543,7 +19562,7 @@
         <v>2610</v>
       </c>
     </row>
-    <row r="59" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="59" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A59" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19566,7 +19585,7 @@
         <v>2612</v>
       </c>
     </row>
-    <row r="60" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="60" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A60" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19589,7 +19608,7 @@
         <v>2614</v>
       </c>
     </row>
-    <row r="61" spans="1:7" s="4" customFormat="1" ht="116">
+    <row r="61" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A61" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19612,7 +19631,7 @@
         <v>2615</v>
       </c>
     </row>
-    <row r="62" spans="1:7" s="4" customFormat="1" ht="130.5">
+    <row r="62" spans="1:7" s="4" customFormat="1" ht="135">
       <c r="A62" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19635,7 +19654,7 @@
         <v>2616</v>
       </c>
     </row>
-    <row r="63" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="63" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A63" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19658,7 +19677,7 @@
         <v>2618</v>
       </c>
     </row>
-    <row r="64" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="64" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A64" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19681,7 +19700,7 @@
         <v>2620</v>
       </c>
     </row>
-    <row r="65" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="65" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A65" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19704,7 +19723,7 @@
         <v>2622</v>
       </c>
     </row>
-    <row r="66" spans="1:7" s="4" customFormat="1" ht="116">
+    <row r="66" spans="1:7" s="4" customFormat="1" ht="120">
       <c r="A66" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19727,7 +19746,7 @@
         <v>2624</v>
       </c>
     </row>
-    <row r="67" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="67" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A67" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19750,7 +19769,7 @@
         <v>2625</v>
       </c>
     </row>
-    <row r="68" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="68" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A68" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19773,7 +19792,7 @@
         <v>2627</v>
       </c>
     </row>
-    <row r="69" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="69" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A69" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19796,7 +19815,7 @@
         <v>2629</v>
       </c>
     </row>
-    <row r="70" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="70" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A70" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19819,7 +19838,7 @@
         <v>2631</v>
       </c>
     </row>
-    <row r="71" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="71" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A71" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19842,7 +19861,7 @@
         <v>2632</v>
       </c>
     </row>
-    <row r="72" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="72" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A72" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19865,7 +19884,7 @@
         <v>2635</v>
       </c>
     </row>
-    <row r="73" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="73" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A73" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19888,7 +19907,7 @@
         <v>2637</v>
       </c>
     </row>
-    <row r="74" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="74" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A74" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19911,7 +19930,7 @@
         <v>2639</v>
       </c>
     </row>
-    <row r="75" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="75" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A75" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19934,7 +19953,7 @@
         <v>2641</v>
       </c>
     </row>
-    <row r="76" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="76" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A76" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19957,7 +19976,7 @@
         <v>2642</v>
       </c>
     </row>
-    <row r="77" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="77" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A77" s="6" t="s">
         <v>1934</v>
       </c>
@@ -19980,7 +19999,7 @@
         <v>2644</v>
       </c>
     </row>
-    <row r="78" spans="1:7" s="4" customFormat="1" ht="58">
+    <row r="78" spans="1:7" s="4" customFormat="1" ht="60">
       <c r="A78" s="6" t="s">
         <v>2024</v>
       </c>
@@ -20003,7 +20022,7 @@
         <v>2646</v>
       </c>
     </row>
-    <row r="79" spans="1:7" s="4" customFormat="1" ht="58">
+    <row r="79" spans="1:7" s="4" customFormat="1" ht="60">
       <c r="A79" s="6" t="s">
         <v>2024</v>
       </c>
@@ -20026,7 +20045,7 @@
         <v>2648</v>
       </c>
     </row>
-    <row r="80" spans="1:7" s="4" customFormat="1" ht="58">
+    <row r="80" spans="1:7" s="4" customFormat="1" ht="60">
       <c r="A80" s="6" t="s">
         <v>2024</v>
       </c>
@@ -20049,7 +20068,7 @@
         <v>2650</v>
       </c>
     </row>
-    <row r="81" spans="1:7" s="4" customFormat="1" ht="58">
+    <row r="81" spans="1:7" s="4" customFormat="1" ht="60">
       <c r="A81" s="6" t="s">
         <v>2024</v>
       </c>
@@ -20072,7 +20091,7 @@
         <v>2652</v>
       </c>
     </row>
-    <row r="82" spans="1:7" s="4" customFormat="1" ht="58">
+    <row r="82" spans="1:7" s="4" customFormat="1" ht="60">
       <c r="A82" s="6" t="s">
         <v>2024</v>
       </c>
@@ -20095,7 +20114,7 @@
         <v>2654</v>
       </c>
     </row>
-    <row r="83" spans="1:7" s="4" customFormat="1" ht="58">
+    <row r="83" spans="1:7" s="4" customFormat="1" ht="60">
       <c r="A83" s="6" t="s">
         <v>2024</v>
       </c>
@@ -20118,7 +20137,7 @@
         <v>2656</v>
       </c>
     </row>
-    <row r="84" spans="1:7" s="4" customFormat="1" ht="58">
+    <row r="84" spans="1:7" s="4" customFormat="1" ht="60">
       <c r="A84" s="6" t="s">
         <v>2024</v>
       </c>
@@ -20141,7 +20160,7 @@
         <v>2658</v>
       </c>
     </row>
-    <row r="85" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="85" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A85" s="6" t="s">
         <v>2039</v>
       </c>
@@ -20164,7 +20183,7 @@
         <v>2660</v>
       </c>
     </row>
-    <row r="86" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="86" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A86" s="6" t="s">
         <v>2039</v>
       </c>
@@ -20187,7 +20206,7 @@
         <v>2662</v>
       </c>
     </row>
-    <row r="87" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="87" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A87" s="6" t="s">
         <v>2039</v>
       </c>
@@ -20210,7 +20229,7 @@
         <v>2664</v>
       </c>
     </row>
-    <row r="88" spans="1:7" s="4" customFormat="1" ht="87">
+    <row r="88" spans="1:7" s="4" customFormat="1" ht="90">
       <c r="A88" s="6" t="s">
         <v>2039</v>
       </c>
@@ -20233,7 +20252,7 @@
         <v>2666</v>
       </c>
     </row>
-    <row r="89" spans="1:7" s="4" customFormat="1" ht="101.5">
+    <row r="89" spans="1:7" s="4" customFormat="1" ht="105">
       <c r="A89" s="6" t="s">
         <v>2039</v>
       </c>
@@ -20256,7 +20275,7 @@
         <v>2668</v>
       </c>
     </row>
-    <row r="90" spans="1:7" s="4" customFormat="1" ht="87">
+    <row r="90" spans="1:7" s="4" customFormat="1" ht="90">
       <c r="A90" s="6" t="s">
         <v>2039</v>
       </c>
@@ -20279,7 +20298,7 @@
         <v>2671</v>
       </c>
     </row>
-    <row r="91" spans="1:7" s="4" customFormat="1" ht="87">
+    <row r="91" spans="1:7" s="4" customFormat="1" ht="90">
       <c r="A91" s="6" t="s">
         <v>2039</v>
       </c>
@@ -20302,7 +20321,7 @@
         <v>2673</v>
       </c>
     </row>
-    <row r="92" spans="1:7" ht="72.5">
+    <row r="92" spans="1:7" ht="75">
       <c r="A92" s="6" t="s">
         <v>2678</v>
       </c>
@@ -20325,7 +20344,7 @@
         <v>2681</v>
       </c>
     </row>
-    <row r="93" spans="1:7" ht="72.5">
+    <row r="93" spans="1:7" ht="75">
       <c r="A93" s="6" t="s">
         <v>2678</v>
       </c>
@@ -20348,7 +20367,7 @@
         <v>2685</v>
       </c>
     </row>
-    <row r="94" spans="1:7" ht="72.5">
+    <row r="94" spans="1:7" ht="75">
       <c r="A94" s="6" t="s">
         <v>2678</v>
       </c>
@@ -20371,7 +20390,7 @@
         <v>2689</v>
       </c>
     </row>
-    <row r="95" spans="1:7" ht="58">
+    <row r="95" spans="1:7" ht="60">
       <c r="A95" s="6" t="s">
         <v>2678</v>
       </c>
@@ -20394,7 +20413,7 @@
         <v>2691</v>
       </c>
     </row>
-    <row r="96" spans="1:7" ht="116">
+    <row r="96" spans="1:7" ht="120">
       <c r="A96" s="6" t="s">
         <v>2678</v>
       </c>
@@ -20417,7 +20436,7 @@
         <v>2695</v>
       </c>
     </row>
-    <row r="97" spans="1:7" ht="145">
+    <row r="97" spans="1:7" ht="150">
       <c r="A97" s="6" t="s">
         <v>2678</v>
       </c>
@@ -20440,7 +20459,7 @@
         <v>2699</v>
       </c>
     </row>
-    <row r="98" spans="1:7" ht="72.5">
+    <row r="98" spans="1:7" ht="75">
       <c r="A98" s="6" t="s">
         <v>2678</v>
       </c>
@@ -20463,7 +20482,7 @@
         <v>2703</v>
       </c>
     </row>
-    <row r="99" spans="1:7" ht="58">
+    <row r="99" spans="1:7" ht="60">
       <c r="A99" s="6" t="s">
         <v>2678</v>
       </c>
@@ -20486,7 +20505,7 @@
         <v>2707</v>
       </c>
     </row>
-    <row r="100" spans="1:7" ht="58">
+    <row r="100" spans="1:7" ht="60">
       <c r="A100" s="6" t="s">
         <v>2678</v>
       </c>
@@ -20509,7 +20528,7 @@
         <v>2711</v>
       </c>
     </row>
-    <row r="101" spans="1:7" ht="58">
+    <row r="101" spans="1:7" ht="60">
       <c r="A101" s="6" t="s">
         <v>3244</v>
       </c>
@@ -20532,7 +20551,7 @@
         <v>3246</v>
       </c>
     </row>
-    <row r="102" spans="1:7" ht="87">
+    <row r="102" spans="1:7" ht="90">
       <c r="A102" s="6" t="s">
         <v>3244</v>
       </c>
@@ -20555,7 +20574,7 @@
         <v>3251</v>
       </c>
     </row>
-    <row r="103" spans="1:7" ht="87">
+    <row r="103" spans="1:7" ht="90">
       <c r="A103" s="6" t="s">
         <v>3244</v>
       </c>
@@ -20578,7 +20597,7 @@
         <v>3255</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="101.5">
+    <row r="104" spans="1:7" ht="105">
       <c r="A104" s="6" t="s">
         <v>3244</v>
       </c>
@@ -20601,7 +20620,7 @@
         <v>3260</v>
       </c>
     </row>
-    <row r="105" spans="1:7" ht="101.5">
+    <row r="105" spans="1:7" ht="105">
       <c r="A105" s="6" t="s">
         <v>3244</v>
       </c>
@@ -20638,16 +20657,16 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:M140"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.75" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="3.33203125" style="5" customWidth="1"/>
+    <col min="3" max="5" width="3.375" style="5" customWidth="1"/>
     <col min="6" max="6" width="16" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="3.58203125" style="5" customWidth="1"/>
-    <col min="10" max="10" width="16.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="3.33203125" style="5" customWidth="1"/>
-    <col min="14" max="16384" width="7.83203125" style="5"/>
+    <col min="7" max="9" width="3.625" style="5" customWidth="1"/>
+    <col min="10" max="10" width="16.375" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="3.375" style="5" customWidth="1"/>
+    <col min="14" max="16384" width="7.875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -26421,12 +26440,12 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:F120"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.25" style="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="12.58203125" style="6" customWidth="1"/>
+    <col min="2" max="4" width="12.625" style="6" customWidth="1"/>
     <col min="5" max="5" width="35.75" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="7.83203125" style="5"/>
+    <col min="6" max="16384" width="7.875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -28843,14 +28862,14 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:F126"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="7.83203125" style="21"/>
+    <col min="1" max="2" width="7.875" style="21"/>
     <col min="3" max="3" width="16.5" style="21" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="40.33203125" style="37" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="40.375" style="37" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="60.75" style="37" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" style="21" customWidth="1"/>
-    <col min="7" max="16384" width="7.83203125" style="21"/>
+    <col min="6" max="6" width="45.875" style="21" customWidth="1"/>
+    <col min="7" max="16384" width="7.875" style="21"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="16" customFormat="1">
@@ -29419,7 +29438,7 @@
         <v>2353</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="29">
+    <row r="31" spans="1:6" ht="30">
       <c r="A31" s="20" t="s">
         <v>2279</v>
       </c>
@@ -29457,7 +29476,7 @@
       </c>
       <c r="F32" s="22"/>
     </row>
-    <row r="33" spans="1:6" ht="58">
+    <row r="33" spans="1:6" ht="60">
       <c r="A33" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29475,7 +29494,7 @@
       </c>
       <c r="F33" s="23"/>
     </row>
-    <row r="34" spans="1:6" s="25" customFormat="1" ht="58">
+    <row r="34" spans="1:6" s="25" customFormat="1" ht="60">
       <c r="A34" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29493,7 +29512,7 @@
       </c>
       <c r="F34" s="24"/>
     </row>
-    <row r="35" spans="1:6" s="26" customFormat="1" ht="58">
+    <row r="35" spans="1:6" s="26" customFormat="1" ht="60">
       <c r="A35" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29511,7 +29530,7 @@
       </c>
       <c r="F35" s="23"/>
     </row>
-    <row r="36" spans="1:6" s="25" customFormat="1" ht="58">
+    <row r="36" spans="1:6" s="25" customFormat="1" ht="60">
       <c r="A36" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29529,7 +29548,7 @@
       </c>
       <c r="F36" s="24"/>
     </row>
-    <row r="37" spans="1:6" s="26" customFormat="1" ht="58">
+    <row r="37" spans="1:6" s="26" customFormat="1" ht="60">
       <c r="A37" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29547,7 +29566,7 @@
       </c>
       <c r="F37" s="23"/>
     </row>
-    <row r="38" spans="1:6" s="27" customFormat="1" ht="58">
+    <row r="38" spans="1:6" s="27" customFormat="1" ht="60">
       <c r="A38" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29565,7 +29584,7 @@
       </c>
       <c r="F38" s="24"/>
     </row>
-    <row r="39" spans="1:6" s="19" customFormat="1" ht="58">
+    <row r="39" spans="1:6" s="19" customFormat="1" ht="60">
       <c r="A39" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29583,7 +29602,7 @@
       </c>
       <c r="F39" s="23"/>
     </row>
-    <row r="40" spans="1:6" s="27" customFormat="1" ht="58">
+    <row r="40" spans="1:6" s="27" customFormat="1" ht="60">
       <c r="A40" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29601,7 +29620,7 @@
       </c>
       <c r="F40" s="24"/>
     </row>
-    <row r="41" spans="1:6" s="19" customFormat="1" ht="58">
+    <row r="41" spans="1:6" s="19" customFormat="1" ht="60">
       <c r="A41" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29619,7 +29638,7 @@
       </c>
       <c r="F41" s="23"/>
     </row>
-    <row r="42" spans="1:6" s="22" customFormat="1" ht="58">
+    <row r="42" spans="1:6" s="22" customFormat="1" ht="60">
       <c r="A42" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29637,7 +29656,7 @@
       </c>
       <c r="F42" s="24"/>
     </row>
-    <row r="43" spans="1:6" s="22" customFormat="1" ht="58">
+    <row r="43" spans="1:6" s="22" customFormat="1" ht="60">
       <c r="A43" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29655,7 +29674,7 @@
       </c>
       <c r="F43" s="23"/>
     </row>
-    <row r="44" spans="1:6" s="22" customFormat="1" ht="58">
+    <row r="44" spans="1:6" s="22" customFormat="1" ht="60">
       <c r="A44" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29673,7 +29692,7 @@
       </c>
       <c r="F44" s="24"/>
     </row>
-    <row r="45" spans="1:6" s="22" customFormat="1" ht="58">
+    <row r="45" spans="1:6" s="22" customFormat="1" ht="60">
       <c r="A45" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29691,7 +29710,7 @@
       </c>
       <c r="F45" s="23"/>
     </row>
-    <row r="46" spans="1:6" s="22" customFormat="1" ht="58">
+    <row r="46" spans="1:6" s="22" customFormat="1" ht="60">
       <c r="A46" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29709,7 +29728,7 @@
       </c>
       <c r="F46" s="24"/>
     </row>
-    <row r="47" spans="1:6" s="22" customFormat="1" ht="58">
+    <row r="47" spans="1:6" s="22" customFormat="1" ht="60">
       <c r="A47" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29727,7 +29746,7 @@
       </c>
       <c r="F47" s="23"/>
     </row>
-    <row r="48" spans="1:6" s="18" customFormat="1" ht="58">
+    <row r="48" spans="1:6" s="18" customFormat="1" ht="60">
       <c r="A48" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29745,7 +29764,7 @@
       </c>
       <c r="F48" s="24"/>
     </row>
-    <row r="49" spans="1:6" s="17" customFormat="1" ht="58">
+    <row r="49" spans="1:6" s="17" customFormat="1" ht="60">
       <c r="A49" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29763,7 +29782,7 @@
       </c>
       <c r="F49" s="23"/>
     </row>
-    <row r="50" spans="1:6" s="18" customFormat="1" ht="58">
+    <row r="50" spans="1:6" s="18" customFormat="1" ht="60">
       <c r="A50" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29781,7 +29800,7 @@
       </c>
       <c r="F50" s="24"/>
     </row>
-    <row r="51" spans="1:6" s="17" customFormat="1" ht="58">
+    <row r="51" spans="1:6" s="17" customFormat="1" ht="60">
       <c r="A51" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29799,7 +29818,7 @@
       </c>
       <c r="F51" s="23"/>
     </row>
-    <row r="52" spans="1:6" s="18" customFormat="1" ht="58">
+    <row r="52" spans="1:6" s="18" customFormat="1" ht="60">
       <c r="A52" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29817,7 +29836,7 @@
       </c>
       <c r="F52" s="24"/>
     </row>
-    <row r="53" spans="1:6" s="17" customFormat="1" ht="58">
+    <row r="53" spans="1:6" s="17" customFormat="1" ht="60">
       <c r="A53" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29835,7 +29854,7 @@
       </c>
       <c r="F53" s="23"/>
     </row>
-    <row r="54" spans="1:6" s="18" customFormat="1" ht="58">
+    <row r="54" spans="1:6" s="18" customFormat="1" ht="60">
       <c r="A54" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29853,7 +29872,7 @@
       </c>
       <c r="F54" s="24"/>
     </row>
-    <row r="55" spans="1:6" s="17" customFormat="1" ht="58">
+    <row r="55" spans="1:6" s="17" customFormat="1" ht="60">
       <c r="A55" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29871,7 +29890,7 @@
       </c>
       <c r="F55" s="23"/>
     </row>
-    <row r="56" spans="1:6" s="18" customFormat="1" ht="58">
+    <row r="56" spans="1:6" s="18" customFormat="1" ht="60">
       <c r="A56" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29889,7 +29908,7 @@
       </c>
       <c r="F56" s="24"/>
     </row>
-    <row r="57" spans="1:6" s="17" customFormat="1" ht="58">
+    <row r="57" spans="1:6" s="17" customFormat="1" ht="60">
       <c r="A57" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29907,7 +29926,7 @@
       </c>
       <c r="F57" s="23"/>
     </row>
-    <row r="58" spans="1:6" s="18" customFormat="1" ht="58">
+    <row r="58" spans="1:6" s="18" customFormat="1" ht="60">
       <c r="A58" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29925,7 +29944,7 @@
       </c>
       <c r="F58" s="24"/>
     </row>
-    <row r="59" spans="1:6" s="17" customFormat="1" ht="58">
+    <row r="59" spans="1:6" s="17" customFormat="1" ht="60">
       <c r="A59" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29943,7 +29962,7 @@
       </c>
       <c r="F59" s="23"/>
     </row>
-    <row r="60" spans="1:6" s="18" customFormat="1" ht="58">
+    <row r="60" spans="1:6" s="18" customFormat="1" ht="60">
       <c r="A60" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29961,7 +29980,7 @@
       </c>
       <c r="F60" s="24"/>
     </row>
-    <row r="61" spans="1:6" s="17" customFormat="1" ht="58">
+    <row r="61" spans="1:6" s="17" customFormat="1" ht="60">
       <c r="A61" s="23" t="s">
         <v>2279</v>
       </c>
@@ -29979,7 +29998,7 @@
       </c>
       <c r="F61" s="23"/>
     </row>
-    <row r="62" spans="1:6" s="18" customFormat="1" ht="58">
+    <row r="62" spans="1:6" s="18" customFormat="1" ht="60">
       <c r="A62" s="24" t="s">
         <v>2279</v>
       </c>
@@ -29997,7 +30016,7 @@
       </c>
       <c r="F62" s="24"/>
     </row>
-    <row r="63" spans="1:6" s="17" customFormat="1" ht="58">
+    <row r="63" spans="1:6" s="17" customFormat="1" ht="60">
       <c r="A63" s="23" t="s">
         <v>2279</v>
       </c>
@@ -30015,7 +30034,7 @@
       </c>
       <c r="F63" s="23"/>
     </row>
-    <row r="64" spans="1:6" s="18" customFormat="1" ht="58">
+    <row r="64" spans="1:6" s="18" customFormat="1" ht="60">
       <c r="A64" s="24" t="s">
         <v>2279</v>
       </c>
@@ -30033,7 +30052,7 @@
       </c>
       <c r="F64" s="24"/>
     </row>
-    <row r="65" spans="1:6" s="17" customFormat="1" ht="58">
+    <row r="65" spans="1:6" s="17" customFormat="1" ht="60">
       <c r="A65" s="23" t="s">
         <v>2279</v>
       </c>
@@ -30051,7 +30070,7 @@
       </c>
       <c r="F65" s="23"/>
     </row>
-    <row r="66" spans="1:6" s="18" customFormat="1" ht="58">
+    <row r="66" spans="1:6" s="18" customFormat="1" ht="60">
       <c r="A66" s="24" t="s">
         <v>2279</v>
       </c>
@@ -30069,7 +30088,7 @@
       </c>
       <c r="F66" s="24"/>
     </row>
-    <row r="67" spans="1:6" s="17" customFormat="1" ht="58">
+    <row r="67" spans="1:6" s="17" customFormat="1" ht="60">
       <c r="A67" s="23" t="s">
         <v>2279</v>
       </c>
@@ -30087,7 +30106,7 @@
       </c>
       <c r="F67" s="23"/>
     </row>
-    <row r="68" spans="1:6" s="18" customFormat="1" ht="58">
+    <row r="68" spans="1:6" s="18" customFormat="1" ht="60">
       <c r="A68" s="24" t="s">
         <v>2279</v>
       </c>
@@ -31193,20 +31212,20 @@
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:L171"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" style="88" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.58203125" style="88" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.58203125" style="89" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.58203125" style="88" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.33203125" style="88" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.58203125" style="89" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.58203125" style="88" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.33203125" style="88" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.58203125" style="89" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.33203125" style="88" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="4.33203125" style="88" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.83203125" style="89" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.375" style="88" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.625" style="88" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.625" style="89" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.625" style="88" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.375" style="88" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.625" style="89" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.625" style="88" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.375" style="88" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.625" style="89" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.375" style="88" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.375" style="88" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.875" style="89" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="9" style="88"/>
   </cols>
   <sheetData>
@@ -32071,7 +32090,7 @@
         <v>3339</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="15">
+    <row r="25" spans="1:12">
       <c r="A25" s="88" t="s">
         <v>59</v>
       </c>
@@ -36583,7 +36602,7 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="9" style="47"/>
     <col min="2" max="2" width="45.75" style="47" customWidth="1"/>
@@ -36707,20 +36726,20 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:Q21"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.83203125" style="1"/>
+    <col min="1" max="1" width="7.875" style="1"/>
     <col min="2" max="2" width="6.5" style="1" customWidth="1"/>
-    <col min="3" max="4" width="7.83203125" style="1"/>
+    <col min="3" max="4" width="7.875" style="1"/>
     <col min="5" max="5" width="12.5" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" style="1" customWidth="1"/>
-    <col min="7" max="8" width="7.83203125" style="1"/>
+    <col min="6" max="6" width="8.875" style="1" customWidth="1"/>
+    <col min="7" max="8" width="7.875" style="1"/>
     <col min="9" max="9" width="10.25" style="1" customWidth="1"/>
     <col min="10" max="10" width="7.25" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.33203125" style="1" customWidth="1"/>
-    <col min="12" max="14" width="7.83203125" style="1"/>
-    <col min="15" max="15" width="9.33203125" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="7.83203125" style="1"/>
+    <col min="11" max="11" width="9.375" style="1" customWidth="1"/>
+    <col min="12" max="14" width="7.875" style="1"/>
+    <col min="15" max="15" width="9.375" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="7.875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -37296,22 +37315,22 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:M20"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.83203125" style="1"/>
-    <col min="2" max="2" width="6.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" style="1"/>
+    <col min="2" max="2" width="6.625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.75" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.08203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.75" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.83203125" style="1"/>
-    <col min="12" max="12" width="10.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.875" style="1"/>
+    <col min="12" max="12" width="10.625" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="7.83203125" style="1"/>
+    <col min="14" max="16384" width="7.875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -37752,20 +37771,20 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:L21"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.83203125" style="1"/>
-    <col min="2" max="2" width="15.08203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" style="1"/>
+    <col min="2" max="2" width="15.125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.5" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.75" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5.25" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.08203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.08203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="7.83203125" style="1"/>
+    <col min="10" max="10" width="16.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="7.875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -38121,7 +38140,7 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="9" style="46"/>
     <col min="2" max="2" width="15" style="46" bestFit="1" customWidth="1"/>
@@ -38235,7 +38254,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83C84FF1-A0EA-48F0-9BC3-5F8DC52E9A0A}">
   <dimension ref="A1:O210"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15" style="12" customWidth="1"/>
     <col min="2" max="5" width="15" style="5" customWidth="1"/>
@@ -38243,7 +38262,7 @@
     <col min="7" max="10" width="15" style="5" customWidth="1"/>
     <col min="11" max="11" width="15" style="12" customWidth="1"/>
     <col min="12" max="15" width="15" style="5" customWidth="1"/>
-    <col min="16" max="16384" width="7.83203125" style="5"/>
+    <col min="16" max="16384" width="7.875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="12" customFormat="1">
@@ -43854,15 +43873,15 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F6A446E-DC4A-45B3-A3E3-4049BF48BC30}">
   <dimension ref="A1:G503"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.58203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.375" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.5" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="7.83203125" style="5"/>
+    <col min="5" max="5" width="6.875" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.875" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="7.875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="12" customFormat="1">
@@ -54853,7 +54872,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="459" spans="1:7" ht="15.5">
+    <row r="459" spans="1:7">
       <c r="A459" t="s">
         <v>694</v>
       </c>

</xml_diff>

<commit_message>
67 junk to reforge unique, 49 junk to reforge set
</commit_message>
<xml_diff>
--- a/Diablo II.xlsx
+++ b/Diablo II.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yatyr\workspace\d2r-loot-filter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C91EBA1-4EC3-4CB0-AF7B-5034F85FDFFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF602AA2-8C9B-4CD7-AC96-C987DF72A4C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{4FA0E628-D5C1-45F8-838A-535ABF901563}"/>
   </bookViews>
@@ -11833,15 +11833,22 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Normal items + Rune01~06 -&gt; Add 1~6 sockets; Any item + Ort + Jewel -&gt; Larzuk Socket</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Enable Reforge Recipes</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Unique/Set item + Scroll of Identify -&gt; Salvage to Andariel Essence, 3x Andariel Essence -&gt; Mephisto Essence, 3x Mephisto Essence -&gt; Diablo Essence, 3x Diablo Essence -&gt; Baal Essence, Unique/Set item + Token of Absolution -&gt; Reforged unique/set item</t>
+    <t>Normal items + Rune01~06 -&gt; Add 1~6 sockets
+Any item + Ort + Jewel -&gt; Larzuk Socket</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Any Unique or set Item + Scroll of Identity -&gt; Salvage to Twisted Essence of Suffering
+3 Twisted Essence of Suffering -&gt; Charged Essense of Hatred
+3 Charged Essense of Hatred -&gt; Burning Essence of Terror
+3 Burning Essence of Terror -&gt; Festering Essence of Destruction
+Any Unique Item + Token of Absolution + Festering Essence of Destruction -&gt; Reforged Unique Item
+Any Set Item + Token of Absolution + Burning Essence of Terror -&gt; Reforged Set Item
+* Warning: Reforging uber charms and jewels results in rare charms and jewels</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -12224,7 +12231,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1">
       <alignment vertical="center"/>
@@ -12415,6 +12422,15 @@
     <xf numFmtId="49" fontId="35" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal 2" xfId="1" xr:uid="{53F17FA5-8A83-41A1-8800-C9AE149B41E5}"/>
@@ -12847,129 +12863,129 @@
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.875" style="88" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9" style="88"/>
-    <col min="3" max="3" width="72.25" style="88" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9" style="88"/>
+    <col min="1" max="1" width="21.875" style="91" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" style="91"/>
+    <col min="3" max="3" width="76.125" style="91" customWidth="1"/>
+    <col min="4" max="16384" width="9" style="91"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="86" t="s">
+      <c r="A1" s="90" t="s">
         <v>1692</v>
       </c>
-      <c r="B1" s="86" t="s">
+      <c r="B1" s="90" t="s">
         <v>1693</v>
       </c>
-      <c r="C1" s="86" t="s">
+      <c r="C1" s="90" t="s">
         <v>2753</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="88" t="s">
+      <c r="A2" s="91" t="s">
         <v>3269</v>
       </c>
-      <c r="B2" s="88" t="s">
+      <c r="B2" s="91" t="s">
         <v>2752</v>
       </c>
-      <c r="C2" s="88" t="s">
+      <c r="C2" s="91" t="s">
         <v>3270</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="88" t="s">
+      <c r="A3" s="91" t="s">
         <v>1697</v>
       </c>
-      <c r="B3" s="88" t="s">
+      <c r="B3" s="91" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="88" t="s">
+      <c r="C3" s="91" t="s">
         <v>3271</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="91" t="s">
         <v>1694</v>
       </c>
-      <c r="B4" s="88" t="s">
+      <c r="B4" s="91" t="s">
         <v>3356</v>
       </c>
-      <c r="C4" s="88" t="s">
+      <c r="C4" s="91" t="s">
         <v>3272</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="88" t="s">
+      <c r="A5" s="91" t="s">
         <v>1695</v>
       </c>
-      <c r="B5" s="88" t="s">
+      <c r="B5" s="91" t="s">
         <v>3357</v>
       </c>
-      <c r="C5" s="88" t="s">
+      <c r="C5" s="91" t="s">
         <v>3273</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="88" t="s">
+      <c r="A6" s="91" t="s">
         <v>1696</v>
       </c>
-      <c r="B6" s="88" t="s">
+      <c r="B6" s="91" t="s">
         <v>3358</v>
       </c>
-      <c r="C6" s="88" t="s">
+      <c r="C6" s="91" t="s">
         <v>3274</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="88" t="s">
+      <c r="A7" s="91" t="s">
         <v>3243</v>
       </c>
-      <c r="B7" s="88" t="s">
+      <c r="B7" s="91" t="s">
         <v>2754</v>
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="88" t="s">
+      <c r="A8" s="91" t="s">
         <v>3266</v>
       </c>
-      <c r="B8" s="88" t="s">
+      <c r="B8" s="91" t="s">
         <v>2752</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" s="88" t="s">
+      <c r="A9" s="91" t="s">
         <v>3267</v>
       </c>
-      <c r="B9" s="88">
+      <c r="B9" s="91">
         <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" s="88" t="s">
+      <c r="A10" s="91" t="s">
         <v>3268</v>
       </c>
-      <c r="B10" s="88">
+      <c r="B10" s="91">
         <v>200</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="88" t="s">
+    <row r="11" spans="1:3" ht="30">
+      <c r="A11" s="91" t="s">
         <v>3359</v>
       </c>
-      <c r="B11" s="88" t="s">
+      <c r="B11" s="91" t="s">
         <v>3360</v>
       </c>
-      <c r="C11" s="88" t="s">
+      <c r="C11" s="92" t="s">
+        <v>3362</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="105">
+      <c r="A12" s="91" t="s">
         <v>3361</v>
       </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" s="88" t="s">
-        <v>3362</v>
-      </c>
-      <c r="B12" s="88" t="s">
+      <c r="B12" s="91" t="s">
         <v>3360</v>
       </c>
-      <c r="C12" s="88" t="s">
+      <c r="C12" s="92" t="s">
         <v>3363</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add hope of cain
</commit_message>
<xml_diff>
--- a/Diablo II.xlsx
+++ b/Diablo II.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yatyr\workspace\d2r-loot-filter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nef\workspace\d2r-loot-filter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90E633AF-FBC8-4AB9-A873-7A47ABFE9F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD375934-993B-4ED5-8BB7-F65BAA0D1C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="8" xr2:uid="{4FA0E628-D5C1-45F8-838A-535ABF901563}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{4FA0E628-D5C1-45F8-838A-535ABF901563}"/>
   </bookViews>
   <sheets>
     <sheet name="Mod-Config" sheetId="6" r:id="rId1"/>
@@ -32,7 +32,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Area Level'!$A$1:$E$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Collection!$A$1:$O$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">Recipes!$A$1:$F$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">Recipes!$A$1:$F$126</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Rune Words'!$A$1:$G$105</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Set&amp;Unique'!$A$1:$L$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">Sockets!$A$1:$M$140</definedName>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6177" uniqueCount="3453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6180" uniqueCount="3455">
   <si>
     <t>Key</t>
   </si>
@@ -11680,10 +11680,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Enable Reforge Recipes</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Normal items + Rune01~06 -&gt; Add 1~6 sockets
 Any item + Ort + Jewel -&gt; Larzuk Socket</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -12132,6 +12128,34 @@
   </si>
   <si>
     <t>Lifibear</t>
+  </si>
+  <si>
+    <t>Enable Law of Kulle</t>
+  </si>
+  <si>
+    <t>Enable Hope of Cain</t>
+  </si>
+  <si>
+    <t>Rare Helm + 3 Festering Essence of Destruction + Northern Worldstone Shard -&gt; Upgraded to Unique Helm
+Rare Armor + 3 Festering Essence of Destruction + Southern Worldstone Shard -&gt; Upgraded to Unique Armor
+Rare Weapon + 3 Festering Essence of Destruction + Western Worldstone Shard -&gt; Upgraded to Unique Weapon
+Rare Shield + 3 Festering Essence of Destruction + Eastern Worldstone Shard -&gt; Upgraded to Unique Shield
+Rare Amulet + 3 Festering Essence of Destruction + Deep Worldstone Shard -&gt; Upgraded to Unique Amulet
+Rare Ring + 3 Festering Essence of Destruction + Deep Worldstone Shard -&gt; Upgraded to Unique Ring
+Rare Ring + 3 Festering Essence of Destruction + Western Worldstone Shard -&gt; Upgraded to Unique Ring
+Rare Gloves + 3 Festering Essence of Destruction + Eastern Worldstone Shard -&gt; Upgraded to Unique Gloves
+Rare Boots + 3 Festering Essence of Destruction + Southern Worldstone Shard -&gt; Upgraded to Unique Boots
+Rare Belt + 3 Festering Essence of Destruction + Northern Worldstone Shard -&gt; Upgraded to Unique Belt
+Rare Helm + 3 Burning Essence of Terror + Northern Worldstone Shard -&gt; Upgraded to Set Helm
+Rare Armor + 3 Burning Essence of Terror + Southern Worldstone Shard -&gt; Upgraded to Set Armor
+Rare Weapon + 3 Burning Essence of Terror + Western Worldstone Shard -&gt; Upgraded to Set Weapon
+Rare Shield + 3 Burning Essence of Terror + Eastern Worldstone Shard -&gt; Upgraded to Set Shield
+Rare Amulet + 3 Burning Essence of Terror + Deep Worldstone Shard -&gt; Upgraded to Set Amulet
+Rare Ring + 3 Burning Essence of Terror + Deep Worldstone Shard -&gt; Upgraded to Set Ring
+Rare Ring + 3 Burning Essence of Terror + Western Worldstone Shard -&gt; Upgraded to Set Ring
+Rare Gloves + 3 Burning Essence of Terror + Eastern Worldstone Shard -&gt; Upgraded to Set Gloves
+Rare Boots + 3 Burning Essence of Terror + Southern Worldstone Shard -&gt; Upgraded to Set Boots
+Rare Belt + 3 Burning Essence of Terror + Northern Worldstone Shard -&gt; Upgraded to Set Belt</t>
   </si>
 </sst>
 </file>
@@ -13205,12 +13229,12 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.83203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.25" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" style="6"/>
-    <col min="3" max="3" width="76.08203125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="86.875" style="6" customWidth="1"/>
     <col min="4" max="16384" width="9" style="6"/>
   </cols>
   <sheetData>
@@ -13312,7 +13336,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="29">
+    <row r="11" spans="1:3" ht="30">
       <c r="A11" s="6" t="s">
         <v>3318</v>
       </c>
@@ -13320,18 +13344,29 @@
         <v>3319</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>3321</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="101.5">
+        <v>3320</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="120">
       <c r="A12" s="6" t="s">
-        <v>3320</v>
+        <v>3452</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>3319</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>3322</v>
+        <v>3321</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="315">
+      <c r="A13" s="6" t="s">
+        <v>3453</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>2712</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>3454</v>
       </c>
     </row>
   </sheetData>
@@ -13346,14 +13381,14 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:F247"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="57.08203125" style="34" customWidth="1"/>
-    <col min="2" max="2" width="14.58203125" style="33" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="57.125" style="34" customWidth="1"/>
+    <col min="2" max="2" width="14.625" style="33" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.5" style="33" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" style="33" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.08203125" style="33" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.83203125" style="33" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.875" style="33" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.125" style="33" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.875" style="33" bestFit="1" customWidth="1"/>
     <col min="7" max="16384" width="9" style="33"/>
   </cols>
   <sheetData>
@@ -15021,7 +15056,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="95" spans="1:6" ht="48">
+    <row r="95" spans="1:6" ht="47.25">
       <c r="A95" s="46" t="s">
         <v>3049</v>
       </c>
@@ -17874,14 +17909,14 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:F34"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.5" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.58203125" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="58.33203125" style="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.625" style="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58.375" style="12" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="38.25" style="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="38.25" style="53" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.83203125" style="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.875" style="12" bestFit="1" customWidth="1"/>
     <col min="7" max="16384" width="9" style="12"/>
   </cols>
   <sheetData>
@@ -18577,14 +18612,14 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:G105"/>
-  <sheetFormatPr defaultColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.08203125" style="56" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.58203125" style="56" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.08203125" style="56" customWidth="1"/>
-    <col min="4" max="4" width="37.08203125" style="56" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.125" style="56" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.625" style="56" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.125" style="56" customWidth="1"/>
+    <col min="4" max="4" width="37.125" style="56" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="26.5" style="56" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="70.83203125" style="62" customWidth="1"/>
+    <col min="6" max="6" width="70.875" style="62" customWidth="1"/>
     <col min="7" max="7" width="34.75" style="53" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="8" style="12"/>
   </cols>
@@ -18612,7 +18647,7 @@
         <v>2635</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="58">
+    <row r="2" spans="1:7" ht="60">
       <c r="A2" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18635,7 +18670,7 @@
         <v>1849</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="87">
+    <row r="3" spans="1:7" ht="90">
       <c r="A3" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18658,7 +18693,7 @@
         <v>1853</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="101.5">
+    <row r="4" spans="1:7" ht="105">
       <c r="A4" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18681,7 +18716,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="101.5">
+    <row r="5" spans="1:7" ht="105">
       <c r="A5" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18704,7 +18739,7 @@
         <v>1862</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="87">
+    <row r="6" spans="1:7" ht="90">
       <c r="A6" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18727,7 +18762,7 @@
         <v>1866</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="87">
+    <row r="7" spans="1:7" ht="90">
       <c r="A7" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18750,7 +18785,7 @@
         <v>1870</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="87">
+    <row r="8" spans="1:7" ht="90">
       <c r="A8" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18773,7 +18808,7 @@
         <v>1875</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="87">
+    <row r="9" spans="1:7" ht="90">
       <c r="A9" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18796,7 +18831,7 @@
         <v>1880</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="58">
+    <row r="10" spans="1:7" ht="60">
       <c r="A10" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18819,7 +18854,7 @@
         <v>1884</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="87">
+    <row r="11" spans="1:7" ht="90">
       <c r="A11" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18842,7 +18877,7 @@
         <v>1888</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="87">
+    <row r="12" spans="1:7" ht="90">
       <c r="A12" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18865,7 +18900,7 @@
         <v>1893</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="101.5">
+    <row r="13" spans="1:7" ht="105">
       <c r="A13" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18888,7 +18923,7 @@
         <v>1898</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="87">
+    <row r="14" spans="1:7" ht="90">
       <c r="A14" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18911,7 +18946,7 @@
         <v>1902</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="87">
+    <row r="15" spans="1:7" ht="90">
       <c r="A15" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18934,7 +18969,7 @@
         <v>1906</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="87">
+    <row r="16" spans="1:7" ht="90">
       <c r="A16" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18957,7 +18992,7 @@
         <v>1910</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="101.5">
+    <row r="17" spans="1:7" ht="105">
       <c r="A17" s="56" t="s">
         <v>1651</v>
       </c>
@@ -18980,7 +19015,7 @@
         <v>1915</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="87">
+    <row r="18" spans="1:7" ht="90">
       <c r="A18" s="56" t="s">
         <v>1651</v>
       </c>
@@ -19003,7 +19038,7 @@
         <v>1919</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="87">
+    <row r="19" spans="1:7" ht="90">
       <c r="A19" s="56" t="s">
         <v>1651</v>
       </c>
@@ -19026,7 +19061,7 @@
         <v>2503</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="72.5">
+    <row r="20" spans="1:7" ht="75">
       <c r="A20" s="56" t="s">
         <v>1651</v>
       </c>
@@ -19049,7 +19084,7 @@
         <v>2505</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="58">
+    <row r="21" spans="1:7" ht="60">
       <c r="A21" s="56" t="s">
         <v>1651</v>
       </c>
@@ -19072,7 +19107,7 @@
         <v>2507</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="72.5">
+    <row r="22" spans="1:7" ht="75">
       <c r="A22" s="56" t="s">
         <v>1651</v>
       </c>
@@ -19095,7 +19130,7 @@
         <v>2509</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="43.5">
+    <row r="23" spans="1:7" ht="45">
       <c r="A23" s="56" t="s">
         <v>1651</v>
       </c>
@@ -19118,7 +19153,7 @@
         <v>2511</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="101.5">
+    <row r="24" spans="1:7" ht="105">
       <c r="A24" s="56" t="s">
         <v>1651</v>
       </c>
@@ -19141,7 +19176,7 @@
         <v>2513</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="87">
+    <row r="25" spans="1:7" ht="90">
       <c r="A25" s="56" t="s">
         <v>1651</v>
       </c>
@@ -19164,7 +19199,7 @@
         <v>2515</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="101.5">
+    <row r="26" spans="1:7" ht="105">
       <c r="A26" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19187,7 +19222,7 @@
         <v>2517</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="101.5">
+    <row r="27" spans="1:7" ht="105">
       <c r="A27" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19210,7 +19245,7 @@
         <v>2519</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="101.5">
+    <row r="28" spans="1:7" ht="105">
       <c r="A28" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19233,7 +19268,7 @@
         <v>2521</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="101.5">
+    <row r="29" spans="1:7" ht="105">
       <c r="A29" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19256,7 +19291,7 @@
         <v>2522</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="101.5">
+    <row r="30" spans="1:7" ht="105">
       <c r="A30" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19279,7 +19314,7 @@
         <v>2524</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="101.5">
+    <row r="31" spans="1:7" ht="105">
       <c r="A31" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19302,7 +19337,7 @@
         <v>2526</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="101.5">
+    <row r="32" spans="1:7" ht="105">
       <c r="A32" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19325,7 +19360,7 @@
         <v>2528</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="101.5">
+    <row r="33" spans="1:7" ht="105">
       <c r="A33" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19348,7 +19383,7 @@
         <v>2530</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="101.5">
+    <row r="34" spans="1:7" ht="105">
       <c r="A34" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19371,7 +19406,7 @@
         <v>2531</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="101.5">
+    <row r="35" spans="1:7" ht="105">
       <c r="A35" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19394,7 +19429,7 @@
         <v>2533</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="116">
+    <row r="36" spans="1:7" ht="120">
       <c r="A36" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19417,7 +19452,7 @@
         <v>2534</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="101.5">
+    <row r="37" spans="1:7" ht="105">
       <c r="A37" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19440,7 +19475,7 @@
         <v>2535</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="101.5">
+    <row r="38" spans="1:7" ht="105">
       <c r="A38" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19463,7 +19498,7 @@
         <v>2536</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="116">
+    <row r="39" spans="1:7" ht="120">
       <c r="A39" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19486,7 +19521,7 @@
         <v>2537</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="101.5">
+    <row r="40" spans="1:7" ht="105">
       <c r="A40" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19509,7 +19544,7 @@
         <v>2539</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="101.5">
+    <row r="41" spans="1:7" ht="105">
       <c r="A41" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19532,7 +19567,7 @@
         <v>2541</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="101.5">
+    <row r="42" spans="1:7" ht="105">
       <c r="A42" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19555,7 +19590,7 @@
         <v>2543</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="101.5">
+    <row r="43" spans="1:7" ht="105">
       <c r="A43" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19578,7 +19613,7 @@
         <v>2544</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="101.5">
+    <row r="44" spans="1:7" ht="105">
       <c r="A44" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19601,7 +19636,7 @@
         <v>2546</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="101.5">
+    <row r="45" spans="1:7" ht="105">
       <c r="A45" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19624,7 +19659,7 @@
         <v>2548</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="101.5">
+    <row r="46" spans="1:7" ht="105">
       <c r="A46" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19647,7 +19682,7 @@
         <v>2550</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="101.5">
+    <row r="47" spans="1:7" ht="105">
       <c r="A47" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19670,7 +19705,7 @@
         <v>2552</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="101.5">
+    <row r="48" spans="1:7" ht="105">
       <c r="A48" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19693,7 +19728,7 @@
         <v>2554</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="101.5">
+    <row r="49" spans="1:7" ht="105">
       <c r="A49" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19716,7 +19751,7 @@
         <v>2556</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="87">
+    <row r="50" spans="1:7" ht="90">
       <c r="A50" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19739,7 +19774,7 @@
         <v>2558</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="101.5">
+    <row r="51" spans="1:7" ht="105">
       <c r="A51" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19762,7 +19797,7 @@
         <v>2560</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="101.5">
+    <row r="52" spans="1:7" ht="105">
       <c r="A52" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19785,7 +19820,7 @@
         <v>2561</v>
       </c>
     </row>
-    <row r="53" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="53" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A53" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19808,7 +19843,7 @@
         <v>2562</v>
       </c>
     </row>
-    <row r="54" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="54" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A54" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19831,7 +19866,7 @@
         <v>2564</v>
       </c>
     </row>
-    <row r="55" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="55" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A55" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19854,7 +19889,7 @@
         <v>2565</v>
       </c>
     </row>
-    <row r="56" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="56" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A56" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19877,7 +19912,7 @@
         <v>2567</v>
       </c>
     </row>
-    <row r="57" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="57" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A57" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19900,7 +19935,7 @@
         <v>2568</v>
       </c>
     </row>
-    <row r="58" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="58" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A58" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19923,7 +19958,7 @@
         <v>2570</v>
       </c>
     </row>
-    <row r="59" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="59" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A59" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19946,7 +19981,7 @@
         <v>2572</v>
       </c>
     </row>
-    <row r="60" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="60" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A60" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19969,7 +20004,7 @@
         <v>2574</v>
       </c>
     </row>
-    <row r="61" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="61" spans="1:7" s="53" customFormat="1" ht="120">
       <c r="A61" s="56" t="s">
         <v>1933</v>
       </c>
@@ -19992,7 +20027,7 @@
         <v>2575</v>
       </c>
     </row>
-    <row r="62" spans="1:7" s="53" customFormat="1" ht="130.5">
+    <row r="62" spans="1:7" s="53" customFormat="1" ht="135">
       <c r="A62" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20015,7 +20050,7 @@
         <v>2576</v>
       </c>
     </row>
-    <row r="63" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="63" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A63" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20038,7 +20073,7 @@
         <v>2578</v>
       </c>
     </row>
-    <row r="64" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="64" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A64" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20061,7 +20096,7 @@
         <v>2580</v>
       </c>
     </row>
-    <row r="65" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="65" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A65" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20084,7 +20119,7 @@
         <v>2582</v>
       </c>
     </row>
-    <row r="66" spans="1:7" s="53" customFormat="1" ht="116">
+    <row r="66" spans="1:7" s="53" customFormat="1" ht="120">
       <c r="A66" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20107,7 +20142,7 @@
         <v>2584</v>
       </c>
     </row>
-    <row r="67" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="67" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A67" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20130,7 +20165,7 @@
         <v>2585</v>
       </c>
     </row>
-    <row r="68" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="68" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A68" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20153,7 +20188,7 @@
         <v>2587</v>
       </c>
     </row>
-    <row r="69" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="69" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A69" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20176,7 +20211,7 @@
         <v>2589</v>
       </c>
     </row>
-    <row r="70" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="70" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A70" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20199,7 +20234,7 @@
         <v>2591</v>
       </c>
     </row>
-    <row r="71" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="71" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A71" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20222,7 +20257,7 @@
         <v>2592</v>
       </c>
     </row>
-    <row r="72" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="72" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A72" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20245,7 +20280,7 @@
         <v>2595</v>
       </c>
     </row>
-    <row r="73" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="73" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A73" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20268,7 +20303,7 @@
         <v>2597</v>
       </c>
     </row>
-    <row r="74" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="74" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A74" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20291,7 +20326,7 @@
         <v>2599</v>
       </c>
     </row>
-    <row r="75" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="75" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A75" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20314,7 +20349,7 @@
         <v>2601</v>
       </c>
     </row>
-    <row r="76" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="76" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A76" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20337,7 +20372,7 @@
         <v>2602</v>
       </c>
     </row>
-    <row r="77" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="77" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A77" s="56" t="s">
         <v>1933</v>
       </c>
@@ -20360,7 +20395,7 @@
         <v>2604</v>
       </c>
     </row>
-    <row r="78" spans="1:7" s="53" customFormat="1" ht="58">
+    <row r="78" spans="1:7" s="53" customFormat="1" ht="60">
       <c r="A78" s="56" t="s">
         <v>2023</v>
       </c>
@@ -20383,7 +20418,7 @@
         <v>2606</v>
       </c>
     </row>
-    <row r="79" spans="1:7" s="53" customFormat="1" ht="58">
+    <row r="79" spans="1:7" s="53" customFormat="1" ht="60">
       <c r="A79" s="56" t="s">
         <v>2023</v>
       </c>
@@ -20406,7 +20441,7 @@
         <v>2608</v>
       </c>
     </row>
-    <row r="80" spans="1:7" s="53" customFormat="1" ht="58">
+    <row r="80" spans="1:7" s="53" customFormat="1" ht="60">
       <c r="A80" s="56" t="s">
         <v>2023</v>
       </c>
@@ -20429,7 +20464,7 @@
         <v>2610</v>
       </c>
     </row>
-    <row r="81" spans="1:7" s="53" customFormat="1" ht="58">
+    <row r="81" spans="1:7" s="53" customFormat="1" ht="60">
       <c r="A81" s="56" t="s">
         <v>2023</v>
       </c>
@@ -20452,7 +20487,7 @@
         <v>2612</v>
       </c>
     </row>
-    <row r="82" spans="1:7" s="53" customFormat="1" ht="58">
+    <row r="82" spans="1:7" s="53" customFormat="1" ht="60">
       <c r="A82" s="56" t="s">
         <v>2023</v>
       </c>
@@ -20475,7 +20510,7 @@
         <v>2614</v>
       </c>
     </row>
-    <row r="83" spans="1:7" s="53" customFormat="1" ht="58">
+    <row r="83" spans="1:7" s="53" customFormat="1" ht="60">
       <c r="A83" s="56" t="s">
         <v>2023</v>
       </c>
@@ -20498,7 +20533,7 @@
         <v>2616</v>
       </c>
     </row>
-    <row r="84" spans="1:7" s="53" customFormat="1" ht="58">
+    <row r="84" spans="1:7" s="53" customFormat="1" ht="60">
       <c r="A84" s="56" t="s">
         <v>2023</v>
       </c>
@@ -20521,7 +20556,7 @@
         <v>2618</v>
       </c>
     </row>
-    <row r="85" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="85" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A85" s="56" t="s">
         <v>2038</v>
       </c>
@@ -20544,7 +20579,7 @@
         <v>2620</v>
       </c>
     </row>
-    <row r="86" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="86" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A86" s="56" t="s">
         <v>2038</v>
       </c>
@@ -20567,7 +20602,7 @@
         <v>2622</v>
       </c>
     </row>
-    <row r="87" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="87" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A87" s="56" t="s">
         <v>2038</v>
       </c>
@@ -20590,7 +20625,7 @@
         <v>2624</v>
       </c>
     </row>
-    <row r="88" spans="1:7" s="53" customFormat="1" ht="87">
+    <row r="88" spans="1:7" s="53" customFormat="1" ht="90">
       <c r="A88" s="56" t="s">
         <v>2038</v>
       </c>
@@ -20613,7 +20648,7 @@
         <v>2626</v>
       </c>
     </row>
-    <row r="89" spans="1:7" s="53" customFormat="1" ht="101.5">
+    <row r="89" spans="1:7" s="53" customFormat="1" ht="105">
       <c r="A89" s="56" t="s">
         <v>2038</v>
       </c>
@@ -20636,7 +20671,7 @@
         <v>2628</v>
       </c>
     </row>
-    <row r="90" spans="1:7" s="53" customFormat="1" ht="87">
+    <row r="90" spans="1:7" s="53" customFormat="1" ht="90">
       <c r="A90" s="56" t="s">
         <v>2038</v>
       </c>
@@ -20659,7 +20694,7 @@
         <v>2631</v>
       </c>
     </row>
-    <row r="91" spans="1:7" s="53" customFormat="1" ht="87">
+    <row r="91" spans="1:7" s="53" customFormat="1" ht="90">
       <c r="A91" s="56" t="s">
         <v>2038</v>
       </c>
@@ -20682,7 +20717,7 @@
         <v>2633</v>
       </c>
     </row>
-    <row r="92" spans="1:7" ht="72.5">
+    <row r="92" spans="1:7" ht="75">
       <c r="A92" s="56" t="s">
         <v>2638</v>
       </c>
@@ -20705,7 +20740,7 @@
         <v>2641</v>
       </c>
     </row>
-    <row r="93" spans="1:7" ht="72.5">
+    <row r="93" spans="1:7" ht="75">
       <c r="A93" s="56" t="s">
         <v>2638</v>
       </c>
@@ -20728,7 +20763,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="94" spans="1:7" ht="72.5">
+    <row r="94" spans="1:7" ht="75">
       <c r="A94" s="56" t="s">
         <v>2638</v>
       </c>
@@ -20751,7 +20786,7 @@
         <v>2649</v>
       </c>
     </row>
-    <row r="95" spans="1:7" ht="58">
+    <row r="95" spans="1:7" ht="60">
       <c r="A95" s="56" t="s">
         <v>2638</v>
       </c>
@@ -20774,7 +20809,7 @@
         <v>2651</v>
       </c>
     </row>
-    <row r="96" spans="1:7" ht="116">
+    <row r="96" spans="1:7" ht="120">
       <c r="A96" s="56" t="s">
         <v>2638</v>
       </c>
@@ -20797,7 +20832,7 @@
         <v>2655</v>
       </c>
     </row>
-    <row r="97" spans="1:7" ht="145">
+    <row r="97" spans="1:7" ht="150">
       <c r="A97" s="56" t="s">
         <v>2638</v>
       </c>
@@ -20820,7 +20855,7 @@
         <v>2659</v>
       </c>
     </row>
-    <row r="98" spans="1:7" ht="72.5">
+    <row r="98" spans="1:7" ht="75">
       <c r="A98" s="56" t="s">
         <v>2638</v>
       </c>
@@ -20843,7 +20878,7 @@
         <v>2663</v>
       </c>
     </row>
-    <row r="99" spans="1:7" ht="58">
+    <row r="99" spans="1:7" ht="60">
       <c r="A99" s="56" t="s">
         <v>2638</v>
       </c>
@@ -20866,7 +20901,7 @@
         <v>2667</v>
       </c>
     </row>
-    <row r="100" spans="1:7" ht="58">
+    <row r="100" spans="1:7" ht="60">
       <c r="A100" s="56" t="s">
         <v>2638</v>
       </c>
@@ -20889,12 +20924,12 @@
         <v>2671</v>
       </c>
     </row>
-    <row r="101" spans="1:7" ht="58">
+    <row r="101" spans="1:7" ht="60">
       <c r="A101" s="56" t="s">
         <v>3203</v>
       </c>
       <c r="B101" s="57" t="s">
-        <v>3342</v>
+        <v>3341</v>
       </c>
       <c r="C101" s="56">
         <v>3</v>
@@ -20912,7 +20947,7 @@
         <v>3205</v>
       </c>
     </row>
-    <row r="102" spans="1:7" ht="87">
+    <row r="102" spans="1:7" ht="90">
       <c r="A102" s="56" t="s">
         <v>3203</v>
       </c>
@@ -20935,7 +20970,7 @@
         <v>3210</v>
       </c>
     </row>
-    <row r="103" spans="1:7" ht="87">
+    <row r="103" spans="1:7" ht="90">
       <c r="A103" s="56" t="s">
         <v>3203</v>
       </c>
@@ -20958,7 +20993,7 @@
         <v>3214</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="101.5">
+    <row r="104" spans="1:7" ht="105">
       <c r="A104" s="56" t="s">
         <v>3203</v>
       </c>
@@ -20981,7 +21016,7 @@
         <v>3219</v>
       </c>
     </row>
-    <row r="105" spans="1:7" ht="101.5">
+    <row r="105" spans="1:7" ht="105">
       <c r="A105" s="56" t="s">
         <v>3203</v>
       </c>
@@ -21018,16 +21053,16 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:M140"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" style="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.75" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="3.33203125" style="12" customWidth="1"/>
+    <col min="3" max="5" width="3.375" style="12" customWidth="1"/>
     <col min="6" max="6" width="16" style="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="3.58203125" style="12" customWidth="1"/>
-    <col min="10" max="10" width="16.33203125" style="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="3.33203125" style="12" customWidth="1"/>
-    <col min="14" max="16384" width="7.83203125" style="12"/>
+    <col min="7" max="9" width="3.625" style="12" customWidth="1"/>
+    <col min="10" max="10" width="16.375" style="12" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="3.375" style="12" customWidth="1"/>
+    <col min="14" max="16384" width="7.875" style="12"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -26801,12 +26836,12 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:F120"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.25" style="64" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="12.58203125" style="56" customWidth="1"/>
+    <col min="2" max="4" width="12.625" style="56" customWidth="1"/>
     <col min="5" max="5" width="35.75" style="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="7.83203125" style="12"/>
+    <col min="6" max="16384" width="7.875" style="12"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -29223,14 +29258,14 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:F126"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="7.83203125" style="75"/>
+    <col min="1" max="2" width="7.875" style="75"/>
     <col min="3" max="3" width="16.5" style="75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="40.33203125" style="76" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="40.375" style="76" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="60.75" style="76" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" style="75" customWidth="1"/>
-    <col min="7" max="16384" width="7.83203125" style="75"/>
+    <col min="6" max="6" width="45.875" style="75" customWidth="1"/>
+    <col min="7" max="16384" width="7.875" style="75"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="65" customFormat="1">
@@ -29799,7 +29834,7 @@
         <v>2313</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="29">
+    <row r="31" spans="1:6" ht="30">
       <c r="A31" s="73" t="s">
         <v>2239</v>
       </c>
@@ -29837,7 +29872,7 @@
       </c>
       <c r="F32" s="77"/>
     </row>
-    <row r="33" spans="1:6" ht="58">
+    <row r="33" spans="1:6" ht="60">
       <c r="A33" s="79" t="s">
         <v>2239</v>
       </c>
@@ -29855,7 +29890,7 @@
       </c>
       <c r="F33" s="79"/>
     </row>
-    <row r="34" spans="1:6" s="83" customFormat="1" ht="58">
+    <row r="34" spans="1:6" s="83" customFormat="1" ht="60">
       <c r="A34" s="81" t="s">
         <v>2239</v>
       </c>
@@ -29873,7 +29908,7 @@
       </c>
       <c r="F34" s="81"/>
     </row>
-    <row r="35" spans="1:6" s="84" customFormat="1" ht="58">
+    <row r="35" spans="1:6" s="84" customFormat="1" ht="60">
       <c r="A35" s="79" t="s">
         <v>2239</v>
       </c>
@@ -29891,7 +29926,7 @@
       </c>
       <c r="F35" s="79"/>
     </row>
-    <row r="36" spans="1:6" s="83" customFormat="1" ht="58">
+    <row r="36" spans="1:6" s="83" customFormat="1" ht="60">
       <c r="A36" s="81" t="s">
         <v>2239</v>
       </c>
@@ -29909,7 +29944,7 @@
       </c>
       <c r="F36" s="81"/>
     </row>
-    <row r="37" spans="1:6" s="84" customFormat="1" ht="58">
+    <row r="37" spans="1:6" s="84" customFormat="1" ht="60">
       <c r="A37" s="79" t="s">
         <v>2239</v>
       </c>
@@ -29927,7 +29962,7 @@
       </c>
       <c r="F37" s="79"/>
     </row>
-    <row r="38" spans="1:6" s="85" customFormat="1" ht="58">
+    <row r="38" spans="1:6" s="85" customFormat="1" ht="60">
       <c r="A38" s="81" t="s">
         <v>2239</v>
       </c>
@@ -29945,7 +29980,7 @@
       </c>
       <c r="F38" s="81"/>
     </row>
-    <row r="39" spans="1:6" s="71" customFormat="1" ht="58">
+    <row r="39" spans="1:6" s="71" customFormat="1" ht="60">
       <c r="A39" s="79" t="s">
         <v>2239</v>
       </c>
@@ -29963,7 +29998,7 @@
       </c>
       <c r="F39" s="79"/>
     </row>
-    <row r="40" spans="1:6" s="85" customFormat="1" ht="58">
+    <row r="40" spans="1:6" s="85" customFormat="1" ht="60">
       <c r="A40" s="81" t="s">
         <v>2239</v>
       </c>
@@ -29981,7 +30016,7 @@
       </c>
       <c r="F40" s="81"/>
     </row>
-    <row r="41" spans="1:6" s="71" customFormat="1" ht="58">
+    <row r="41" spans="1:6" s="71" customFormat="1" ht="60">
       <c r="A41" s="79" t="s">
         <v>2239</v>
       </c>
@@ -29999,7 +30034,7 @@
       </c>
       <c r="F41" s="79"/>
     </row>
-    <row r="42" spans="1:6" s="77" customFormat="1" ht="58">
+    <row r="42" spans="1:6" s="77" customFormat="1" ht="60">
       <c r="A42" s="81" t="s">
         <v>2239</v>
       </c>
@@ -30017,7 +30052,7 @@
       </c>
       <c r="F42" s="81"/>
     </row>
-    <row r="43" spans="1:6" s="77" customFormat="1" ht="58">
+    <row r="43" spans="1:6" s="77" customFormat="1" ht="60">
       <c r="A43" s="79" t="s">
         <v>2239</v>
       </c>
@@ -30035,7 +30070,7 @@
       </c>
       <c r="F43" s="79"/>
     </row>
-    <row r="44" spans="1:6" s="77" customFormat="1" ht="58">
+    <row r="44" spans="1:6" s="77" customFormat="1" ht="60">
       <c r="A44" s="81" t="s">
         <v>2239</v>
       </c>
@@ -30053,7 +30088,7 @@
       </c>
       <c r="F44" s="81"/>
     </row>
-    <row r="45" spans="1:6" s="77" customFormat="1" ht="58">
+    <row r="45" spans="1:6" s="77" customFormat="1" ht="60">
       <c r="A45" s="79" t="s">
         <v>2239</v>
       </c>
@@ -30071,7 +30106,7 @@
       </c>
       <c r="F45" s="79"/>
     </row>
-    <row r="46" spans="1:6" s="77" customFormat="1" ht="58">
+    <row r="46" spans="1:6" s="77" customFormat="1" ht="60">
       <c r="A46" s="81" t="s">
         <v>2239</v>
       </c>
@@ -30089,7 +30124,7 @@
       </c>
       <c r="F46" s="81"/>
     </row>
-    <row r="47" spans="1:6" s="77" customFormat="1" ht="58">
+    <row r="47" spans="1:6" s="77" customFormat="1" ht="60">
       <c r="A47" s="79" t="s">
         <v>2239</v>
       </c>
@@ -30107,7 +30142,7 @@
       </c>
       <c r="F47" s="79"/>
     </row>
-    <row r="48" spans="1:6" s="69" customFormat="1" ht="58">
+    <row r="48" spans="1:6" s="69" customFormat="1" ht="60">
       <c r="A48" s="81" t="s">
         <v>2239</v>
       </c>
@@ -30125,7 +30160,7 @@
       </c>
       <c r="F48" s="81"/>
     </row>
-    <row r="49" spans="1:6" s="67" customFormat="1" ht="58">
+    <row r="49" spans="1:6" s="67" customFormat="1" ht="60">
       <c r="A49" s="79" t="s">
         <v>2239</v>
       </c>
@@ -30143,7 +30178,7 @@
       </c>
       <c r="F49" s="79"/>
     </row>
-    <row r="50" spans="1:6" s="69" customFormat="1" ht="58">
+    <row r="50" spans="1:6" s="69" customFormat="1" ht="60">
       <c r="A50" s="81" t="s">
         <v>2239</v>
       </c>
@@ -30161,7 +30196,7 @@
       </c>
       <c r="F50" s="81"/>
     </row>
-    <row r="51" spans="1:6" s="67" customFormat="1" ht="58">
+    <row r="51" spans="1:6" s="67" customFormat="1" ht="60">
       <c r="A51" s="79" t="s">
         <v>2239</v>
       </c>
@@ -30179,7 +30214,7 @@
       </c>
       <c r="F51" s="79"/>
     </row>
-    <row r="52" spans="1:6" s="69" customFormat="1" ht="58">
+    <row r="52" spans="1:6" s="69" customFormat="1" ht="60">
       <c r="A52" s="81" t="s">
         <v>2239</v>
       </c>
@@ -30197,7 +30232,7 @@
       </c>
       <c r="F52" s="81"/>
     </row>
-    <row r="53" spans="1:6" s="67" customFormat="1" ht="58">
+    <row r="53" spans="1:6" s="67" customFormat="1" ht="60">
       <c r="A53" s="79" t="s">
         <v>2239</v>
       </c>
@@ -30215,7 +30250,7 @@
       </c>
       <c r="F53" s="79"/>
     </row>
-    <row r="54" spans="1:6" s="69" customFormat="1" ht="58">
+    <row r="54" spans="1:6" s="69" customFormat="1" ht="60">
       <c r="A54" s="81" t="s">
         <v>2239</v>
       </c>
@@ -30233,7 +30268,7 @@
       </c>
       <c r="F54" s="81"/>
     </row>
-    <row r="55" spans="1:6" s="67" customFormat="1" ht="58">
+    <row r="55" spans="1:6" s="67" customFormat="1" ht="60">
       <c r="A55" s="79" t="s">
         <v>2239</v>
       </c>
@@ -30251,7 +30286,7 @@
       </c>
       <c r="F55" s="79"/>
     </row>
-    <row r="56" spans="1:6" s="69" customFormat="1" ht="58">
+    <row r="56" spans="1:6" s="69" customFormat="1" ht="60">
       <c r="A56" s="81" t="s">
         <v>2239</v>
       </c>
@@ -30269,7 +30304,7 @@
       </c>
       <c r="F56" s="81"/>
     </row>
-    <row r="57" spans="1:6" s="67" customFormat="1" ht="58">
+    <row r="57" spans="1:6" s="67" customFormat="1" ht="60">
       <c r="A57" s="79" t="s">
         <v>2239</v>
       </c>
@@ -30287,7 +30322,7 @@
       </c>
       <c r="F57" s="79"/>
     </row>
-    <row r="58" spans="1:6" s="69" customFormat="1" ht="58">
+    <row r="58" spans="1:6" s="69" customFormat="1" ht="60">
       <c r="A58" s="81" t="s">
         <v>2239</v>
       </c>
@@ -30305,7 +30340,7 @@
       </c>
       <c r="F58" s="81"/>
     </row>
-    <row r="59" spans="1:6" s="67" customFormat="1" ht="58">
+    <row r="59" spans="1:6" s="67" customFormat="1" ht="60">
       <c r="A59" s="79" t="s">
         <v>2239</v>
       </c>
@@ -30323,7 +30358,7 @@
       </c>
       <c r="F59" s="79"/>
     </row>
-    <row r="60" spans="1:6" s="69" customFormat="1" ht="58">
+    <row r="60" spans="1:6" s="69" customFormat="1" ht="60">
       <c r="A60" s="81" t="s">
         <v>2239</v>
       </c>
@@ -30341,7 +30376,7 @@
       </c>
       <c r="F60" s="81"/>
     </row>
-    <row r="61" spans="1:6" s="67" customFormat="1" ht="58">
+    <row r="61" spans="1:6" s="67" customFormat="1" ht="60">
       <c r="A61" s="79" t="s">
         <v>2239</v>
       </c>
@@ -30359,7 +30394,7 @@
       </c>
       <c r="F61" s="79"/>
     </row>
-    <row r="62" spans="1:6" s="69" customFormat="1" ht="58">
+    <row r="62" spans="1:6" s="69" customFormat="1" ht="60">
       <c r="A62" s="81" t="s">
         <v>2239</v>
       </c>
@@ -30377,7 +30412,7 @@
       </c>
       <c r="F62" s="81"/>
     </row>
-    <row r="63" spans="1:6" s="67" customFormat="1" ht="58">
+    <row r="63" spans="1:6" s="67" customFormat="1" ht="60">
       <c r="A63" s="79" t="s">
         <v>2239</v>
       </c>
@@ -30395,7 +30430,7 @@
       </c>
       <c r="F63" s="79"/>
     </row>
-    <row r="64" spans="1:6" s="69" customFormat="1" ht="58">
+    <row r="64" spans="1:6" s="69" customFormat="1" ht="60">
       <c r="A64" s="81" t="s">
         <v>2239</v>
       </c>
@@ -30413,7 +30448,7 @@
       </c>
       <c r="F64" s="81"/>
     </row>
-    <row r="65" spans="1:6" s="67" customFormat="1" ht="58">
+    <row r="65" spans="1:6" s="67" customFormat="1" ht="60">
       <c r="A65" s="79" t="s">
         <v>2239</v>
       </c>
@@ -30431,7 +30466,7 @@
       </c>
       <c r="F65" s="79"/>
     </row>
-    <row r="66" spans="1:6" s="69" customFormat="1" ht="58">
+    <row r="66" spans="1:6" s="69" customFormat="1" ht="60">
       <c r="A66" s="81" t="s">
         <v>2239</v>
       </c>
@@ -30449,7 +30484,7 @@
       </c>
       <c r="F66" s="81"/>
     </row>
-    <row r="67" spans="1:6" s="67" customFormat="1" ht="58">
+    <row r="67" spans="1:6" s="67" customFormat="1" ht="60">
       <c r="A67" s="79" t="s">
         <v>2239</v>
       </c>
@@ -30467,7 +30502,7 @@
       </c>
       <c r="F67" s="79"/>
     </row>
-    <row r="68" spans="1:6" s="69" customFormat="1" ht="58">
+    <row r="68" spans="1:6" s="69" customFormat="1" ht="60">
       <c r="A68" s="81" t="s">
         <v>2239</v>
       </c>
@@ -31556,7 +31591,7 @@
       <c r="F126" s="67"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F119" xr:uid="{9BDF046B-9994-41EA-929E-00B1B3972364}"/>
+  <autoFilter ref="A1:F126" xr:uid="{9BDF046B-9994-41EA-929E-00B1B3972364}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -31569,20 +31604,20 @@
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:L171"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.58203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.58203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.58203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.58203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.58203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.58203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="4.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.375" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.375" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.375" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.625" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.375" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.375" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.875" style="4" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
@@ -32447,7 +32482,7 @@
         <v>3298</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="15">
+    <row r="25" spans="1:12">
       <c r="A25" s="3" t="s">
         <v>59</v>
       </c>
@@ -36959,7 +36994,7 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9" style="3"/>
     <col min="2" max="2" width="45.75" style="3" customWidth="1"/>
@@ -37083,20 +37118,20 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:Q21"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.83203125" style="32"/>
+    <col min="1" max="1" width="7.875" style="32"/>
     <col min="2" max="2" width="6.5" style="32" customWidth="1"/>
-    <col min="3" max="4" width="7.83203125" style="32"/>
+    <col min="3" max="4" width="7.875" style="32"/>
     <col min="5" max="5" width="12.5" style="32" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" style="32" customWidth="1"/>
-    <col min="7" max="8" width="7.83203125" style="32"/>
+    <col min="6" max="6" width="8.875" style="32" customWidth="1"/>
+    <col min="7" max="8" width="7.875" style="32"/>
     <col min="9" max="9" width="10.25" style="32" customWidth="1"/>
     <col min="10" max="10" width="7.25" style="32" customWidth="1"/>
-    <col min="11" max="11" width="9.33203125" style="32" customWidth="1"/>
-    <col min="12" max="14" width="7.83203125" style="32"/>
-    <col min="15" max="15" width="9.33203125" style="32" customWidth="1"/>
-    <col min="16" max="16384" width="7.83203125" style="32"/>
+    <col min="11" max="11" width="9.375" style="32" customWidth="1"/>
+    <col min="12" max="14" width="7.875" style="32"/>
+    <col min="15" max="15" width="9.375" style="32" customWidth="1"/>
+    <col min="16" max="16384" width="7.875" style="32"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -37672,22 +37707,22 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:M20"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.83203125" style="32"/>
-    <col min="2" max="2" width="6.58203125" style="32" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" style="32"/>
+    <col min="2" max="2" width="6.625" style="32" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.75" style="32" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8" style="32" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.25" style="32" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.08203125" style="32" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.125" style="32" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8" style="32" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.75" style="32" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.25" style="32" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.33203125" style="32" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.83203125" style="32"/>
-    <col min="12" max="12" width="10.58203125" style="32" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.375" style="32" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.875" style="32"/>
+    <col min="12" max="12" width="10.625" style="32" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8" style="32" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="7.83203125" style="32"/>
+    <col min="14" max="16384" width="7.875" style="32"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -38128,20 +38163,20 @@
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:L21"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.83203125" style="32"/>
-    <col min="2" max="2" width="15.08203125" style="32" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" style="32"/>
+    <col min="2" max="2" width="15.125" style="32" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.5" style="32" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.75" style="32" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8" style="32" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5.25" style="32" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8" style="32" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.08203125" style="32" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.125" style="32" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.75" style="32" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.33203125" style="32" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.08203125" style="32" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="7.83203125" style="32"/>
+    <col min="10" max="10" width="16.375" style="32" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.125" style="32" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="7.875" style="32"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -38497,7 +38532,7 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="9" style="33"/>
     <col min="2" max="2" width="15" style="33" bestFit="1" customWidth="1"/>
@@ -38611,7 +38646,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83C84FF1-A0EA-48F0-9BC3-5F8DC52E9A0A}">
   <dimension ref="A1:O232"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15" style="9" customWidth="1"/>
     <col min="2" max="5" width="15" style="12" customWidth="1"/>
@@ -38619,7 +38654,7 @@
     <col min="7" max="10" width="15" style="12" customWidth="1"/>
     <col min="11" max="11" width="15" style="9" customWidth="1"/>
     <col min="12" max="15" width="15" style="12" customWidth="1"/>
-    <col min="16" max="16384" width="7.83203125" style="12"/>
+    <col min="16" max="16384" width="7.875" style="12"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="9" customFormat="1">
@@ -38851,7 +38886,7 @@
         <v>1380</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>3323</v>
+        <v>3322</v>
       </c>
       <c r="I7" s="11" t="s">
         <v>1534</v>
@@ -38865,7 +38900,7 @@
       </c>
       <c r="M7" s="10"/>
       <c r="N7" s="11" t="s">
-        <v>3338</v>
+        <v>3337</v>
       </c>
       <c r="O7" s="10"/>
     </row>
@@ -39079,7 +39114,7 @@
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="11" t="s">
-        <v>3337</v>
+        <v>3336</v>
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="8" t="s">
@@ -39270,7 +39305,7 @@
       </c>
       <c r="H21" s="10"/>
       <c r="I21" s="11" t="s">
-        <v>3339</v>
+        <v>3338</v>
       </c>
       <c r="J21" s="10"/>
       <c r="K21" s="8" t="s">
@@ -39514,7 +39549,7 @@
       </c>
       <c r="H29" s="10"/>
       <c r="I29" s="11" t="s">
-        <v>3340</v>
+        <v>3339</v>
       </c>
       <c r="J29" s="10"/>
       <c r="K29" s="8" t="s">
@@ -39800,11 +39835,11 @@
         <v>1142</v>
       </c>
       <c r="L38" s="11" t="s">
-        <v>3324</v>
+        <v>3323</v>
       </c>
       <c r="M38" s="10"/>
       <c r="N38" s="10" t="s">
-        <v>3355</v>
+        <v>3354</v>
       </c>
       <c r="O38" s="10"/>
     </row>
@@ -39901,7 +39936,7 @@
         <v>753</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>3335</v>
+        <v>3334</v>
       </c>
       <c r="F42" s="8" t="s">
         <v>267</v>
@@ -39990,7 +40025,7 @@
         <v>1152</v>
       </c>
       <c r="L44" s="11" t="s">
-        <v>3325</v>
+        <v>3324</v>
       </c>
       <c r="M44" s="10"/>
       <c r="N44" s="11" t="s">
@@ -40583,7 +40618,7 @@
         <v>874</v>
       </c>
       <c r="L65" s="11" t="s">
-        <v>3327</v>
+        <v>3326</v>
       </c>
       <c r="M65" s="10"/>
       <c r="N65" s="10"/>
@@ -41125,7 +41160,7 @@
         <v>888</v>
       </c>
       <c r="L85" s="11" t="s">
-        <v>3326</v>
+        <v>3325</v>
       </c>
       <c r="M85" s="10"/>
       <c r="N85" s="10"/>
@@ -41140,7 +41175,7 @@
       </c>
       <c r="C86" s="10"/>
       <c r="D86" s="11" t="s">
-        <v>3336</v>
+        <v>3335</v>
       </c>
       <c r="E86" s="10"/>
       <c r="F86" s="8" t="s">
@@ -43963,7 +43998,7 @@
         <v>3235</v>
       </c>
       <c r="G199" s="3" t="s">
-        <v>3344</v>
+        <v>3343</v>
       </c>
       <c r="H199" s="4"/>
       <c r="K199" s="14" t="s">
@@ -43984,7 +44019,7 @@
         <v>3239</v>
       </c>
       <c r="L200" s="4" t="s">
-        <v>3348</v>
+        <v>3347</v>
       </c>
     </row>
     <row r="201" spans="1:15" s="3" customFormat="1">
@@ -44001,7 +44036,7 @@
       </c>
       <c r="L201" s="4"/>
       <c r="N201" s="15" t="s">
-        <v>3341</v>
+        <v>3340</v>
       </c>
     </row>
     <row r="202" spans="1:15" s="3" customFormat="1">
@@ -44017,7 +44052,7 @@
         <v>3245</v>
       </c>
       <c r="L202" s="4" t="s">
-        <v>3345</v>
+        <v>3344</v>
       </c>
     </row>
     <row r="203" spans="1:15" s="3" customFormat="1">
@@ -44033,7 +44068,7 @@
         <v>3248</v>
       </c>
       <c r="L203" s="4" t="s">
-        <v>3354</v>
+        <v>3353</v>
       </c>
     </row>
     <row r="204" spans="1:15">
@@ -44157,7 +44192,7 @@
         <v>1340</v>
       </c>
       <c r="C209" s="10" t="s">
-        <v>3343</v>
+        <v>3342</v>
       </c>
       <c r="D209" s="10"/>
       <c r="E209" s="10"/>
@@ -44177,7 +44212,7 @@
         <v>518</v>
       </c>
       <c r="B210" s="10" t="s">
-        <v>3350</v>
+        <v>3349</v>
       </c>
       <c r="C210" s="10"/>
       <c r="D210" s="10"/>
@@ -44388,7 +44423,7 @@
         <v>516</v>
       </c>
       <c r="B219" s="10" t="s">
-        <v>3352</v>
+        <v>3351</v>
       </c>
       <c r="C219" s="10"/>
       <c r="D219" s="10"/>
@@ -44428,7 +44463,7 @@
         <v>1425</v>
       </c>
       <c r="C223" s="13" t="s">
-        <v>3328</v>
+        <v>3327</v>
       </c>
     </row>
     <row r="224" spans="1:15">
@@ -44436,10 +44471,10 @@
         <v>1643</v>
       </c>
       <c r="B224" s="12" t="s">
+        <v>3345</v>
+      </c>
+      <c r="C224" s="12" t="s">
         <v>3346</v>
-      </c>
-      <c r="C224" s="12" t="s">
-        <v>3347</v>
       </c>
     </row>
     <row r="225" spans="1:3">
@@ -44447,10 +44482,10 @@
         <v>1643</v>
       </c>
       <c r="B225" s="12" t="s">
-        <v>3349</v>
+        <v>3348</v>
       </c>
       <c r="C225" s="12" t="s">
-        <v>3351</v>
+        <v>3350</v>
       </c>
     </row>
     <row r="226" spans="1:3">
@@ -44458,7 +44493,7 @@
         <v>1643</v>
       </c>
       <c r="B226" s="12" t="s">
-        <v>3353</v>
+        <v>3352</v>
       </c>
     </row>
     <row r="228" spans="1:3">
@@ -44488,10 +44523,10 @@
         <v>1586</v>
       </c>
       <c r="B230" s="13" t="s">
+        <v>3328</v>
+      </c>
+      <c r="C230" s="13" t="s">
         <v>3329</v>
-      </c>
-      <c r="C230" s="13" t="s">
-        <v>3330</v>
       </c>
     </row>
     <row r="231" spans="1:3">
@@ -44499,10 +44534,10 @@
         <v>1586</v>
       </c>
       <c r="B231" s="13" t="s">
+        <v>3330</v>
+      </c>
+      <c r="C231" s="13" t="s">
         <v>3331</v>
-      </c>
-      <c r="C231" s="13" t="s">
-        <v>3332</v>
       </c>
     </row>
     <row r="232" spans="1:3">
@@ -44510,10 +44545,10 @@
         <v>1586</v>
       </c>
       <c r="B232" s="13" t="s">
+        <v>3332</v>
+      </c>
+      <c r="C232" s="13" t="s">
         <v>3333</v>
-      </c>
-      <c r="C232" s="13" t="s">
-        <v>3334</v>
       </c>
     </row>
   </sheetData>
@@ -44592,74 +44627,74 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F6A446E-DC4A-45B3-A3E3-4049BF48BC30}">
   <dimension ref="A1:N501"/>
-  <sheetFormatPr defaultColWidth="7.83203125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="7.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.08203125" style="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.125" style="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.25" style="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.25" style="12" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.25" style="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23" style="12" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.75" style="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.08203125" style="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.83203125" style="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.125" style="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.875" style="12" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19" style="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.75" style="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.08203125" style="12" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.125" style="12" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="7.25" style="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.33203125" style="12" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="7.83203125" style="12"/>
+    <col min="13" max="13" width="13.375" style="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="7.875" style="12"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" s="9" customFormat="1">
       <c r="A1" s="9" t="s">
+        <v>3390</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>3389</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>3391</v>
       </c>
-      <c r="B1" s="9" t="s">
-        <v>3390</v>
-      </c>
-      <c r="C1" s="9" t="s">
+      <c r="D1" s="9" t="s">
         <v>3392</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E1" s="9" t="s">
         <v>3393</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>3394</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>3395</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>3396</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>3397</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
+        <v>3400</v>
+      </c>
+      <c r="K1" s="9" t="s">
         <v>3398</v>
       </c>
-      <c r="J1" s="9" t="s">
-        <v>3401</v>
-      </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>3399</v>
-      </c>
-      <c r="L1" s="9" t="s">
-        <v>3400</v>
       </c>
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="12" t="s">
-        <v>3374</v>
+        <v>3373</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>3422</v>
+        <v>3421</v>
       </c>
       <c r="C2" s="96" t="s">
         <v>1547</v>
       </c>
       <c r="D2" s="97" t="s">
-        <v>3402</v>
+        <v>3401</v>
       </c>
       <c r="E2" s="100" t="s">
         <v>1552</v>
@@ -44677,21 +44712,21 @@
         <v>1548</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>3426</v>
+        <v>3425</v>
       </c>
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="10" t="s">
-        <v>3378</v>
+        <v>3377</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>3419</v>
+        <v>3418</v>
       </c>
       <c r="C3" s="96" t="s">
         <v>1499</v>
       </c>
       <c r="D3" s="97" t="s">
-        <v>3402</v>
+        <v>3401</v>
       </c>
       <c r="E3" s="100" t="s">
         <v>1495</v>
@@ -44706,21 +44741,21 @@
         <v>1498</v>
       </c>
       <c r="M3" s="12" t="s">
-        <v>3427</v>
+        <v>3426</v>
       </c>
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="10" t="s">
-        <v>3382</v>
+        <v>3381</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="C4" s="96" t="s">
         <v>1503</v>
       </c>
       <c r="D4" s="97" t="s">
-        <v>3402</v>
+        <v>3401</v>
       </c>
       <c r="E4" s="100" t="s">
         <v>1504</v>
@@ -44729,24 +44764,24 @@
         <v>1505</v>
       </c>
       <c r="H4" s="105" t="s">
-        <v>3411</v>
+        <v>3410</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>3441</v>
+        <v>3440</v>
       </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="10" t="s">
-        <v>3363</v>
+        <v>3362</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>3420</v>
+        <v>3419</v>
       </c>
       <c r="C5" s="95" t="s">
         <v>726</v>
       </c>
       <c r="D5" s="97" t="s">
-        <v>3402</v>
+        <v>3401</v>
       </c>
       <c r="E5" s="99" t="s">
         <v>724</v>
@@ -44761,21 +44796,21 @@
         <v>722</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>3442</v>
+        <v>3441</v>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="10" t="s">
-        <v>3371</v>
+        <v>3370</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>3420</v>
+        <v>3419</v>
       </c>
       <c r="C6" s="96" t="s">
         <v>756</v>
       </c>
       <c r="D6" s="97" t="s">
-        <v>3402</v>
+        <v>3401</v>
       </c>
       <c r="E6" s="100" t="s">
         <v>757</v>
@@ -44787,15 +44822,15 @@
         <v>755</v>
       </c>
       <c r="M6" s="12" t="s">
-        <v>3428</v>
+        <v>3427</v>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="10" t="s">
-        <v>3360</v>
+        <v>3359</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="C7" s="95" t="s">
         <v>713</v>
@@ -44810,15 +44845,15 @@
         <v>711</v>
       </c>
       <c r="M7" s="12" t="s">
-        <v>3440</v>
+        <v>3439</v>
       </c>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="12" t="s">
-        <v>3362</v>
+        <v>3361</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>3417</v>
+        <v>3416</v>
       </c>
       <c r="C8" s="95" t="s">
         <v>720</v>
@@ -44833,18 +44868,18 @@
         <v>718</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>3443</v>
+        <v>3442</v>
       </c>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="12" t="s">
-        <v>3376</v>
+        <v>3375</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>3417</v>
+        <v>3416</v>
       </c>
       <c r="C9" s="96" t="s">
-        <v>3406</v>
+        <v>3405</v>
       </c>
       <c r="D9" s="98" t="s">
         <v>1487</v>
@@ -44856,44 +44891,44 @@
         <v>1488</v>
       </c>
       <c r="N9" s="12" t="s">
-        <v>3434</v>
+        <v>3433</v>
       </c>
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="12" t="s">
-        <v>3380</v>
+        <v>3379</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="C10" s="96" t="s">
         <v>1536</v>
       </c>
       <c r="D10" s="98" t="s">
-        <v>3408</v>
+        <v>3407</v>
       </c>
       <c r="E10" s="100" t="s">
         <v>1537</v>
       </c>
       <c r="F10" s="102" t="s">
-        <v>3409</v>
+        <v>3408</v>
       </c>
       <c r="M10" s="12" t="s">
-        <v>3437</v>
+        <v>3436</v>
       </c>
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="10" t="s">
-        <v>3386</v>
+        <v>3385</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>3420</v>
+        <v>3419</v>
       </c>
       <c r="C11" s="96" t="s">
         <v>1465</v>
       </c>
       <c r="D11" s="97" t="s">
-        <v>3402</v>
+        <v>3401</v>
       </c>
       <c r="E11" s="100" t="s">
         <v>1543</v>
@@ -44902,21 +44937,21 @@
         <v>1542</v>
       </c>
       <c r="M11" s="12" t="s">
-        <v>3444</v>
+        <v>3443</v>
       </c>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="12" t="s">
-        <v>3370</v>
+        <v>3369</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>3419</v>
+        <v>3418</v>
       </c>
       <c r="C12" s="96" t="s">
         <v>751</v>
       </c>
       <c r="D12" s="97" t="s">
-        <v>3402</v>
+        <v>3401</v>
       </c>
       <c r="F12" s="102" t="s">
         <v>752</v>
@@ -44928,21 +44963,21 @@
         <v>753</v>
       </c>
       <c r="M12" s="12" t="s">
-        <v>3445</v>
+        <v>3444</v>
       </c>
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="10" t="s">
-        <v>3361</v>
+        <v>3360</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>3419</v>
+        <v>3418</v>
       </c>
       <c r="C13" s="95" t="s">
         <v>717</v>
       </c>
       <c r="D13" s="97" t="s">
-        <v>3402</v>
+        <v>3401</v>
       </c>
       <c r="F13" s="101" t="s">
         <v>715</v>
@@ -44954,15 +44989,15 @@
         <v>714</v>
       </c>
       <c r="M13" s="12" t="s">
-        <v>3446</v>
+        <v>3445</v>
       </c>
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="111" t="s">
-        <v>3358</v>
+        <v>3357</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="C14" s="95" t="s">
         <v>703</v>
@@ -44974,15 +45009,15 @@
         <v>705</v>
       </c>
       <c r="M14" s="12" t="s">
-        <v>3447</v>
+        <v>3446</v>
       </c>
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="111" t="s">
-        <v>3385</v>
+        <v>3384</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="E15" s="100" t="s">
         <v>1511</v>
@@ -44991,18 +45026,18 @@
         <v>1512</v>
       </c>
       <c r="I15" s="107" t="s">
-        <v>3412</v>
+        <v>3411</v>
       </c>
       <c r="M15" s="12" t="s">
-        <v>3450</v>
+        <v>3449</v>
       </c>
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="12" t="s">
-        <v>3356</v>
+        <v>3355</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>3417</v>
+        <v>3416</v>
       </c>
       <c r="C16" s="95" t="s">
         <v>699</v>
@@ -45014,15 +45049,15 @@
         <v>698</v>
       </c>
       <c r="M16" s="12" t="s">
-        <v>3448</v>
+        <v>3447</v>
       </c>
     </row>
     <row r="17" spans="1:14">
       <c r="A17" s="111" t="s">
-        <v>3384</v>
+        <v>3383</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>3422</v>
+        <v>3421</v>
       </c>
       <c r="C17" s="96" t="s">
         <v>1490</v>
@@ -45031,18 +45066,18 @@
         <v>1491</v>
       </c>
       <c r="M17" s="12" t="s">
-        <v>3436</v>
+        <v>3435</v>
       </c>
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="111" t="s">
-        <v>3379</v>
+        <v>3378</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="F18" s="102" t="s">
-        <v>3407</v>
+        <v>3406</v>
       </c>
       <c r="G18" s="103" t="s">
         <v>1507</v>
@@ -45057,15 +45092,15 @@
         <v>1506</v>
       </c>
       <c r="M18" s="12" t="s">
-        <v>3450</v>
+        <v>3449</v>
       </c>
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="12" t="s">
-        <v>3375</v>
+        <v>3374</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>3420</v>
+        <v>3419</v>
       </c>
       <c r="C19" s="96" t="s">
         <v>1533</v>
@@ -45074,24 +45109,24 @@
         <v>1534</v>
       </c>
       <c r="F19" s="102" t="s">
-        <v>3405</v>
+        <v>3404</v>
       </c>
       <c r="H19" s="105" t="s">
-        <v>3404</v>
+        <v>3403</v>
       </c>
       <c r="J19" s="110" t="s">
         <v>1531</v>
       </c>
       <c r="M19" s="12" t="s">
-        <v>3429</v>
+        <v>3428</v>
       </c>
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="95" t="s">
-        <v>3364</v>
+        <v>3363</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="C20" s="95" t="s">
         <v>727</v>
@@ -45109,15 +45144,15 @@
         <v>730</v>
       </c>
       <c r="N20" s="12" t="s">
-        <v>3433</v>
+        <v>3432</v>
       </c>
     </row>
     <row r="21" spans="1:14">
       <c r="A21" s="111" t="s">
-        <v>3368</v>
+        <v>3367</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="C21" s="96" t="s">
         <v>746</v>
@@ -45131,10 +45166,10 @@
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="10" t="s">
-        <v>3372</v>
+        <v>3371</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>3423</v>
+        <v>3422</v>
       </c>
       <c r="C22" s="96" t="s">
         <v>1483</v>
@@ -45149,18 +45184,18 @@
         <v>1485</v>
       </c>
       <c r="M22" s="12" t="s">
-        <v>3430</v>
+        <v>3429</v>
       </c>
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="10" t="s">
-        <v>3373</v>
+        <v>3372</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>3424</v>
+        <v>3423</v>
       </c>
       <c r="C23" s="96" t="s">
-        <v>3403</v>
+        <v>3402</v>
       </c>
       <c r="E23" s="100" t="s">
         <v>1492</v>
@@ -45172,15 +45207,15 @@
         <v>1494</v>
       </c>
       <c r="N23" s="12" t="s">
-        <v>3435</v>
+        <v>3434</v>
       </c>
     </row>
     <row r="24" spans="1:14">
       <c r="A24" s="95" t="s">
-        <v>3367</v>
+        <v>3366</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>3422</v>
+        <v>3421</v>
       </c>
       <c r="C24" s="96" t="s">
         <v>743</v>
@@ -45192,18 +45227,18 @@
         <v>742</v>
       </c>
       <c r="M24" s="12" t="s">
-        <v>3449</v>
+        <v>3448</v>
       </c>
       <c r="N24" s="12" t="s">
-        <v>3433</v>
+        <v>3432</v>
       </c>
     </row>
     <row r="25" spans="1:14">
       <c r="A25" s="95" t="s">
-        <v>3357</v>
+        <v>3356</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="D25" s="97" t="s">
         <v>701</v>
@@ -45215,15 +45250,15 @@
         <v>700</v>
       </c>
       <c r="M25" s="12" t="s">
-        <v>3450</v>
+        <v>3449</v>
       </c>
     </row>
     <row r="26" spans="1:14">
       <c r="A26" s="10" t="s">
-        <v>3383</v>
+        <v>3382</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="C26" s="96" t="s">
         <v>1500</v>
@@ -45235,15 +45270,15 @@
         <v>1501</v>
       </c>
       <c r="M26" s="12" t="s">
-        <v>3439</v>
+        <v>3438</v>
       </c>
     </row>
     <row r="27" spans="1:14">
       <c r="A27" s="111" t="s">
-        <v>3366</v>
+        <v>3365</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>3421</v>
+        <v>3420</v>
       </c>
       <c r="C27" s="96" t="s">
         <v>739</v>
@@ -45255,15 +45290,15 @@
         <v>740</v>
       </c>
       <c r="N27" s="12" t="s">
-        <v>3433</v>
+        <v>3432</v>
       </c>
     </row>
     <row r="28" spans="1:14">
       <c r="A28" s="111" t="s">
-        <v>3369</v>
+        <v>3368</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="C28" s="96" t="s">
         <v>747</v>
@@ -45280,10 +45315,10 @@
     </row>
     <row r="29" spans="1:14">
       <c r="A29" s="10" t="s">
-        <v>3365</v>
+        <v>3364</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="D29" s="98" t="s">
         <v>737</v>
@@ -45304,55 +45339,55 @@
         <v>735</v>
       </c>
       <c r="M29" s="12" t="s">
-        <v>3452</v>
+        <v>3451</v>
       </c>
     </row>
     <row r="30" spans="1:14">
       <c r="A30" s="95" t="s">
-        <v>3388</v>
+        <v>3387</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>3425</v>
+        <v>3424</v>
       </c>
       <c r="C30" s="96" t="s">
+        <v>3335</v>
+      </c>
+      <c r="F30" s="102" t="s">
         <v>3336</v>
       </c>
-      <c r="F30" s="102" t="s">
-        <v>3337</v>
-      </c>
       <c r="H30" s="105" t="s">
-        <v>3335</v>
+        <v>3334</v>
       </c>
       <c r="N30" s="12" t="s">
-        <v>3433</v>
+        <v>3432</v>
       </c>
     </row>
     <row r="31" spans="1:14">
       <c r="A31" s="111" t="s">
-        <v>3387</v>
+        <v>3386</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>3421</v>
+        <v>3420</v>
       </c>
       <c r="C31" s="96" t="s">
-        <v>3416</v>
+        <v>3415</v>
       </c>
       <c r="E31" s="100" t="s">
+        <v>3412</v>
+      </c>
+      <c r="G31" s="103" t="s">
+        <v>3414</v>
+      </c>
+      <c r="I31" s="107" t="s">
         <v>3413</v>
-      </c>
-      <c r="G31" s="103" t="s">
-        <v>3415</v>
-      </c>
-      <c r="I31" s="107" t="s">
-        <v>3414</v>
       </c>
     </row>
     <row r="32" spans="1:14">
       <c r="A32" s="10" t="s">
-        <v>3377</v>
+        <v>3376</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>3421</v>
+        <v>3420</v>
       </c>
       <c r="D32" s="98" t="s">
         <v>1478</v>
@@ -45370,44 +45405,44 @@
         <v>1481</v>
       </c>
       <c r="M32" s="12" t="s">
-        <v>3431</v>
+        <v>3430</v>
       </c>
     </row>
     <row r="33" spans="1:13">
       <c r="A33" s="12" t="s">
-        <v>3389</v>
+        <v>3388</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>3425</v>
+        <v>3424</v>
       </c>
       <c r="D33" s="98" t="s">
-        <v>3341</v>
+        <v>3340</v>
       </c>
       <c r="E33" s="100" t="s">
+        <v>3337</v>
+      </c>
+      <c r="F33" s="102" t="s">
         <v>3338</v>
       </c>
-      <c r="F33" s="102" t="s">
+      <c r="G33" s="103" t="s">
         <v>3339</v>
       </c>
-      <c r="G33" s="103" t="s">
-        <v>3340</v>
-      </c>
       <c r="I33" s="107" t="s">
-        <v>3355</v>
+        <v>3354</v>
       </c>
       <c r="M33" s="12" t="s">
-        <v>3432</v>
+        <v>3431</v>
       </c>
     </row>
     <row r="34" spans="1:13">
       <c r="A34" s="10" t="s">
-        <v>3381</v>
+        <v>3380</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="D34" s="98" t="s">
-        <v>3410</v>
+        <v>3409</v>
       </c>
       <c r="E34" s="100" t="s">
         <v>1514</v>
@@ -45419,15 +45454,15 @@
         <v>1546</v>
       </c>
       <c r="M34" s="12" t="s">
-        <v>3438</v>
+        <v>3437</v>
       </c>
     </row>
     <row r="35" spans="1:13">
       <c r="A35" s="12" t="s">
-        <v>3359</v>
+        <v>3358</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="E35" s="99" t="s">
         <v>707</v>
@@ -45442,7 +45477,7 @@
         <v>709</v>
       </c>
       <c r="M35" s="12" t="s">
-        <v>3451</v>
+        <v>3450</v>
       </c>
     </row>
     <row r="36" spans="1:13">

</xml_diff>

<commit_message>
Caldesann's Despair complete balance
</commit_message>
<xml_diff>
--- a/Diablo II.xlsx
+++ b/Diablo II.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yatyr\workspace\d2r-loot-filter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C07BDB-A805-4D42-950C-9B4CC06C806F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D6D3984-0BAB-4E90-817B-835233B8568C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{4FA0E628-D5C1-45F8-838A-535ABF901563}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{4FA0E628-D5C1-45F8-838A-535ABF901563}"/>
   </bookViews>
   <sheets>
     <sheet name="Mod-Config" sheetId="6" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6659" uniqueCount="3636">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6596" uniqueCount="3604">
   <si>
     <t>Key</t>
   </si>
@@ -12408,105 +12408,6 @@
     <t>skill-war</t>
   </si>
   <si>
-    <t>r01</t>
-  </si>
-  <si>
-    <t>r02</t>
-  </si>
-  <si>
-    <t>r03</t>
-  </si>
-  <si>
-    <t>r04</t>
-  </si>
-  <si>
-    <t>r05</t>
-  </si>
-  <si>
-    <t>r06</t>
-  </si>
-  <si>
-    <t>r07</t>
-  </si>
-  <si>
-    <t>r08</t>
-  </si>
-  <si>
-    <t>r09</t>
-  </si>
-  <si>
-    <t>r10</t>
-  </si>
-  <si>
-    <t>r11</t>
-  </si>
-  <si>
-    <t>r12</t>
-  </si>
-  <si>
-    <t>r13</t>
-  </si>
-  <si>
-    <t>r14</t>
-  </si>
-  <si>
-    <t>r15</t>
-  </si>
-  <si>
-    <t>r16</t>
-  </si>
-  <si>
-    <t>r17</t>
-  </si>
-  <si>
-    <t>r18</t>
-  </si>
-  <si>
-    <t>r19</t>
-  </si>
-  <si>
-    <t>r20</t>
-  </si>
-  <si>
-    <t>r21</t>
-  </si>
-  <si>
-    <t>r22</t>
-  </si>
-  <si>
-    <t>r23</t>
-  </si>
-  <si>
-    <t>r24</t>
-  </si>
-  <si>
-    <t>r25</t>
-  </si>
-  <si>
-    <t>r26</t>
-  </si>
-  <si>
-    <t>r27</t>
-  </si>
-  <si>
-    <t>r28</t>
-  </si>
-  <si>
-    <t>r29</t>
-  </si>
-  <si>
-    <t>r30</t>
-  </si>
-  <si>
-    <t>r31</t>
-  </si>
-  <si>
-    <t>r32</t>
-  </si>
-  <si>
-    <t>r33</t>
-  </si>
-  <si>
     <t>111</t>
   </si>
   <si>
@@ -12714,6 +12615,9 @@
 Rare Gloves + 3 Burning Essence of Terror + Eastern Worldstone Shard -&gt; Upgraded to Set Gloves
 Rare Boots + 3 Burning Essence of Terror + Southern Worldstone Shard -&gt; Upgraded to Set Boots
 Rare Belt + 3 Burning Essence of Terror + Northern Worldstone Shard -&gt; Upgraded to Set Belt</t>
+  </si>
+  <si>
+    <t>abs-mag%</t>
   </si>
 </sst>
 </file>
@@ -13937,7 +13841,7 @@
         <v>2711</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>3635</v>
+        <v>3602</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -13959,7 +13863,7 @@
         <v>3306</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>3610</v>
+        <v>3577</v>
       </c>
     </row>
   </sheetData>
@@ -39012,7 +38916,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="A1:S99"/>
+  <dimension ref="A1:R107"/>
   <sheetFormatPr defaultRowHeight="15.5"/>
   <cols>
     <col min="2" max="2" width="10.4140625" style="113" bestFit="1" customWidth="1"/>
@@ -39021,7 +38925,7 @@
     <col min="8" max="8" width="11.9140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:18">
       <c r="A1" t="s">
         <v>3457</v>
       </c>
@@ -39035,7 +38939,7 @@
         <v>3460</v>
       </c>
       <c r="E1" t="s">
-        <v>3592</v>
+        <v>3559</v>
       </c>
       <c r="F1" t="s">
         <v>3461</v>
@@ -39044,134 +38948,149 @@
         <v>3462</v>
       </c>
       <c r="I1" s="113" t="s">
-        <v>3572</v>
+        <v>3539</v>
       </c>
       <c r="J1" s="113" t="s">
-        <v>3574</v>
+        <v>3541</v>
       </c>
       <c r="K1" s="113" t="s">
-        <v>3575</v>
+        <v>3542</v>
       </c>
       <c r="L1" s="113" t="s">
-        <v>3573</v>
+        <v>3540</v>
       </c>
       <c r="M1" s="113" t="s">
-        <v>3577</v>
+        <v>3544</v>
       </c>
       <c r="N1" s="113" t="s">
-        <v>3578</v>
+        <v>3545</v>
       </c>
       <c r="O1" s="113" t="s">
-        <v>3579</v>
+        <v>3546</v>
       </c>
       <c r="P1" s="113" t="s">
-        <v>3580</v>
+        <v>3547</v>
       </c>
       <c r="Q1" s="113"/>
       <c r="R1" s="113"/>
-      <c r="S1" s="113"/>
-    </row>
-    <row r="2" spans="1:19">
+    </row>
+    <row r="2" spans="1:18">
       <c r="A2" t="s">
-        <v>3608</v>
+        <v>3575</v>
       </c>
       <c r="B2" s="113" t="s">
-        <v>3572</v>
-      </c>
-      <c r="C2" t="s">
         <v>3539</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
       </c>
       <c r="D2" t="s">
         <v>2754</v>
       </c>
       <c r="F2">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="G2">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="I2" t="s">
         <v>2754</v>
       </c>
-    </row>
-    <row r="3" spans="1:19">
+      <c r="Q2">
+        <f>C2-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
       <c r="A3" t="s">
         <v>2697</v>
       </c>
       <c r="B3" s="113" t="s">
-        <v>3573</v>
-      </c>
-      <c r="C3" t="s">
         <v>3540</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
       </c>
       <c r="D3" t="s">
         <v>2752</v>
       </c>
       <c r="F3">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="G3">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="L3" t="s">
         <v>2752</v>
       </c>
-    </row>
-    <row r="4" spans="1:19">
+      <c r="Q3">
+        <f t="shared" ref="Q3:Q66" si="0">C3-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18">
       <c r="A4" t="s">
-        <v>3609</v>
+        <v>3576</v>
       </c>
       <c r="B4" s="113" t="s">
-        <v>3575</v>
-      </c>
-      <c r="C4" t="s">
-        <v>3541</v>
+        <v>3542</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
       </c>
       <c r="D4" t="s">
         <v>2813</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="G4">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="K4" s="112" t="s">
         <v>2813</v>
       </c>
-    </row>
-    <row r="5" spans="1:19">
+      <c r="Q4">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18">
       <c r="A5" t="s">
-        <v>3609</v>
+        <v>3576</v>
       </c>
       <c r="B5" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C5" t="s">
-        <v>3542</v>
+        <v>3541</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
       </c>
       <c r="D5" t="s">
         <v>2710</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="G5">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="J5" s="112" t="s">
         <v>2710</v>
       </c>
-    </row>
-    <row r="6" spans="1:19">
+      <c r="Q5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18">
       <c r="A6" t="s">
-        <v>3609</v>
+        <v>3576</v>
       </c>
       <c r="B6" s="113" t="s">
-        <v>3575</v>
-      </c>
-      <c r="C6" t="s">
-        <v>3543</v>
+        <v>3542</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
       </c>
       <c r="D6" t="s">
         <v>2719</v>
@@ -39188,16 +39107,20 @@
       <c r="K6" t="s">
         <v>2719</v>
       </c>
-    </row>
-    <row r="7" spans="1:19">
+      <c r="Q6">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18">
       <c r="A7" t="s">
-        <v>3609</v>
+        <v>3576</v>
       </c>
       <c r="B7" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C7" t="s">
-        <v>3543</v>
+        <v>3541</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
       </c>
       <c r="D7" t="s">
         <v>2837</v>
@@ -39208,16 +39131,20 @@
       <c r="G7">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:19">
+      <c r="Q7">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18">
       <c r="A8" t="s">
-        <v>3609</v>
+        <v>3576</v>
       </c>
       <c r="B8" s="113" t="s">
-        <v>3575</v>
-      </c>
-      <c r="C8" t="s">
-        <v>3544</v>
+        <v>3542</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
       </c>
       <c r="D8" t="s">
         <v>2718</v>
@@ -39234,19 +39161,23 @@
       <c r="K8" s="112" t="s">
         <v>3496</v>
       </c>
-    </row>
-    <row r="9" spans="1:19">
+      <c r="Q8">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18">
       <c r="A9" t="s">
-        <v>3609</v>
+        <v>3576</v>
       </c>
       <c r="B9" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C9" t="s">
-        <v>3544</v>
+        <v>3541</v>
+      </c>
+      <c r="C9">
+        <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>3576</v>
+        <v>3543</v>
       </c>
       <c r="F9">
         <v>1</v>
@@ -39256,19 +39187,23 @@
       </c>
       <c r="J9" s="112"/>
       <c r="K9" s="112"/>
-    </row>
-    <row r="10" spans="1:19">
+      <c r="Q9">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18">
       <c r="A10" t="s">
-        <v>3609</v>
+        <v>3576</v>
       </c>
       <c r="B10" s="113" t="s">
-        <v>3575</v>
-      </c>
-      <c r="C10" t="s">
-        <v>3545</v>
+        <v>3542</v>
+      </c>
+      <c r="C10">
+        <v>5</v>
       </c>
       <c r="D10" t="s">
-        <v>3581</v>
+        <v>3548</v>
       </c>
       <c r="F10">
         <v>1</v>
@@ -39282,19 +39217,23 @@
       <c r="K10" s="112" t="s">
         <v>3499</v>
       </c>
-    </row>
-    <row r="11" spans="1:19">
+      <c r="Q10">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18">
       <c r="A11" t="s">
-        <v>3609</v>
+        <v>3576</v>
       </c>
       <c r="B11" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C11" t="s">
-        <v>3545</v>
+        <v>3541</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>3582</v>
+        <v>3549</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -39304,117 +39243,137 @@
       </c>
       <c r="J11" s="112"/>
       <c r="K11" s="112"/>
-    </row>
-    <row r="12" spans="1:19">
+      <c r="Q11">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18">
       <c r="A12" t="s">
         <v>2696</v>
       </c>
       <c r="B12" s="113" t="s">
-        <v>3577</v>
-      </c>
-      <c r="C12" t="s">
-        <v>3546</v>
+        <v>3544</v>
+      </c>
+      <c r="C12">
+        <v>6</v>
       </c>
       <c r="D12" t="s">
         <v>2784</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G12">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M12" s="112" t="s">
         <v>3463</v>
       </c>
-    </row>
-    <row r="13" spans="1:19">
+      <c r="Q12">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18">
       <c r="A13" t="s">
         <v>2696</v>
       </c>
       <c r="B13" s="113" t="s">
-        <v>3578</v>
-      </c>
-      <c r="C13" t="s">
-        <v>3547</v>
+        <v>3545</v>
+      </c>
+      <c r="C13">
+        <v>7</v>
       </c>
       <c r="D13" t="s">
         <v>2792</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G13">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N13" s="112" t="s">
         <v>3464</v>
       </c>
-    </row>
-    <row r="14" spans="1:19">
+      <c r="Q13">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18">
       <c r="A14" t="s">
         <v>2696</v>
       </c>
       <c r="B14" s="113" t="s">
-        <v>3579</v>
-      </c>
-      <c r="C14" t="s">
-        <v>3548</v>
+        <v>3546</v>
+      </c>
+      <c r="C14">
+        <v>8</v>
       </c>
       <c r="D14" t="s">
         <v>2783</v>
       </c>
       <c r="F14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O14" s="112" t="s">
         <v>3465</v>
       </c>
-    </row>
-    <row r="15" spans="1:19">
+      <c r="Q14">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18">
       <c r="A15" t="s">
         <v>2696</v>
       </c>
       <c r="B15" s="113" t="s">
-        <v>3580</v>
-      </c>
-      <c r="C15" t="s">
-        <v>3549</v>
+        <v>3547</v>
+      </c>
+      <c r="C15">
+        <v>9</v>
       </c>
       <c r="D15" t="s">
         <v>2762</v>
       </c>
       <c r="F15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G15">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P15" s="112" t="s">
         <v>3466</v>
       </c>
-    </row>
-    <row r="16" spans="1:19">
+      <c r="Q15">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18">
       <c r="A16" t="s">
         <v>2697</v>
       </c>
       <c r="B16" s="113" t="s">
-        <v>3578</v>
-      </c>
-      <c r="C16" t="s">
-        <v>3550</v>
+        <v>3545</v>
+      </c>
+      <c r="C16">
+        <v>10</v>
       </c>
       <c r="D16" t="s">
         <v>2731</v>
       </c>
       <c r="F16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I16" s="112" t="s">
         <v>3468</v>
@@ -39434,25 +39393,29 @@
       <c r="O16" s="112" t="s">
         <v>3471</v>
       </c>
-    </row>
-    <row r="17" spans="1:16">
+      <c r="Q16">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17">
       <c r="A17" t="s">
         <v>2697</v>
       </c>
       <c r="B17" s="113" t="s">
-        <v>3572</v>
-      </c>
-      <c r="C17" t="s">
-        <v>3550</v>
+        <v>3539</v>
+      </c>
+      <c r="C17">
+        <v>10</v>
       </c>
       <c r="D17" t="s">
         <v>2729</v>
       </c>
       <c r="F17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G17">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I17" s="112"/>
       <c r="J17" s="112"/>
@@ -39460,25 +39423,29 @@
       <c r="L17" s="112"/>
       <c r="N17" s="112"/>
       <c r="O17" s="112"/>
-    </row>
-    <row r="18" spans="1:16">
+      <c r="Q17">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17">
       <c r="A18" t="s">
         <v>2697</v>
       </c>
       <c r="B18" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C18" t="s">
-        <v>3550</v>
+        <v>3541</v>
+      </c>
+      <c r="C18">
+        <v>10</v>
       </c>
       <c r="D18" t="s">
         <v>2733</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I18" s="112"/>
       <c r="J18" s="112"/>
@@ -39486,25 +39453,29 @@
       <c r="L18" s="112"/>
       <c r="N18" s="112"/>
       <c r="O18" s="112"/>
-    </row>
-    <row r="19" spans="1:16">
+      <c r="Q18">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17">
       <c r="A19" t="s">
         <v>2697</v>
       </c>
       <c r="B19" s="113" t="s">
-        <v>3575</v>
-      </c>
-      <c r="C19" t="s">
-        <v>3550</v>
+        <v>3542</v>
+      </c>
+      <c r="C19">
+        <v>10</v>
       </c>
       <c r="D19" t="s">
         <v>2726</v>
       </c>
       <c r="F19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I19" s="112"/>
       <c r="J19" s="112"/>
@@ -39512,25 +39483,29 @@
       <c r="L19" s="112"/>
       <c r="N19" s="112"/>
       <c r="O19" s="112"/>
-    </row>
-    <row r="20" spans="1:16">
+      <c r="Q19">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17">
       <c r="A20" t="s">
         <v>2697</v>
       </c>
       <c r="B20" s="113" t="s">
-        <v>3579</v>
-      </c>
-      <c r="C20" t="s">
+        <v>3546</v>
+      </c>
+      <c r="C20">
+        <v>10</v>
+      </c>
+      <c r="D20" t="s">
         <v>3550</v>
       </c>
-      <c r="D20" t="s">
-        <v>3583</v>
-      </c>
       <c r="F20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I20" s="112"/>
       <c r="J20" s="112"/>
@@ -39538,25 +39513,29 @@
       <c r="L20" s="112"/>
       <c r="N20" s="112"/>
       <c r="O20" s="112"/>
-    </row>
-    <row r="21" spans="1:16">
+      <c r="Q20">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17">
       <c r="A21" t="s">
         <v>2697</v>
       </c>
       <c r="B21" s="113" t="s">
-        <v>3573</v>
-      </c>
-      <c r="C21" t="s">
-        <v>3550</v>
+        <v>3540</v>
+      </c>
+      <c r="C21">
+        <v>10</v>
       </c>
       <c r="D21" t="s">
         <v>2720</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I21" s="112"/>
       <c r="J21" s="112"/>
@@ -39564,65 +39543,77 @@
       <c r="L21" s="112"/>
       <c r="N21" s="112"/>
       <c r="O21" s="112"/>
-    </row>
-    <row r="22" spans="1:16">
+      <c r="Q21">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17">
       <c r="A22" t="s">
-        <v>3607</v>
+        <v>3574</v>
       </c>
       <c r="B22" s="113" t="s">
-        <v>3575</v>
-      </c>
-      <c r="C22" t="s">
-        <v>3551</v>
+        <v>3542</v>
+      </c>
+      <c r="C22">
+        <v>11</v>
       </c>
       <c r="D22" t="s">
         <v>2773</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G22">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="K22" s="112" t="s">
         <v>3502</v>
       </c>
-    </row>
-    <row r="23" spans="1:16">
+      <c r="Q22">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17">
       <c r="A23" t="s">
-        <v>3607</v>
+        <v>3574</v>
       </c>
       <c r="B23" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C23" t="s">
-        <v>3552</v>
+        <v>3541</v>
+      </c>
+      <c r="C23">
+        <v>12</v>
       </c>
       <c r="D23" t="s">
         <v>2772</v>
       </c>
       <c r="F23">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G23">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J23" s="112" t="s">
         <v>3501</v>
       </c>
-    </row>
-    <row r="24" spans="1:16">
+      <c r="Q23">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17">
       <c r="A24" t="s">
         <v>2697</v>
       </c>
       <c r="B24" s="113" t="s">
-        <v>3573</v>
-      </c>
-      <c r="C24" t="s">
-        <v>3553</v>
+        <v>3540</v>
+      </c>
+      <c r="C24">
+        <v>13</v>
       </c>
       <c r="D24" t="s">
-        <v>3584</v>
+        <v>3551</v>
       </c>
       <c r="F24">
         <v>1</v>
@@ -39633,19 +39624,23 @@
       <c r="L24" s="112" t="s">
         <v>3490</v>
       </c>
-    </row>
-    <row r="25" spans="1:16">
+      <c r="Q24">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17">
       <c r="A25" t="s">
-        <v>3608</v>
+        <v>3575</v>
       </c>
       <c r="B25" s="113" t="s">
-        <v>3573</v>
-      </c>
-      <c r="C25" t="s">
-        <v>3554</v>
+        <v>3540</v>
+      </c>
+      <c r="C25">
+        <v>14</v>
       </c>
       <c r="D25" t="s">
-        <v>3585</v>
+        <v>3552</v>
       </c>
       <c r="F25">
         <v>1</v>
@@ -39656,19 +39651,23 @@
       <c r="L25" s="112" t="s">
         <v>3491</v>
       </c>
-    </row>
-    <row r="26" spans="1:16">
+      <c r="Q25">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17">
       <c r="A26" t="s">
-        <v>3608</v>
+        <v>3575</v>
       </c>
       <c r="B26" s="113" t="s">
-        <v>3573</v>
-      </c>
-      <c r="C26" t="s">
-        <v>3555</v>
+        <v>3539</v>
+      </c>
+      <c r="C26">
+        <v>14</v>
       </c>
       <c r="D26" t="s">
-        <v>3586</v>
+        <v>3553</v>
       </c>
       <c r="F26">
         <v>1</v>
@@ -39676,78 +39675,76 @@
       <c r="G26">
         <v>1</v>
       </c>
-      <c r="L26" s="112" t="s">
+      <c r="I26" s="112" t="s">
         <v>3492</v>
       </c>
-    </row>
-    <row r="27" spans="1:16">
+      <c r="Q26">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17">
       <c r="A27" t="s">
-        <v>2697</v>
+        <v>3576</v>
       </c>
       <c r="B27" s="113" t="s">
-        <v>3578</v>
-      </c>
-      <c r="C27" t="s">
-        <v>3556</v>
+        <v>3542</v>
+      </c>
+      <c r="C27">
+        <v>15</v>
       </c>
       <c r="D27" t="s">
-        <v>3587</v>
+        <v>2722</v>
       </c>
       <c r="F27">
         <v>1</v>
       </c>
       <c r="G27">
-        <v>1</v>
-      </c>
-      <c r="I27" s="112" t="s">
-        <v>3485</v>
-      </c>
-      <c r="J27" s="112" t="s">
-        <v>3486</v>
-      </c>
-      <c r="K27" s="112" t="s">
-        <v>3487</v>
-      </c>
-      <c r="N27" s="112" t="s">
-        <v>3484</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16">
+        <v>2</v>
+      </c>
+      <c r="L27" s="112"/>
+      <c r="Q27">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17">
       <c r="A28" t="s">
-        <v>2697</v>
+        <v>3576</v>
       </c>
       <c r="B28" s="113" t="s">
-        <v>3572</v>
-      </c>
-      <c r="C28" t="s">
-        <v>3556</v>
+        <v>3541</v>
+      </c>
+      <c r="C28">
+        <v>15</v>
       </c>
       <c r="D28" t="s">
-        <v>3588</v>
+        <v>2848</v>
       </c>
       <c r="F28">
         <v>1</v>
       </c>
       <c r="G28">
-        <v>1</v>
-      </c>
-      <c r="I28" s="112"/>
-      <c r="J28" s="112"/>
-      <c r="K28" s="112"/>
-      <c r="N28" s="112"/>
-    </row>
-    <row r="29" spans="1:16">
+        <v>2</v>
+      </c>
+      <c r="L28" s="112"/>
+      <c r="Q28">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17">
       <c r="A29" t="s">
         <v>2697</v>
       </c>
       <c r="B29" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C29" t="s">
-        <v>3556</v>
+        <v>3545</v>
+      </c>
+      <c r="C29">
+        <v>16</v>
       </c>
       <c r="D29" t="s">
-        <v>3589</v>
+        <v>3554</v>
       </c>
       <c r="F29">
         <v>1</v>
@@ -39755,23 +39752,35 @@
       <c r="G29">
         <v>1</v>
       </c>
-      <c r="I29" s="112"/>
-      <c r="J29" s="112"/>
-      <c r="K29" s="112"/>
-      <c r="N29" s="112"/>
-    </row>
-    <row r="30" spans="1:16">
+      <c r="I29" s="112" t="s">
+        <v>3485</v>
+      </c>
+      <c r="J29" s="112" t="s">
+        <v>3486</v>
+      </c>
+      <c r="K29" s="112" t="s">
+        <v>3487</v>
+      </c>
+      <c r="N29" s="112" t="s">
+        <v>3484</v>
+      </c>
+      <c r="Q29">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17">
       <c r="A30" t="s">
         <v>2697</v>
       </c>
       <c r="B30" s="113" t="s">
-        <v>3575</v>
-      </c>
-      <c r="C30" t="s">
-        <v>3556</v>
+        <v>3539</v>
+      </c>
+      <c r="C30">
+        <v>16</v>
       </c>
       <c r="D30" t="s">
-        <v>3590</v>
+        <v>3555</v>
       </c>
       <c r="F30">
         <v>1</v>
@@ -39783,19 +39792,23 @@
       <c r="J30" s="112"/>
       <c r="K30" s="112"/>
       <c r="N30" s="112"/>
-    </row>
-    <row r="31" spans="1:16">
+      <c r="Q30">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17">
       <c r="A31" t="s">
         <v>2697</v>
       </c>
       <c r="B31" s="113" t="s">
-        <v>3579</v>
-      </c>
-      <c r="C31" t="s">
+        <v>3541</v>
+      </c>
+      <c r="C31">
+        <v>16</v>
+      </c>
+      <c r="D31" t="s">
         <v>3556</v>
-      </c>
-      <c r="D31" t="s">
-        <v>3591</v>
       </c>
       <c r="F31">
         <v>1</v>
@@ -39807,22 +39820,23 @@
       <c r="J31" s="112"/>
       <c r="K31" s="112"/>
       <c r="N31" s="112"/>
-    </row>
-    <row r="32" spans="1:16">
+      <c r="Q31">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17">
       <c r="A32" t="s">
-        <v>3606</v>
+        <v>2697</v>
       </c>
       <c r="B32" s="113" t="s">
-        <v>3572</v>
-      </c>
-      <c r="C32" t="s">
+        <v>3542</v>
+      </c>
+      <c r="C32">
+        <v>16</v>
+      </c>
+      <c r="D32" t="s">
         <v>3557</v>
-      </c>
-      <c r="D32" t="s">
-        <v>2735</v>
-      </c>
-      <c r="E32">
-        <v>0</v>
       </c>
       <c r="F32">
         <v>1</v>
@@ -39830,83 +39844,58 @@
       <c r="G32">
         <v>1</v>
       </c>
-      <c r="H32" t="s">
-        <v>3615</v>
-      </c>
-      <c r="I32" s="112" t="s">
-        <v>3507</v>
-      </c>
-      <c r="J32" s="112" t="s">
-        <v>3508</v>
-      </c>
-      <c r="K32" s="112" t="s">
-        <v>3509</v>
-      </c>
-      <c r="L32" s="112" t="s">
-        <v>3510</v>
-      </c>
-      <c r="M32" s="112" t="s">
-        <v>3511</v>
-      </c>
-      <c r="N32" s="112" t="s">
-        <v>3514</v>
-      </c>
-      <c r="O32" s="112" t="s">
-        <v>3512</v>
-      </c>
-      <c r="P32" s="112" t="s">
-        <v>3513</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16">
+      <c r="I32" s="112"/>
+      <c r="J32" s="112"/>
+      <c r="K32" s="112"/>
+      <c r="N32" s="112"/>
+      <c r="Q32">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17">
       <c r="A33" t="s">
-        <v>3606</v>
+        <v>2697</v>
       </c>
       <c r="B33" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C33" t="s">
-        <v>3557</v>
+        <v>3546</v>
+      </c>
+      <c r="C33">
+        <v>16</v>
       </c>
       <c r="D33" t="s">
-        <v>2735</v>
-      </c>
-      <c r="E33">
-        <v>3</v>
+        <v>3558</v>
       </c>
       <c r="F33">
         <v>1</v>
       </c>
       <c r="G33">
         <v>1</v>
-      </c>
-      <c r="H33" t="s">
-        <v>3612</v>
       </c>
       <c r="I33" s="112"/>
       <c r="J33" s="112"/>
       <c r="K33" s="112"/>
-      <c r="L33" s="112"/>
-      <c r="M33" s="112"/>
       <c r="N33" s="112"/>
-      <c r="O33" s="112"/>
-      <c r="P33" s="112"/>
-    </row>
-    <row r="34" spans="1:16">
+      <c r="Q33">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17">
       <c r="A34" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B34" s="113" t="s">
-        <v>3575</v>
-      </c>
-      <c r="C34" t="s">
-        <v>3557</v>
+        <v>3539</v>
+      </c>
+      <c r="C34">
+        <v>17</v>
       </c>
       <c r="D34" t="s">
         <v>2735</v>
       </c>
       <c r="E34">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F34">
         <v>1</v>
@@ -39915,32 +39904,52 @@
         <v>1</v>
       </c>
       <c r="H34" t="s">
-        <v>3611</v>
-      </c>
-      <c r="I34" s="112"/>
-      <c r="J34" s="112"/>
-      <c r="K34" s="112"/>
-      <c r="L34" s="112"/>
-      <c r="M34" s="112"/>
-      <c r="N34" s="112"/>
-      <c r="O34" s="112"/>
-      <c r="P34" s="112"/>
-    </row>
-    <row r="35" spans="1:16">
+        <v>3582</v>
+      </c>
+      <c r="I34" s="112" t="s">
+        <v>3507</v>
+      </c>
+      <c r="J34" s="112" t="s">
+        <v>3508</v>
+      </c>
+      <c r="K34" s="112" t="s">
+        <v>3509</v>
+      </c>
+      <c r="L34" s="112" t="s">
+        <v>3510</v>
+      </c>
+      <c r="M34" s="112" t="s">
+        <v>3511</v>
+      </c>
+      <c r="N34" s="112" t="s">
+        <v>3514</v>
+      </c>
+      <c r="O34" s="112" t="s">
+        <v>3512</v>
+      </c>
+      <c r="P34" s="112" t="s">
+        <v>3513</v>
+      </c>
+      <c r="Q34">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17">
       <c r="A35" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B35" s="113" t="s">
-        <v>3573</v>
-      </c>
-      <c r="C35" t="s">
-        <v>3557</v>
+        <v>3541</v>
+      </c>
+      <c r="C35">
+        <v>17</v>
       </c>
       <c r="D35" t="s">
         <v>2735</v>
       </c>
       <c r="E35">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F35">
         <v>1</v>
@@ -39949,7 +39958,7 @@
         <v>1</v>
       </c>
       <c r="H35" t="s">
-        <v>3621</v>
+        <v>3579</v>
       </c>
       <c r="I35" s="112"/>
       <c r="J35" s="112"/>
@@ -39959,22 +39968,26 @@
       <c r="N35" s="112"/>
       <c r="O35" s="112"/>
       <c r="P35" s="112"/>
-    </row>
-    <row r="36" spans="1:16">
+      <c r="Q35">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17">
       <c r="A36" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B36" s="113" t="s">
-        <v>3577</v>
-      </c>
-      <c r="C36" t="s">
-        <v>3557</v>
+        <v>3542</v>
+      </c>
+      <c r="C36">
+        <v>17</v>
       </c>
       <c r="D36" t="s">
         <v>2735</v>
       </c>
       <c r="E36">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F36">
         <v>1</v>
@@ -39983,7 +39996,7 @@
         <v>1</v>
       </c>
       <c r="H36" t="s">
-        <v>3622</v>
+        <v>3578</v>
       </c>
       <c r="I36" s="112"/>
       <c r="J36" s="112"/>
@@ -39993,22 +40006,26 @@
       <c r="N36" s="112"/>
       <c r="O36" s="112"/>
       <c r="P36" s="112"/>
-    </row>
-    <row r="37" spans="1:16">
+      <c r="Q36">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17">
       <c r="A37" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B37" s="113" t="s">
-        <v>3578</v>
-      </c>
-      <c r="C37" t="s">
-        <v>3557</v>
+        <v>3540</v>
+      </c>
+      <c r="C37">
+        <v>17</v>
       </c>
       <c r="D37" t="s">
         <v>2735</v>
       </c>
       <c r="E37">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F37">
         <v>1</v>
@@ -40017,7 +40034,7 @@
         <v>1</v>
       </c>
       <c r="H37" t="s">
-        <v>3620</v>
+        <v>3588</v>
       </c>
       <c r="I37" s="112"/>
       <c r="J37" s="112"/>
@@ -40027,22 +40044,26 @@
       <c r="N37" s="112"/>
       <c r="O37" s="112"/>
       <c r="P37" s="112"/>
-    </row>
-    <row r="38" spans="1:16">
+      <c r="Q37">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17">
       <c r="A38" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B38" s="113" t="s">
-        <v>3579</v>
-      </c>
-      <c r="C38" t="s">
-        <v>3557</v>
+        <v>3544</v>
+      </c>
+      <c r="C38">
+        <v>17</v>
       </c>
       <c r="D38" t="s">
         <v>2735</v>
       </c>
       <c r="E38">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F38">
         <v>1</v>
@@ -40051,7 +40072,7 @@
         <v>1</v>
       </c>
       <c r="H38" t="s">
-        <v>3629</v>
+        <v>3589</v>
       </c>
       <c r="I38" s="112"/>
       <c r="J38" s="112"/>
@@ -40061,22 +40082,26 @@
       <c r="N38" s="112"/>
       <c r="O38" s="112"/>
       <c r="P38" s="112"/>
-    </row>
-    <row r="39" spans="1:16">
+      <c r="Q38">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17">
       <c r="A39" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B39" s="113" t="s">
-        <v>3580</v>
-      </c>
-      <c r="C39" t="s">
-        <v>3557</v>
+        <v>3545</v>
+      </c>
+      <c r="C39">
+        <v>17</v>
       </c>
       <c r="D39" t="s">
         <v>2735</v>
       </c>
       <c r="E39">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F39">
         <v>1</v>
@@ -40085,7 +40110,7 @@
         <v>1</v>
       </c>
       <c r="H39" t="s">
-        <v>3632</v>
+        <v>3587</v>
       </c>
       <c r="I39" s="112"/>
       <c r="J39" s="112"/>
@@ -40095,22 +40120,26 @@
       <c r="N39" s="112"/>
       <c r="O39" s="112"/>
       <c r="P39" s="112"/>
-    </row>
-    <row r="40" spans="1:16">
+      <c r="Q39">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17">
       <c r="A40" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B40" s="113" t="s">
-        <v>3572</v>
-      </c>
-      <c r="C40" t="s">
-        <v>3558</v>
+        <v>3546</v>
+      </c>
+      <c r="C40">
+        <v>17</v>
       </c>
       <c r="D40" t="s">
         <v>2735</v>
       </c>
       <c r="E40">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="F40">
         <v>1</v>
@@ -40119,48 +40148,36 @@
         <v>1</v>
       </c>
       <c r="H40" t="s">
-        <v>3616</v>
-      </c>
-      <c r="I40" s="112" t="s">
-        <v>3515</v>
-      </c>
-      <c r="J40" s="112" t="s">
-        <v>3516</v>
-      </c>
-      <c r="K40" s="112" t="s">
-        <v>3517</v>
-      </c>
-      <c r="L40" s="112" t="s">
-        <v>3518</v>
-      </c>
-      <c r="M40" s="112" t="s">
-        <v>3519</v>
-      </c>
-      <c r="N40" s="112" t="s">
-        <v>3522</v>
-      </c>
-      <c r="O40" s="112" t="s">
-        <v>3520</v>
-      </c>
-      <c r="P40" s="112" t="s">
-        <v>3521</v>
-      </c>
-    </row>
-    <row r="41" spans="1:16">
+        <v>3596</v>
+      </c>
+      <c r="I40" s="112"/>
+      <c r="J40" s="112"/>
+      <c r="K40" s="112"/>
+      <c r="L40" s="112"/>
+      <c r="M40" s="112"/>
+      <c r="N40" s="112"/>
+      <c r="O40" s="112"/>
+      <c r="P40" s="112"/>
+      <c r="Q40">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17">
       <c r="A41" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B41" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C41" t="s">
-        <v>3558</v>
+        <v>3547</v>
+      </c>
+      <c r="C41">
+        <v>17</v>
       </c>
       <c r="D41" t="s">
         <v>2735</v>
       </c>
       <c r="E41">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -40169,7 +40186,7 @@
         <v>1</v>
       </c>
       <c r="H41" t="s">
-        <v>3613</v>
+        <v>3599</v>
       </c>
       <c r="I41" s="112"/>
       <c r="J41" s="112"/>
@@ -40179,22 +40196,26 @@
       <c r="N41" s="112"/>
       <c r="O41" s="112"/>
       <c r="P41" s="112"/>
-    </row>
-    <row r="42" spans="1:16">
+      <c r="Q41">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17">
       <c r="A42" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B42" s="113" t="s">
-        <v>3575</v>
-      </c>
-      <c r="C42" t="s">
-        <v>3558</v>
+        <v>3539</v>
+      </c>
+      <c r="C42">
+        <v>18</v>
       </c>
       <c r="D42" t="s">
         <v>2735</v>
       </c>
       <c r="E42">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F42">
         <v>1</v>
@@ -40203,32 +40224,52 @@
         <v>1</v>
       </c>
       <c r="H42" t="s">
-        <v>3618</v>
-      </c>
-      <c r="I42" s="112"/>
-      <c r="J42" s="112"/>
-      <c r="K42" s="112"/>
-      <c r="L42" s="112"/>
-      <c r="M42" s="112"/>
-      <c r="N42" s="112"/>
-      <c r="O42" s="112"/>
-      <c r="P42" s="112"/>
-    </row>
-    <row r="43" spans="1:16">
+        <v>3583</v>
+      </c>
+      <c r="I42" s="112" t="s">
+        <v>3515</v>
+      </c>
+      <c r="J42" s="112" t="s">
+        <v>3516</v>
+      </c>
+      <c r="K42" s="112" t="s">
+        <v>3517</v>
+      </c>
+      <c r="L42" s="112" t="s">
+        <v>3518</v>
+      </c>
+      <c r="M42" s="112" t="s">
+        <v>3519</v>
+      </c>
+      <c r="N42" s="112" t="s">
+        <v>3522</v>
+      </c>
+      <c r="O42" s="112" t="s">
+        <v>3520</v>
+      </c>
+      <c r="P42" s="112" t="s">
+        <v>3521</v>
+      </c>
+      <c r="Q42">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17">
       <c r="A43" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B43" s="113" t="s">
-        <v>3573</v>
-      </c>
-      <c r="C43" t="s">
-        <v>3558</v>
+        <v>3541</v>
+      </c>
+      <c r="C43">
+        <v>18</v>
       </c>
       <c r="D43" t="s">
         <v>2735</v>
       </c>
       <c r="E43">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -40237,7 +40278,7 @@
         <v>1</v>
       </c>
       <c r="H43" t="s">
-        <v>3623</v>
+        <v>3580</v>
       </c>
       <c r="I43" s="112"/>
       <c r="J43" s="112"/>
@@ -40247,22 +40288,26 @@
       <c r="N43" s="112"/>
       <c r="O43" s="112"/>
       <c r="P43" s="112"/>
-    </row>
-    <row r="44" spans="1:16">
+      <c r="Q43">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17">
       <c r="A44" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B44" s="113" t="s">
-        <v>3577</v>
-      </c>
-      <c r="C44" t="s">
-        <v>3558</v>
+        <v>3542</v>
+      </c>
+      <c r="C44">
+        <v>18</v>
       </c>
       <c r="D44" t="s">
         <v>2735</v>
       </c>
       <c r="E44">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F44">
         <v>1</v>
@@ -40271,7 +40316,7 @@
         <v>1</v>
       </c>
       <c r="H44" t="s">
-        <v>3625</v>
+        <v>3585</v>
       </c>
       <c r="I44" s="112"/>
       <c r="J44" s="112"/>
@@ -40281,22 +40326,26 @@
       <c r="N44" s="112"/>
       <c r="O44" s="112"/>
       <c r="P44" s="112"/>
-    </row>
-    <row r="45" spans="1:16">
+      <c r="Q44">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17">
       <c r="A45" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B45" s="113" t="s">
-        <v>3578</v>
-      </c>
-      <c r="C45" t="s">
-        <v>3558</v>
+        <v>3540</v>
+      </c>
+      <c r="C45">
+        <v>18</v>
       </c>
       <c r="D45" t="s">
         <v>2735</v>
       </c>
       <c r="E45">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F45">
         <v>1</v>
@@ -40305,7 +40354,7 @@
         <v>1</v>
       </c>
       <c r="H45" t="s">
-        <v>3627</v>
+        <v>3590</v>
       </c>
       <c r="I45" s="112"/>
       <c r="J45" s="112"/>
@@ -40315,22 +40364,26 @@
       <c r="N45" s="112"/>
       <c r="O45" s="112"/>
       <c r="P45" s="112"/>
-    </row>
-    <row r="46" spans="1:16">
+      <c r="Q45">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17">
       <c r="A46" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B46" s="113" t="s">
-        <v>3579</v>
-      </c>
-      <c r="C46" t="s">
-        <v>3558</v>
+        <v>3544</v>
+      </c>
+      <c r="C46">
+        <v>18</v>
       </c>
       <c r="D46" t="s">
         <v>2735</v>
       </c>
       <c r="E46">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F46">
         <v>1</v>
@@ -40339,7 +40392,7 @@
         <v>1</v>
       </c>
       <c r="H46" t="s">
-        <v>3630</v>
+        <v>3592</v>
       </c>
       <c r="I46" s="112"/>
       <c r="J46" s="112"/>
@@ -40349,22 +40402,26 @@
       <c r="N46" s="112"/>
       <c r="O46" s="112"/>
       <c r="P46" s="112"/>
-    </row>
-    <row r="47" spans="1:16">
+      <c r="Q46">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17">
       <c r="A47" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B47" s="113" t="s">
-        <v>3580</v>
-      </c>
-      <c r="C47" t="s">
-        <v>3558</v>
+        <v>3545</v>
+      </c>
+      <c r="C47">
+        <v>18</v>
       </c>
       <c r="D47" t="s">
         <v>2735</v>
       </c>
       <c r="E47">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F47">
         <v>1</v>
@@ -40373,7 +40430,7 @@
         <v>1</v>
       </c>
       <c r="H47" t="s">
-        <v>3633</v>
+        <v>3594</v>
       </c>
       <c r="I47" s="112"/>
       <c r="J47" s="112"/>
@@ -40383,22 +40440,26 @@
       <c r="N47" s="112"/>
       <c r="O47" s="112"/>
       <c r="P47" s="112"/>
-    </row>
-    <row r="48" spans="1:16">
+      <c r="Q47">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17">
       <c r="A48" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B48" s="113" t="s">
-        <v>3572</v>
-      </c>
-      <c r="C48" t="s">
-        <v>3559</v>
+        <v>3546</v>
+      </c>
+      <c r="C48">
+        <v>18</v>
       </c>
       <c r="D48" t="s">
         <v>2735</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="F48">
         <v>1</v>
@@ -40407,48 +40468,36 @@
         <v>1</v>
       </c>
       <c r="H48" t="s">
-        <v>3617</v>
-      </c>
-      <c r="I48" s="112" t="s">
-        <v>3523</v>
-      </c>
-      <c r="J48" s="112" t="s">
-        <v>3524</v>
-      </c>
-      <c r="K48" s="112" t="s">
-        <v>3525</v>
-      </c>
-      <c r="L48" s="112" t="s">
-        <v>3526</v>
-      </c>
-      <c r="M48" s="112" t="s">
-        <v>3527</v>
-      </c>
-      <c r="N48" s="112" t="s">
-        <v>3530</v>
-      </c>
-      <c r="O48" s="112" t="s">
-        <v>3528</v>
-      </c>
-      <c r="P48" s="112" t="s">
-        <v>3529</v>
-      </c>
-    </row>
-    <row r="49" spans="1:16">
+        <v>3597</v>
+      </c>
+      <c r="I48" s="112"/>
+      <c r="J48" s="112"/>
+      <c r="K48" s="112"/>
+      <c r="L48" s="112"/>
+      <c r="M48" s="112"/>
+      <c r="N48" s="112"/>
+      <c r="O48" s="112"/>
+      <c r="P48" s="112"/>
+      <c r="Q48">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17">
       <c r="A49" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B49" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C49" t="s">
-        <v>3559</v>
+        <v>3547</v>
+      </c>
+      <c r="C49">
+        <v>18</v>
       </c>
       <c r="D49" t="s">
         <v>2735</v>
       </c>
       <c r="E49">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="F49">
         <v>1</v>
@@ -40457,7 +40506,7 @@
         <v>1</v>
       </c>
       <c r="H49" t="s">
-        <v>3614</v>
+        <v>3600</v>
       </c>
       <c r="I49" s="112"/>
       <c r="J49" s="112"/>
@@ -40467,22 +40516,26 @@
       <c r="N49" s="112"/>
       <c r="O49" s="112"/>
       <c r="P49" s="112"/>
-    </row>
-    <row r="50" spans="1:16">
+      <c r="Q49">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17">
       <c r="A50" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B50" s="113" t="s">
-        <v>3575</v>
-      </c>
-      <c r="C50" t="s">
-        <v>3559</v>
+        <v>3539</v>
+      </c>
+      <c r="C50">
+        <v>19</v>
       </c>
       <c r="D50" t="s">
         <v>2735</v>
       </c>
       <c r="E50">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F50">
         <v>1</v>
@@ -40491,32 +40544,52 @@
         <v>1</v>
       </c>
       <c r="H50" t="s">
-        <v>3619</v>
-      </c>
-      <c r="I50" s="112"/>
-      <c r="J50" s="112"/>
-      <c r="K50" s="112"/>
-      <c r="L50" s="112"/>
-      <c r="M50" s="112"/>
-      <c r="N50" s="112"/>
-      <c r="O50" s="112"/>
-      <c r="P50" s="112"/>
-    </row>
-    <row r="51" spans="1:16">
+        <v>3584</v>
+      </c>
+      <c r="I50" s="112" t="s">
+        <v>3523</v>
+      </c>
+      <c r="J50" s="112" t="s">
+        <v>3524</v>
+      </c>
+      <c r="K50" s="112" t="s">
+        <v>3525</v>
+      </c>
+      <c r="L50" s="112" t="s">
+        <v>3526</v>
+      </c>
+      <c r="M50" s="112" t="s">
+        <v>3527</v>
+      </c>
+      <c r="N50" s="112" t="s">
+        <v>3530</v>
+      </c>
+      <c r="O50" s="112" t="s">
+        <v>3528</v>
+      </c>
+      <c r="P50" s="112" t="s">
+        <v>3529</v>
+      </c>
+      <c r="Q50">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17">
       <c r="A51" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B51" s="113" t="s">
-        <v>3573</v>
-      </c>
-      <c r="C51" t="s">
-        <v>3559</v>
+        <v>3541</v>
+      </c>
+      <c r="C51">
+        <v>19</v>
       </c>
       <c r="D51" t="s">
         <v>2735</v>
       </c>
       <c r="E51">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F51">
         <v>1</v>
@@ -40525,7 +40598,7 @@
         <v>1</v>
       </c>
       <c r="H51" t="s">
-        <v>3624</v>
+        <v>3581</v>
       </c>
       <c r="I51" s="112"/>
       <c r="J51" s="112"/>
@@ -40535,22 +40608,26 @@
       <c r="N51" s="112"/>
       <c r="O51" s="112"/>
       <c r="P51" s="112"/>
-    </row>
-    <row r="52" spans="1:16">
+      <c r="Q51">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17">
       <c r="A52" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B52" s="113" t="s">
-        <v>3577</v>
-      </c>
-      <c r="C52" t="s">
-        <v>3559</v>
+        <v>3542</v>
+      </c>
+      <c r="C52">
+        <v>19</v>
       </c>
       <c r="D52" t="s">
         <v>2735</v>
       </c>
       <c r="E52">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F52">
         <v>1</v>
@@ -40559,7 +40636,7 @@
         <v>1</v>
       </c>
       <c r="H52" t="s">
-        <v>3626</v>
+        <v>3586</v>
       </c>
       <c r="I52" s="112"/>
       <c r="J52" s="112"/>
@@ -40569,22 +40646,26 @@
       <c r="N52" s="112"/>
       <c r="O52" s="112"/>
       <c r="P52" s="112"/>
-    </row>
-    <row r="53" spans="1:16">
+      <c r="Q52">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17">
       <c r="A53" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B53" s="113" t="s">
-        <v>3578</v>
-      </c>
-      <c r="C53" t="s">
-        <v>3559</v>
+        <v>3540</v>
+      </c>
+      <c r="C53">
+        <v>19</v>
       </c>
       <c r="D53" t="s">
         <v>2735</v>
       </c>
       <c r="E53">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F53">
         <v>1</v>
@@ -40593,7 +40674,7 @@
         <v>1</v>
       </c>
       <c r="H53" t="s">
-        <v>3628</v>
+        <v>3591</v>
       </c>
       <c r="I53" s="112"/>
       <c r="J53" s="112"/>
@@ -40603,22 +40684,26 @@
       <c r="N53" s="112"/>
       <c r="O53" s="112"/>
       <c r="P53" s="112"/>
-    </row>
-    <row r="54" spans="1:16">
+      <c r="Q53">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17">
       <c r="A54" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B54" s="113" t="s">
-        <v>3579</v>
-      </c>
-      <c r="C54" t="s">
-        <v>3559</v>
+        <v>3544</v>
+      </c>
+      <c r="C54">
+        <v>19</v>
       </c>
       <c r="D54" t="s">
         <v>2735</v>
       </c>
       <c r="E54">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F54">
         <v>1</v>
@@ -40627,7 +40712,7 @@
         <v>1</v>
       </c>
       <c r="H54" t="s">
-        <v>3631</v>
+        <v>3593</v>
       </c>
       <c r="I54" s="112"/>
       <c r="J54" s="112"/>
@@ -40637,22 +40722,26 @@
       <c r="N54" s="112"/>
       <c r="O54" s="112"/>
       <c r="P54" s="112"/>
-    </row>
-    <row r="55" spans="1:16">
+      <c r="Q54">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17">
       <c r="A55" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B55" s="113" t="s">
-        <v>3580</v>
-      </c>
-      <c r="C55" t="s">
-        <v>3559</v>
+        <v>3545</v>
+      </c>
+      <c r="C55">
+        <v>19</v>
       </c>
       <c r="D55" t="s">
         <v>2735</v>
       </c>
       <c r="E55">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F55">
         <v>1</v>
@@ -40661,7 +40750,7 @@
         <v>1</v>
       </c>
       <c r="H55" t="s">
-        <v>3634</v>
+        <v>3595</v>
       </c>
       <c r="I55" s="112"/>
       <c r="J55" s="112"/>
@@ -40671,159 +40760,207 @@
       <c r="N55" s="112"/>
       <c r="O55" s="112"/>
       <c r="P55" s="112"/>
-    </row>
-    <row r="56" spans="1:16">
+      <c r="Q55">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17">
       <c r="A56" t="s">
-        <v>2696</v>
+        <v>3573</v>
       </c>
       <c r="B56" s="113" t="s">
-        <v>3578</v>
-      </c>
-      <c r="C56" t="s">
-        <v>3560</v>
+        <v>3546</v>
+      </c>
+      <c r="C56">
+        <v>19</v>
       </c>
       <c r="D56" t="s">
-        <v>2825</v>
+        <v>2735</v>
+      </c>
+      <c r="E56">
+        <v>20</v>
       </c>
       <c r="F56">
         <v>1</v>
       </c>
       <c r="G56">
-        <v>2</v>
-      </c>
-      <c r="I56" t="s">
-        <v>3505</v>
-      </c>
-      <c r="J56" t="s">
-        <v>3506</v>
-      </c>
-      <c r="N56" t="s">
-        <v>2825</v>
-      </c>
-      <c r="O56" t="s">
-        <v>2797</v>
-      </c>
-    </row>
-    <row r="57" spans="1:16">
+        <v>1</v>
+      </c>
+      <c r="H56" t="s">
+        <v>3598</v>
+      </c>
+      <c r="I56" s="112"/>
+      <c r="J56" s="112"/>
+      <c r="K56" s="112"/>
+      <c r="L56" s="112"/>
+      <c r="M56" s="112"/>
+      <c r="N56" s="112"/>
+      <c r="O56" s="112"/>
+      <c r="P56" s="112"/>
+      <c r="Q56">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17">
       <c r="A57" t="s">
-        <v>2696</v>
+        <v>3573</v>
       </c>
       <c r="B57" s="113" t="s">
-        <v>3572</v>
-      </c>
-      <c r="C57" t="s">
-        <v>3560</v>
+        <v>3547</v>
+      </c>
+      <c r="C57">
+        <v>19</v>
       </c>
       <c r="D57" t="s">
-        <v>3505</v>
+        <v>2735</v>
+      </c>
+      <c r="E57">
+        <v>23</v>
       </c>
       <c r="F57">
         <v>1</v>
       </c>
       <c r="G57">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="58" spans="1:16">
+        <v>1</v>
+      </c>
+      <c r="H57" t="s">
+        <v>3601</v>
+      </c>
+      <c r="I57" s="112"/>
+      <c r="J57" s="112"/>
+      <c r="K57" s="112"/>
+      <c r="L57" s="112"/>
+      <c r="M57" s="112"/>
+      <c r="N57" s="112"/>
+      <c r="O57" s="112"/>
+      <c r="P57" s="112"/>
+      <c r="Q57">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17">
       <c r="A58" t="s">
         <v>2696</v>
       </c>
       <c r="B58" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C58" t="s">
-        <v>3560</v>
+        <v>3545</v>
+      </c>
+      <c r="C58">
+        <v>20</v>
       </c>
       <c r="D58" t="s">
+        <v>2825</v>
+      </c>
+      <c r="F58">
+        <v>5</v>
+      </c>
+      <c r="G58">
+        <v>10</v>
+      </c>
+      <c r="I58" t="s">
+        <v>3505</v>
+      </c>
+      <c r="J58" t="s">
         <v>3506</v>
       </c>
-      <c r="F58">
-        <v>1</v>
-      </c>
-      <c r="G58">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="59" spans="1:16">
+      <c r="N58" t="s">
+        <v>2825</v>
+      </c>
+      <c r="O58" t="s">
+        <v>2797</v>
+      </c>
+      <c r="Q58">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17">
       <c r="A59" t="s">
         <v>2696</v>
       </c>
       <c r="B59" s="113" t="s">
-        <v>3579</v>
-      </c>
-      <c r="C59" t="s">
-        <v>3560</v>
+        <v>3539</v>
+      </c>
+      <c r="C59">
+        <v>20</v>
       </c>
       <c r="D59" t="s">
+        <v>3505</v>
+      </c>
+      <c r="F59">
+        <v>5</v>
+      </c>
+      <c r="G59">
+        <v>10</v>
+      </c>
+      <c r="Q59">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17">
+      <c r="A60" t="s">
+        <v>2696</v>
+      </c>
+      <c r="B60" s="113" t="s">
+        <v>3541</v>
+      </c>
+      <c r="C60">
+        <v>20</v>
+      </c>
+      <c r="D60" t="s">
+        <v>3506</v>
+      </c>
+      <c r="F60">
+        <v>5</v>
+      </c>
+      <c r="G60">
+        <v>10</v>
+      </c>
+      <c r="Q60">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17">
+      <c r="A61" t="s">
+        <v>2696</v>
+      </c>
+      <c r="B61" s="113" t="s">
+        <v>3546</v>
+      </c>
+      <c r="C61">
+        <v>20</v>
+      </c>
+      <c r="D61" t="s">
         <v>2797</v>
       </c>
-      <c r="F59">
-        <v>1</v>
-      </c>
-      <c r="G59">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="60" spans="1:16">
-      <c r="A60" t="s">
-        <v>2746</v>
-      </c>
-      <c r="B60" s="113" t="s">
-        <v>3572</v>
-      </c>
-      <c r="C60" t="s">
-        <v>3561</v>
-      </c>
-      <c r="D60" t="s">
-        <v>2844</v>
-      </c>
-      <c r="F60">
-        <v>1</v>
-      </c>
-      <c r="G60">
-        <v>3</v>
-      </c>
-      <c r="I60" s="112" t="s">
-        <v>3488</v>
-      </c>
-      <c r="J60" s="112" t="s">
-        <v>3489</v>
-      </c>
-    </row>
-    <row r="61" spans="1:16">
-      <c r="A61" t="s">
-        <v>2746</v>
-      </c>
-      <c r="B61" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C61" t="s">
-        <v>3561</v>
-      </c>
-      <c r="D61" t="s">
-        <v>3593</v>
-      </c>
       <c r="F61">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G61">
-        <v>3</v>
-      </c>
-      <c r="I61" s="112"/>
-      <c r="J61" s="112"/>
-    </row>
-    <row r="62" spans="1:16">
+        <v>10</v>
+      </c>
+      <c r="Q61">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17">
       <c r="A62" t="s">
-        <v>2746</v>
+        <v>2696</v>
       </c>
       <c r="B62" s="113" t="s">
-        <v>3573</v>
-      </c>
-      <c r="C62" t="s">
-        <v>3562</v>
+        <v>3540</v>
+      </c>
+      <c r="C62">
+        <v>20</v>
       </c>
       <c r="D62" t="s">
-        <v>2874</v>
+        <v>2778</v>
       </c>
       <c r="F62">
         <v>5</v>
@@ -40831,112 +40968,106 @@
       <c r="G62">
         <v>10</v>
       </c>
-      <c r="L62" t="s">
-        <v>2874</v>
-      </c>
-    </row>
-    <row r="63" spans="1:16">
+      <c r="Q62">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17">
       <c r="A63" t="s">
         <v>2746</v>
       </c>
       <c r="B63" s="113" t="s">
-        <v>3578</v>
-      </c>
-      <c r="C63" t="s">
-        <v>3563</v>
+        <v>3539</v>
+      </c>
+      <c r="C63">
+        <v>21</v>
       </c>
       <c r="D63" t="s">
-        <v>2740</v>
+        <v>2844</v>
       </c>
       <c r="F63">
         <v>1</v>
       </c>
       <c r="G63">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I63" s="112" t="s">
-        <v>3473</v>
+        <v>3488</v>
       </c>
       <c r="J63" s="112" t="s">
-        <v>3474</v>
-      </c>
-      <c r="K63" s="112" t="s">
-        <v>3475</v>
-      </c>
-      <c r="L63" s="112" t="s">
-        <v>3477</v>
-      </c>
-      <c r="N63" s="112" t="s">
-        <v>2740</v>
-      </c>
-      <c r="O63" s="112" t="s">
-        <v>3476</v>
-      </c>
-    </row>
-    <row r="64" spans="1:16">
+        <v>3489</v>
+      </c>
+      <c r="Q63">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="64" spans="1:17">
       <c r="A64" t="s">
         <v>2746</v>
       </c>
       <c r="B64" s="113" t="s">
-        <v>3572</v>
-      </c>
-      <c r="C64" t="s">
-        <v>3563</v>
+        <v>3541</v>
+      </c>
+      <c r="C64">
+        <v>21</v>
       </c>
       <c r="D64" t="s">
-        <v>2739</v>
+        <v>3560</v>
       </c>
       <c r="F64">
         <v>1</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I64" s="112"/>
       <c r="J64" s="112"/>
-      <c r="K64" s="112"/>
-      <c r="L64" s="112"/>
-      <c r="N64" s="112"/>
-      <c r="O64" s="112"/>
-    </row>
-    <row r="65" spans="1:16">
+      <c r="Q64">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="65" spans="1:17">
       <c r="A65" t="s">
         <v>2746</v>
       </c>
       <c r="B65" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C65" t="s">
-        <v>3563</v>
+        <v>3540</v>
+      </c>
+      <c r="C65">
+        <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>3594</v>
+        <v>2874</v>
       </c>
       <c r="F65">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G65">
-        <v>2</v>
-      </c>
-      <c r="I65" s="112"/>
-      <c r="J65" s="112"/>
-      <c r="K65" s="112"/>
-      <c r="L65" s="112"/>
-      <c r="N65" s="112"/>
-      <c r="O65" s="112"/>
-    </row>
-    <row r="66" spans="1:16">
+        <v>20</v>
+      </c>
+      <c r="L65" t="s">
+        <v>2874</v>
+      </c>
+      <c r="Q65">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="66" spans="1:17">
       <c r="A66" t="s">
         <v>2746</v>
       </c>
       <c r="B66" s="113" t="s">
-        <v>3575</v>
-      </c>
-      <c r="C66" t="s">
-        <v>3563</v>
+        <v>3545</v>
+      </c>
+      <c r="C66">
+        <v>23</v>
       </c>
       <c r="D66" t="s">
-        <v>2916</v>
+        <v>2740</v>
       </c>
       <c r="F66">
         <v>1</v>
@@ -40944,25 +41075,41 @@
       <c r="G66">
         <v>2</v>
       </c>
-      <c r="I66" s="112"/>
-      <c r="J66" s="112"/>
-      <c r="K66" s="112"/>
-      <c r="L66" s="112"/>
-      <c r="N66" s="112"/>
-      <c r="O66" s="112"/>
-    </row>
-    <row r="67" spans="1:16">
+      <c r="I66" s="112" t="s">
+        <v>3473</v>
+      </c>
+      <c r="J66" s="112" t="s">
+        <v>3474</v>
+      </c>
+      <c r="K66" s="112" t="s">
+        <v>3475</v>
+      </c>
+      <c r="L66" s="112" t="s">
+        <v>3477</v>
+      </c>
+      <c r="N66" s="112" t="s">
+        <v>2740</v>
+      </c>
+      <c r="O66" s="112" t="s">
+        <v>3476</v>
+      </c>
+      <c r="Q66">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="67" spans="1:17">
       <c r="A67" t="s">
         <v>2746</v>
       </c>
       <c r="B67" s="113" t="s">
-        <v>3579</v>
-      </c>
-      <c r="C67" t="s">
-        <v>3563</v>
+        <v>3539</v>
+      </c>
+      <c r="C67">
+        <v>23</v>
       </c>
       <c r="D67" t="s">
-        <v>3595</v>
+        <v>2739</v>
       </c>
       <c r="F67">
         <v>1</v>
@@ -40976,25 +41123,29 @@
       <c r="L67" s="112"/>
       <c r="N67" s="112"/>
       <c r="O67" s="112"/>
-    </row>
-    <row r="68" spans="1:16">
+      <c r="Q67">
+        <f t="shared" ref="Q67:Q96" si="1">C67-1</f>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="68" spans="1:17">
       <c r="A68" t="s">
         <v>2746</v>
       </c>
       <c r="B68" s="113" t="s">
-        <v>3573</v>
-      </c>
-      <c r="C68" t="s">
-        <v>3563</v>
+        <v>3541</v>
+      </c>
+      <c r="C68">
+        <v>23</v>
       </c>
       <c r="D68" t="s">
-        <v>2741</v>
+        <v>3561</v>
       </c>
       <c r="F68">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G68">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="I68" s="112"/>
       <c r="J68" s="112"/>
@@ -41002,114 +41153,113 @@
       <c r="L68" s="112"/>
       <c r="N68" s="112"/>
       <c r="O68" s="112"/>
-    </row>
-    <row r="69" spans="1:16">
+      <c r="Q68">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="69" spans="1:17">
       <c r="A69" t="s">
-        <v>3607</v>
+        <v>2746</v>
       </c>
       <c r="B69" s="113" t="s">
-        <v>3572</v>
-      </c>
-      <c r="C69" t="s">
-        <v>3564</v>
+        <v>3542</v>
+      </c>
+      <c r="C69">
+        <v>23</v>
       </c>
       <c r="D69" t="s">
-        <v>3596</v>
+        <v>2916</v>
       </c>
       <c r="F69">
         <v>1</v>
       </c>
       <c r="G69">
-        <v>5</v>
-      </c>
-      <c r="I69" s="112" t="s">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="70" spans="1:16">
+        <v>2</v>
+      </c>
+      <c r="I69" s="112"/>
+      <c r="J69" s="112"/>
+      <c r="K69" s="112"/>
+      <c r="L69" s="112"/>
+      <c r="N69" s="112"/>
+      <c r="O69" s="112"/>
+      <c r="Q69">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="70" spans="1:17">
       <c r="A70" t="s">
-        <v>3606</v>
+        <v>2746</v>
       </c>
       <c r="B70" s="113" t="s">
-        <v>3572</v>
-      </c>
-      <c r="C70" t="s">
-        <v>3565</v>
+        <v>3546</v>
+      </c>
+      <c r="C70">
+        <v>23</v>
       </c>
       <c r="D70" t="s">
-        <v>1003</v>
+        <v>3562</v>
       </c>
       <c r="F70">
         <v>1</v>
       </c>
       <c r="G70">
-        <v>1</v>
-      </c>
-      <c r="I70" s="112" t="s">
-        <v>3531</v>
-      </c>
-      <c r="J70" s="112" t="s">
-        <v>3532</v>
-      </c>
-      <c r="K70" s="112" t="s">
-        <v>3533</v>
-      </c>
-      <c r="L70" s="112" t="s">
-        <v>3534</v>
-      </c>
-      <c r="M70" s="112" t="s">
-        <v>3535</v>
-      </c>
-      <c r="N70" s="112" t="s">
-        <v>3538</v>
-      </c>
-      <c r="O70" s="112" t="s">
-        <v>3536</v>
-      </c>
-      <c r="P70" s="112" t="s">
-        <v>3537</v>
-      </c>
-    </row>
-    <row r="71" spans="1:16">
+        <v>2</v>
+      </c>
+      <c r="I70" s="112"/>
+      <c r="J70" s="112"/>
+      <c r="K70" s="112"/>
+      <c r="L70" s="112"/>
+      <c r="N70" s="112"/>
+      <c r="O70" s="112"/>
+      <c r="Q70">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="71" spans="1:17">
       <c r="A71" t="s">
-        <v>3606</v>
+        <v>2746</v>
       </c>
       <c r="B71" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C71" t="s">
-        <v>3565</v>
+        <v>3540</v>
+      </c>
+      <c r="C71">
+        <v>23</v>
       </c>
       <c r="D71" t="s">
-        <v>2847</v>
+        <v>2741</v>
       </c>
       <c r="F71">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G71">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="I71" s="112"/>
       <c r="J71" s="112"/>
       <c r="K71" s="112"/>
       <c r="L71" s="112"/>
-      <c r="M71" s="112"/>
       <c r="N71" s="112"/>
       <c r="O71" s="112"/>
-      <c r="P71" s="112"/>
-    </row>
-    <row r="72" spans="1:16">
+      <c r="Q71">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="72" spans="1:17">
       <c r="A72" t="s">
-        <v>3606</v>
+        <v>2697</v>
       </c>
       <c r="B72" s="113" t="s">
-        <v>3575</v>
-      </c>
-      <c r="C72" t="s">
-        <v>3565</v>
+        <v>3545</v>
+      </c>
+      <c r="C72">
+        <v>24</v>
       </c>
       <c r="D72" t="s">
-        <v>1231</v>
+        <v>2730</v>
       </c>
       <c r="F72">
         <v>1</v>
@@ -41121,23 +41271,25 @@
       <c r="J72" s="112"/>
       <c r="K72" s="112"/>
       <c r="L72" s="112"/>
-      <c r="M72" s="112"/>
       <c r="N72" s="112"/>
       <c r="O72" s="112"/>
-      <c r="P72" s="112"/>
-    </row>
-    <row r="73" spans="1:16">
+      <c r="Q72">
+        <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="73" spans="1:17">
       <c r="A73" t="s">
-        <v>3606</v>
+        <v>2697</v>
       </c>
       <c r="B73" s="113" t="s">
-        <v>3573</v>
-      </c>
-      <c r="C73" t="s">
-        <v>3565</v>
+        <v>3539</v>
+      </c>
+      <c r="C73">
+        <v>24</v>
       </c>
       <c r="D73" t="s">
-        <v>2814</v>
+        <v>2728</v>
       </c>
       <c r="F73">
         <v>1</v>
@@ -41149,23 +41301,25 @@
       <c r="J73" s="112"/>
       <c r="K73" s="112"/>
       <c r="L73" s="112"/>
-      <c r="M73" s="112"/>
       <c r="N73" s="112"/>
       <c r="O73" s="112"/>
-      <c r="P73" s="112"/>
-    </row>
-    <row r="74" spans="1:16">
+      <c r="Q73">
+        <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="74" spans="1:17">
       <c r="A74" t="s">
-        <v>3606</v>
+        <v>2697</v>
       </c>
       <c r="B74" s="113" t="s">
-        <v>3577</v>
-      </c>
-      <c r="C74" t="s">
-        <v>3565</v>
+        <v>3541</v>
+      </c>
+      <c r="C74">
+        <v>24</v>
       </c>
       <c r="D74" t="s">
-        <v>208</v>
+        <v>2732</v>
       </c>
       <c r="F74">
         <v>1</v>
@@ -41177,23 +41331,25 @@
       <c r="J74" s="112"/>
       <c r="K74" s="112"/>
       <c r="L74" s="112"/>
-      <c r="M74" s="112"/>
       <c r="N74" s="112"/>
       <c r="O74" s="112"/>
-      <c r="P74" s="112"/>
-    </row>
-    <row r="75" spans="1:16">
+      <c r="Q74">
+        <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="75" spans="1:17">
       <c r="A75" t="s">
-        <v>3606</v>
+        <v>2697</v>
       </c>
       <c r="B75" s="113" t="s">
-        <v>3578</v>
-      </c>
-      <c r="C75" t="s">
-        <v>3565</v>
+        <v>3546</v>
+      </c>
+      <c r="C75">
+        <v>24</v>
       </c>
       <c r="D75" t="s">
-        <v>2808</v>
+        <v>3603</v>
       </c>
       <c r="F75">
         <v>1</v>
@@ -41205,51 +41361,52 @@
       <c r="J75" s="112"/>
       <c r="K75" s="112"/>
       <c r="L75" s="112"/>
-      <c r="M75" s="112"/>
       <c r="N75" s="112"/>
       <c r="O75" s="112"/>
-      <c r="P75" s="112"/>
-    </row>
-    <row r="76" spans="1:16">
+      <c r="Q75">
+        <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="76" spans="1:17">
       <c r="A76" t="s">
-        <v>3606</v>
+        <v>3574</v>
       </c>
       <c r="B76" s="113" t="s">
-        <v>3579</v>
-      </c>
-      <c r="C76" t="s">
-        <v>3565</v>
+        <v>3539</v>
+      </c>
+      <c r="C76">
+        <v>25</v>
       </c>
       <c r="D76" t="s">
-        <v>2708</v>
+        <v>3563</v>
       </c>
       <c r="F76">
         <v>1</v>
       </c>
       <c r="G76">
-        <v>1</v>
-      </c>
-      <c r="I76" s="112"/>
-      <c r="J76" s="112"/>
-      <c r="K76" s="112"/>
-      <c r="L76" s="112"/>
-      <c r="M76" s="112"/>
-      <c r="N76" s="112"/>
-      <c r="O76" s="112"/>
-      <c r="P76" s="112"/>
-    </row>
-    <row r="77" spans="1:16">
+        <v>5</v>
+      </c>
+      <c r="I76" s="112" t="s">
+        <v>3500</v>
+      </c>
+      <c r="Q76">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="77" spans="1:17">
       <c r="A77" t="s">
-        <v>3606</v>
+        <v>3573</v>
       </c>
       <c r="B77" s="113" t="s">
-        <v>3580</v>
-      </c>
-      <c r="C77" t="s">
-        <v>3565</v>
+        <v>3539</v>
+      </c>
+      <c r="C77">
+        <v>26</v>
       </c>
       <c r="D77" t="s">
-        <v>3597</v>
+        <v>1003</v>
       </c>
       <c r="F77">
         <v>1</v>
@@ -41257,27 +41414,47 @@
       <c r="G77">
         <v>1</v>
       </c>
-      <c r="I77" s="112"/>
-      <c r="J77" s="112"/>
-      <c r="K77" s="112"/>
-      <c r="L77" s="112"/>
-      <c r="M77" s="112"/>
-      <c r="N77" s="112"/>
-      <c r="O77" s="112"/>
-      <c r="P77" s="112"/>
-    </row>
-    <row r="78" spans="1:16">
+      <c r="I77" s="112" t="s">
+        <v>3531</v>
+      </c>
+      <c r="J77" s="112" t="s">
+        <v>3532</v>
+      </c>
+      <c r="K77" s="112" t="s">
+        <v>3533</v>
+      </c>
+      <c r="L77" s="112" t="s">
+        <v>3534</v>
+      </c>
+      <c r="M77" s="112" t="s">
+        <v>3535</v>
+      </c>
+      <c r="N77" s="112" t="s">
+        <v>3538</v>
+      </c>
+      <c r="O77" s="112" t="s">
+        <v>3536</v>
+      </c>
+      <c r="P77" s="112" t="s">
+        <v>3537</v>
+      </c>
+      <c r="Q77">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="78" spans="1:17">
       <c r="A78" t="s">
-        <v>3608</v>
+        <v>3573</v>
       </c>
       <c r="B78" s="113" t="s">
-        <v>3572</v>
-      </c>
-      <c r="C78" t="s">
-        <v>3566</v>
+        <v>3541</v>
+      </c>
+      <c r="C78">
+        <v>26</v>
       </c>
       <c r="D78" t="s">
-        <v>3598</v>
+        <v>2847</v>
       </c>
       <c r="F78">
         <v>1</v>
@@ -41285,22 +41462,31 @@
       <c r="G78">
         <v>1</v>
       </c>
-      <c r="I78" s="112" t="s">
-        <v>3494</v>
-      </c>
-    </row>
-    <row r="79" spans="1:16">
+      <c r="I78" s="112"/>
+      <c r="J78" s="112"/>
+      <c r="K78" s="112"/>
+      <c r="L78" s="112"/>
+      <c r="M78" s="112"/>
+      <c r="N78" s="112"/>
+      <c r="O78" s="112"/>
+      <c r="P78" s="112"/>
+      <c r="Q78">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="79" spans="1:17">
       <c r="A79" t="s">
-        <v>3608</v>
+        <v>3573</v>
       </c>
       <c r="B79" s="113" t="s">
-        <v>3580</v>
-      </c>
-      <c r="C79" t="s">
-        <v>3567</v>
+        <v>3542</v>
+      </c>
+      <c r="C79">
+        <v>26</v>
       </c>
       <c r="D79" t="s">
-        <v>2788</v>
+        <v>1231</v>
       </c>
       <c r="F79">
         <v>1</v>
@@ -41308,22 +41494,31 @@
       <c r="G79">
         <v>1</v>
       </c>
-      <c r="P79" s="112" t="s">
-        <v>3493</v>
-      </c>
-    </row>
-    <row r="80" spans="1:16">
+      <c r="I79" s="112"/>
+      <c r="J79" s="112"/>
+      <c r="K79" s="112"/>
+      <c r="L79" s="112"/>
+      <c r="M79" s="112"/>
+      <c r="N79" s="112"/>
+      <c r="O79" s="112"/>
+      <c r="P79" s="112"/>
+      <c r="Q79">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="80" spans="1:17">
       <c r="A80" t="s">
-        <v>3608</v>
+        <v>3573</v>
       </c>
       <c r="B80" s="113" t="s">
-        <v>3577</v>
-      </c>
-      <c r="C80" t="s">
-        <v>3568</v>
+        <v>3540</v>
+      </c>
+      <c r="C80">
+        <v>26</v>
       </c>
       <c r="D80" t="s">
-        <v>3599</v>
+        <v>2814</v>
       </c>
       <c r="F80">
         <v>1</v>
@@ -41331,22 +41526,31 @@
       <c r="G80">
         <v>1</v>
       </c>
-      <c r="M80" s="112" t="s">
-        <v>3495</v>
-      </c>
-    </row>
-    <row r="81" spans="1:15">
+      <c r="I80" s="112"/>
+      <c r="J80" s="112"/>
+      <c r="K80" s="112"/>
+      <c r="L80" s="112"/>
+      <c r="M80" s="112"/>
+      <c r="N80" s="112"/>
+      <c r="O80" s="112"/>
+      <c r="P80" s="112"/>
+      <c r="Q80">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="81" spans="1:17">
       <c r="A81" t="s">
-        <v>2746</v>
+        <v>3573</v>
       </c>
       <c r="B81" s="113" t="s">
-        <v>3578</v>
-      </c>
-      <c r="C81" t="s">
-        <v>3569</v>
+        <v>3544</v>
+      </c>
+      <c r="C81">
+        <v>26</v>
       </c>
       <c r="D81" t="s">
-        <v>3600</v>
+        <v>208</v>
       </c>
       <c r="F81">
         <v>1</v>
@@ -41354,37 +41558,31 @@
       <c r="G81">
         <v>1</v>
       </c>
-      <c r="I81" s="112" t="s">
-        <v>3479</v>
-      </c>
-      <c r="J81" s="112" t="s">
-        <v>3480</v>
-      </c>
-      <c r="K81" s="112" t="s">
-        <v>3481</v>
-      </c>
-      <c r="L81" s="112" t="s">
-        <v>3483</v>
-      </c>
-      <c r="N81" s="112" t="s">
-        <v>3478</v>
-      </c>
-      <c r="O81" s="112" t="s">
-        <v>3482</v>
-      </c>
-    </row>
-    <row r="82" spans="1:15">
+      <c r="I81" s="112"/>
+      <c r="J81" s="112"/>
+      <c r="K81" s="112"/>
+      <c r="L81" s="112"/>
+      <c r="M81" s="112"/>
+      <c r="N81" s="112"/>
+      <c r="O81" s="112"/>
+      <c r="P81" s="112"/>
+      <c r="Q81">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="82" spans="1:17">
       <c r="A82" t="s">
-        <v>2746</v>
+        <v>3573</v>
       </c>
       <c r="B82" s="113" t="s">
-        <v>3572</v>
-      </c>
-      <c r="C82" t="s">
-        <v>3569</v>
+        <v>3545</v>
+      </c>
+      <c r="C82">
+        <v>26</v>
       </c>
       <c r="D82" t="s">
-        <v>3601</v>
+        <v>2808</v>
       </c>
       <c r="F82">
         <v>1</v>
@@ -41396,21 +41594,27 @@
       <c r="J82" s="112"/>
       <c r="K82" s="112"/>
       <c r="L82" s="112"/>
+      <c r="M82" s="112"/>
       <c r="N82" s="112"/>
       <c r="O82" s="112"/>
-    </row>
-    <row r="83" spans="1:15">
+      <c r="P82" s="112"/>
+      <c r="Q82">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="83" spans="1:17">
       <c r="A83" t="s">
-        <v>2746</v>
+        <v>3573</v>
       </c>
       <c r="B83" s="113" t="s">
-        <v>3574</v>
-      </c>
-      <c r="C83" t="s">
-        <v>3569</v>
+        <v>3546</v>
+      </c>
+      <c r="C83">
+        <v>26</v>
       </c>
       <c r="D83" t="s">
-        <v>3602</v>
+        <v>2708</v>
       </c>
       <c r="F83">
         <v>1</v>
@@ -41422,21 +41626,27 @@
       <c r="J83" s="112"/>
       <c r="K83" s="112"/>
       <c r="L83" s="112"/>
+      <c r="M83" s="112"/>
       <c r="N83" s="112"/>
       <c r="O83" s="112"/>
-    </row>
-    <row r="84" spans="1:15">
+      <c r="P83" s="112"/>
+      <c r="Q83">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="84" spans="1:17">
       <c r="A84" t="s">
-        <v>2746</v>
+        <v>3573</v>
       </c>
       <c r="B84" s="113" t="s">
-        <v>3575</v>
-      </c>
-      <c r="C84" t="s">
-        <v>3569</v>
+        <v>3547</v>
+      </c>
+      <c r="C84">
+        <v>26</v>
       </c>
       <c r="D84" t="s">
-        <v>2822</v>
+        <v>3564</v>
       </c>
       <c r="F84">
         <v>1</v>
@@ -41448,21 +41658,27 @@
       <c r="J84" s="112"/>
       <c r="K84" s="112"/>
       <c r="L84" s="112"/>
+      <c r="M84" s="112"/>
       <c r="N84" s="112"/>
       <c r="O84" s="112"/>
-    </row>
-    <row r="85" spans="1:15">
+      <c r="P84" s="112"/>
+      <c r="Q84">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="85" spans="1:17">
       <c r="A85" t="s">
-        <v>2746</v>
+        <v>3575</v>
       </c>
       <c r="B85" s="113" t="s">
-        <v>3579</v>
-      </c>
-      <c r="C85" t="s">
-        <v>3569</v>
+        <v>3544</v>
+      </c>
+      <c r="C85">
+        <v>27</v>
       </c>
       <c r="D85" t="s">
-        <v>3603</v>
+        <v>2763</v>
       </c>
       <c r="F85">
         <v>1</v>
@@ -41474,101 +41690,341 @@
       <c r="J85" s="112"/>
       <c r="K85" s="112"/>
       <c r="L85" s="112"/>
+      <c r="M85" s="112"/>
       <c r="N85" s="112"/>
       <c r="O85" s="112"/>
-    </row>
-    <row r="86" spans="1:15">
+      <c r="P85" s="112"/>
+      <c r="Q85">
+        <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="86" spans="1:17">
       <c r="A86" t="s">
-        <v>2746</v>
+        <v>3575</v>
       </c>
       <c r="B86" s="113" t="s">
-        <v>3573</v>
-      </c>
-      <c r="C86" t="s">
-        <v>3569</v>
+        <v>3539</v>
+      </c>
+      <c r="C86">
+        <v>28</v>
       </c>
       <c r="D86" t="s">
-        <v>3604</v>
+        <v>3565</v>
       </c>
       <c r="F86">
         <v>1</v>
       </c>
       <c r="G86">
-        <v>1</v>
-      </c>
-      <c r="I86" s="112"/>
-      <c r="J86" s="112"/>
-      <c r="K86" s="112"/>
-      <c r="L86" s="112"/>
-      <c r="N86" s="112"/>
-      <c r="O86" s="112"/>
-    </row>
-    <row r="87" spans="1:15">
+        <v>2</v>
+      </c>
+      <c r="I86" s="112" t="s">
+        <v>3494</v>
+      </c>
+      <c r="Q86">
+        <f t="shared" si="1"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="87" spans="1:17">
       <c r="A87" t="s">
-        <v>3607</v>
+        <v>3575</v>
       </c>
       <c r="B87" s="113" t="s">
-        <v>3573</v>
-      </c>
-      <c r="C87" t="s">
-        <v>3570</v>
+        <v>3547</v>
+      </c>
+      <c r="C87">
+        <v>29</v>
       </c>
       <c r="D87" t="s">
-        <v>3605</v>
+        <v>2788</v>
       </c>
       <c r="F87">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G87">
-        <v>1</v>
-      </c>
-      <c r="L87" s="112" t="s">
-        <v>3503</v>
-      </c>
-    </row>
-    <row r="88" spans="1:15">
+        <v>4</v>
+      </c>
+      <c r="P87" s="112" t="s">
+        <v>3493</v>
+      </c>
+      <c r="Q87">
+        <f t="shared" si="1"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="88" spans="1:17">
       <c r="A88" t="s">
-        <v>3606</v>
+        <v>3575</v>
       </c>
       <c r="B88" s="113" t="s">
-        <v>3572</v>
-      </c>
-      <c r="C88" t="s">
-        <v>3571</v>
+        <v>3544</v>
+      </c>
+      <c r="C88">
+        <v>30</v>
       </c>
       <c r="D88" t="s">
-        <v>2793</v>
+        <v>3566</v>
       </c>
       <c r="F88">
         <v>1</v>
       </c>
       <c r="G88">
+        <v>2</v>
+      </c>
+      <c r="M88" s="112" t="s">
+        <v>3495</v>
+      </c>
+      <c r="Q88">
+        <f t="shared" si="1"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="89" spans="1:17">
+      <c r="A89" t="s">
+        <v>2746</v>
+      </c>
+      <c r="B89" s="113" t="s">
+        <v>3545</v>
+      </c>
+      <c r="C89">
+        <v>31</v>
+      </c>
+      <c r="D89" t="s">
+        <v>3567</v>
+      </c>
+      <c r="F89">
         <v>1</v>
       </c>
-      <c r="I88" s="112" t="s">
+      <c r="G89">
+        <v>1</v>
+      </c>
+      <c r="I89" s="112" t="s">
+        <v>3479</v>
+      </c>
+      <c r="J89" s="112" t="s">
+        <v>3480</v>
+      </c>
+      <c r="K89" s="112" t="s">
+        <v>3481</v>
+      </c>
+      <c r="L89" s="112" t="s">
+        <v>3483</v>
+      </c>
+      <c r="N89" s="112" t="s">
+        <v>3478</v>
+      </c>
+      <c r="O89" s="112" t="s">
+        <v>3482</v>
+      </c>
+      <c r="Q89">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="90" spans="1:17">
+      <c r="A90" t="s">
+        <v>2746</v>
+      </c>
+      <c r="B90" s="113" t="s">
+        <v>3539</v>
+      </c>
+      <c r="C90">
+        <v>31</v>
+      </c>
+      <c r="D90" t="s">
+        <v>3568</v>
+      </c>
+      <c r="F90">
+        <v>1</v>
+      </c>
+      <c r="G90">
+        <v>1</v>
+      </c>
+      <c r="I90" s="112"/>
+      <c r="J90" s="112"/>
+      <c r="K90" s="112"/>
+      <c r="L90" s="112"/>
+      <c r="N90" s="112"/>
+      <c r="O90" s="112"/>
+      <c r="Q90">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="91" spans="1:17">
+      <c r="A91" t="s">
+        <v>2746</v>
+      </c>
+      <c r="B91" s="113" t="s">
+        <v>3541</v>
+      </c>
+      <c r="C91">
+        <v>31</v>
+      </c>
+      <c r="D91" t="s">
+        <v>3569</v>
+      </c>
+      <c r="F91">
+        <v>1</v>
+      </c>
+      <c r="G91">
+        <v>1</v>
+      </c>
+      <c r="I91" s="112"/>
+      <c r="J91" s="112"/>
+      <c r="K91" s="112"/>
+      <c r="L91" s="112"/>
+      <c r="N91" s="112"/>
+      <c r="O91" s="112"/>
+      <c r="Q91">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="92" spans="1:17">
+      <c r="A92" t="s">
+        <v>2746</v>
+      </c>
+      <c r="B92" s="113" t="s">
+        <v>3542</v>
+      </c>
+      <c r="C92">
+        <v>31</v>
+      </c>
+      <c r="D92" t="s">
+        <v>2822</v>
+      </c>
+      <c r="F92">
+        <v>1</v>
+      </c>
+      <c r="G92">
+        <v>1</v>
+      </c>
+      <c r="I92" s="112"/>
+      <c r="J92" s="112"/>
+      <c r="K92" s="112"/>
+      <c r="L92" s="112"/>
+      <c r="N92" s="112"/>
+      <c r="O92" s="112"/>
+      <c r="Q92">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="93" spans="1:17">
+      <c r="A93" t="s">
+        <v>2746</v>
+      </c>
+      <c r="B93" s="113" t="s">
+        <v>3546</v>
+      </c>
+      <c r="C93">
+        <v>31</v>
+      </c>
+      <c r="D93" t="s">
+        <v>3570</v>
+      </c>
+      <c r="F93">
+        <v>1</v>
+      </c>
+      <c r="G93">
+        <v>1</v>
+      </c>
+      <c r="I93" s="112"/>
+      <c r="J93" s="112"/>
+      <c r="K93" s="112"/>
+      <c r="L93" s="112"/>
+      <c r="N93" s="112"/>
+      <c r="O93" s="112"/>
+      <c r="Q93">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="94" spans="1:17">
+      <c r="A94" t="s">
+        <v>2746</v>
+      </c>
+      <c r="B94" s="113" t="s">
+        <v>3540</v>
+      </c>
+      <c r="C94">
+        <v>31</v>
+      </c>
+      <c r="D94" t="s">
+        <v>3571</v>
+      </c>
+      <c r="F94">
+        <v>1</v>
+      </c>
+      <c r="G94">
+        <v>1</v>
+      </c>
+      <c r="I94" s="112"/>
+      <c r="J94" s="112"/>
+      <c r="K94" s="112"/>
+      <c r="L94" s="112"/>
+      <c r="N94" s="112"/>
+      <c r="O94" s="112"/>
+      <c r="Q94">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="95" spans="1:17">
+      <c r="A95" t="s">
+        <v>3574</v>
+      </c>
+      <c r="B95" s="113" t="s">
+        <v>3540</v>
+      </c>
+      <c r="C95">
+        <v>32</v>
+      </c>
+      <c r="D95" t="s">
+        <v>3572</v>
+      </c>
+      <c r="F95">
+        <v>1</v>
+      </c>
+      <c r="G95">
+        <v>1</v>
+      </c>
+      <c r="L95" s="112" t="s">
+        <v>3503</v>
+      </c>
+      <c r="Q95">
+        <f t="shared" si="1"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="96" spans="1:17">
+      <c r="A96" t="s">
+        <v>3573</v>
+      </c>
+      <c r="B96" s="113" t="s">
+        <v>3539</v>
+      </c>
+      <c r="C96">
+        <v>33</v>
+      </c>
+      <c r="D96" t="s">
+        <v>2793</v>
+      </c>
+      <c r="F96">
+        <v>1</v>
+      </c>
+      <c r="G96">
+        <v>1</v>
+      </c>
+      <c r="I96" s="112" t="s">
         <v>3504</v>
       </c>
-    </row>
-    <row r="89" spans="1:15">
-      <c r="I89" s="112"/>
-    </row>
-    <row r="90" spans="1:15">
-      <c r="I90" s="112"/>
-    </row>
-    <row r="91" spans="1:15">
-      <c r="I91" s="112"/>
-    </row>
-    <row r="92" spans="1:15">
-      <c r="I92" s="112"/>
-    </row>
-    <row r="93" spans="1:15">
-      <c r="I93" s="112"/>
-    </row>
-    <row r="94" spans="1:15">
-      <c r="I94" s="112"/>
-    </row>
-    <row r="96" spans="1:15">
-      <c r="I96" s="112"/>
+      <c r="Q96">
+        <f t="shared" si="1"/>
+        <v>32</v>
+      </c>
     </row>
     <row r="97" spans="9:9">
       <c r="I97" s="112"/>
@@ -41578,6 +42034,27 @@
     </row>
     <row r="99" spans="9:9">
       <c r="I99" s="112"/>
+    </row>
+    <row r="100" spans="9:9">
+      <c r="I100" s="112"/>
+    </row>
+    <row r="101" spans="9:9">
+      <c r="I101" s="112"/>
+    </row>
+    <row r="102" spans="9:9">
+      <c r="I102" s="112"/>
+    </row>
+    <row r="104" spans="9:9">
+      <c r="I104" s="112"/>
+    </row>
+    <row r="105" spans="9:9">
+      <c r="I105" s="112"/>
+    </row>
+    <row r="106" spans="9:9">
+      <c r="I106" s="112"/>
+    </row>
+    <row r="107" spans="9:9">
+      <c r="I107" s="112"/>
     </row>
   </sheetData>
   <phoneticPr fontId="35" type="noConversion"/>

</xml_diff>